<commit_message>
Isolate scraped email transactions from canonical Excel data
Adds a source ('excel'/'email') and promoted column to transactions,
with a migration that backfills existing rows by raw_email_uid prefix.
match.py, export.py, and dashboard's real metrics now only consider
source='excel' rows, so newly scraped emails are captured for review
but never automatically merged into matching/export/dashboard totals
until explicitly promoted (no promotion mechanism yet, by design).

Adds review_pending.py to list unpromoted scraped transactions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N140"/>
+  <dimension ref="A1:N139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -546,66 +546,74 @@
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
-          <t>GRiZ - Free Shows for the People</t>
+          <t>Levity</t>
         </is>
       </c>
       <c r="C2" s="8" t="n">
-        <v>46292</v>
+        <v>45981</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46283</v>
+        <v>45960</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>JUNKYARD — Denver, CO</t>
-        </is>
-      </c>
-      <c r="G2" s="9" t="n"/>
+          <t>Boulder Theater</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
       <c r="I2" s="9" t="n">
-        <v>0</v>
+        <v>30</v>
+      </c>
+      <c r="J2" s="8" t="n">
+        <v>45980</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
         <is>
-          <t>Levity</t>
+          <t>Its Murph</t>
         </is>
       </c>
       <c r="C3" s="8" t="n">
-        <v>45981</v>
+        <v>46116</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>45960</v>
+        <v>45939</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Boulder Theater</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>30</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I3" s="9" t="n">
-        <v>30</v>
+        <v>296.7</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>45980</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Its Murph</t>
+          <t>Cloonee</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
-        <v>46116</v>
+        <v>46151</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>45939</v>
+        <v>45973</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -613,86 +621,86 @@
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>98.90000000000001</v>
+        <v>75.84941176470589</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>296.7</v>
+        <v>1289.44</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>46242</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cloonee</t>
+          <t>Max Styler</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>46151</v>
+        <v>46067</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>45973</v>
+        <v>45980</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Lula Club, Madrid</t>
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>75.84941176470589</v>
+        <v>19.562</v>
       </c>
       <c r="H5" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="I5" s="9" t="n">
-        <v>1289.44</v>
+        <v>97.81</v>
       </c>
       <c r="J5" s="8" t="n">
-        <v>46186</v>
+        <v>46066</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>Max Styler</t>
+          <t>Josh Johnson Fri 7</t>
         </is>
       </c>
       <c r="C6" s="8" t="n">
-        <v>46067</v>
+        <v>46108</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>45980</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Lula Club, Madrid</t>
+          <t>Houston Improv 7 PM</t>
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>19.562</v>
+        <v>50</v>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I6" s="9" t="n">
-        <v>97.81</v>
+        <v>550</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>46066</v>
+        <v>46103</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
         <is>
-          <t>Josh Johnson Fri 7</t>
+          <t>Josh Johnson Sat 7</t>
         </is>
       </c>
       <c r="C7" s="8" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>45980</v>
@@ -706,53 +714,53 @@
         <v>50</v>
       </c>
       <c r="H7" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="I7" s="9" t="n">
-        <v>550</v>
+        <v>250</v>
       </c>
       <c r="J7" s="8" t="n">
-        <v>46103</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
         <is>
-          <t>Josh Johnson Sat 7</t>
+          <t>Josh Johnson Fri 9</t>
         </is>
       </c>
       <c r="C8" s="8" t="n">
-        <v>46109</v>
+        <v>46108</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>45980</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Houston Improv 7 PM</t>
+          <t>Houston Improv 9:30PM</t>
         </is>
       </c>
       <c r="G8" s="9" t="n">
         <v>50</v>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="I8" s="9" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>46098</v>
+        <v>46054</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>Josh Johnson Fri 9</t>
+          <t>Josh Johnson Sat 9</t>
         </is>
       </c>
       <c r="C9" s="8" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>45980</v>
@@ -766,383 +774,383 @@
         <v>50</v>
       </c>
       <c r="H9" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="I9" s="9" t="n">
-        <v>700</v>
+        <v>150</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>46054</v>
+        <v>46001</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>Josh Johnson Sat 9</t>
+          <t>Whethan</t>
         </is>
       </c>
       <c r="C10" s="8" t="n">
-        <v>46109</v>
+        <v>46074</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>45980</v>
+        <v>45981</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Houston Improv 9:30PM</t>
+          <t>Webster Hall, NY 11:30</t>
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>50</v>
+        <v>34.57</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10" s="9" t="n">
-        <v>150</v>
+        <v>138.28</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>46001</v>
+        <v>46075</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>Whethan</t>
+          <t>Teletech</t>
         </is>
       </c>
       <c r="C11" s="8" t="n">
-        <v>46074</v>
+        <v>46060</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>45981</v>
+        <v>45993</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Webster Hall, NY 11:30</t>
+          <t>Brooklyn Storehouse</t>
         </is>
       </c>
       <c r="G11" s="9" t="n">
-        <v>34.57</v>
+        <v>54.8</v>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>138.28</v>
+        <v>328.8</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>46075</v>
+        <v>46055</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>Teletech</t>
+          <t>John Summit</t>
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>46060</v>
+        <v>46102</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>45993</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Brooklyn Storehouse</t>
+          <t>Vail</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>54.8</v>
+        <v>231.92</v>
       </c>
       <c r="H12" t="n">
         <v>6</v>
       </c>
       <c r="I12" s="9" t="n">
-        <v>328.8</v>
+        <v>1391.52</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>46055</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>John Summit</t>
+          <t>Kettama Boston</t>
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>46102</v>
+        <v>46094</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>45993</v>
+        <v>45995</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Vail</t>
+          <t>Royale</t>
         </is>
       </c>
       <c r="G13" s="9" t="n">
-        <v>231.92</v>
+        <v>35.54</v>
       </c>
       <c r="H13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I13" s="9" t="n">
-        <v>1391.52</v>
+        <v>35.54</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>46098</v>
+        <v>46051</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>Kettama Boston</t>
+          <t>Kettama Austin</t>
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>46094</v>
+        <v>46137</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>45995</v>
+        <v>45996</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Royale</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G14" s="9" t="n">
-        <v>35.54</v>
+        <v>38.27</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I14" s="9" t="n">
-        <v>35.54</v>
+        <v>191.35</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>46051</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kettama Austin</t>
+          <t>Iliza Shlesinger</t>
         </is>
       </c>
       <c r="C15" s="8" t="n">
-        <v>46137</v>
+        <v>46066</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>45996</v>
+        <v>46016</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t xml:space="preserve">Brea Improv </t>
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>38.27</v>
+        <v>49.21833333333333</v>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I15" s="9" t="n">
-        <v>191.35</v>
+        <v>590.62</v>
       </c>
       <c r="J15" s="8" t="n">
-        <v>46153</v>
+        <v>46061</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>Iliza Shlesinger</t>
+          <t>Mardi Gras</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>46066</v>
+        <v>46065</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>46016</v>
+        <v>46029</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brea Improv </t>
+          <t>Boot Block Party</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>49.21833333333333</v>
+        <v>33.28</v>
       </c>
       <c r="H16" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I16" s="9" t="n">
-        <v>590.62</v>
+        <v>199.68</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>46061</v>
+        <v>46065</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mardi Gras</t>
+          <t>Max Styler SF</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>46065</v>
+        <v>46137</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>46029</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Boot Block Party</t>
+          <t>Regency Ballroom</t>
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>33.28</v>
+        <v>39.44</v>
       </c>
       <c r="H17" t="n">
         <v>6</v>
       </c>
       <c r="I17" s="9" t="n">
-        <v>199.68</v>
+        <v>236.64</v>
       </c>
       <c r="J17" s="8" t="n">
-        <v>46065</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>Max Styler SF</t>
+          <t>Zeds Dead Thurs</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>46137</v>
+        <v>46205</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>46029</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Regency Ballroom</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G18" s="9" t="n">
-        <v>39.44</v>
+        <v>115.95</v>
       </c>
       <c r="H18" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I18" s="9" t="n">
-        <v>236.64</v>
+        <v>347.85</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>46153</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>Zeds Dead Thurs</t>
+          <t>Diplo &amp; Sonny Fodera</t>
         </is>
       </c>
       <c r="C19" s="8" t="n">
-        <v>46205</v>
+        <v>46059</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>46029</v>
+        <v>46031</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>888 Garage</t>
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>115.95</v>
+        <v>92.7</v>
       </c>
       <c r="H19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I19" s="9" t="n">
-        <v>347.85</v>
+        <v>185.4</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>46242</v>
+        <v>46059</v>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>Diplo &amp; Sonny Fodera</t>
+          <t>Riordan</t>
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>46059</v>
+        <v>46068</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>46031</v>
+        <v>46036</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>888 Garage</t>
+          <t>Headquarters Beercade</t>
         </is>
       </c>
       <c r="G20" s="9" t="n">
-        <v>92.7</v>
+        <v>24.25</v>
       </c>
       <c r="H20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I20" s="9" t="n">
-        <v>185.4</v>
+        <v>97</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>46059</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>Riordan</t>
+          <t>Subtronics Thurs</t>
         </is>
       </c>
       <c r="C21" s="8" t="n">
-        <v>46068</v>
+        <v>46135</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>46036</v>
+        <v>46037</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Headquarters Beercade</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G21" s="9" t="n">
-        <v>24.25</v>
+        <v>97.13500000000001</v>
       </c>
       <c r="H21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I21" s="9" t="n">
-        <v>97</v>
+        <v>485.675</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>46068</v>
+        <v>46135</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>Subtronics Thurs</t>
+          <t>Subtronics Fri</t>
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>46037</v>
@@ -1153,146 +1161,146 @@
         </is>
       </c>
       <c r="G22" s="9" t="n">
-        <v>97.13500000000001</v>
+        <v>80.94583333333334</v>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I22" s="9" t="n">
         <v>485.675</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>46135</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>Subtronics Fri</t>
+          <t>Illenium</t>
         </is>
       </c>
       <c r="C23" s="8" t="n">
-        <v>46136</v>
+        <v>46058</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>46037</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Pier 80 Warehouse</t>
         </is>
       </c>
       <c r="G23" s="9" t="n">
-        <v>80.94583333333334</v>
+        <v>110.62</v>
       </c>
       <c r="H23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I23" s="9" t="n">
-        <v>485.675</v>
+        <v>221.24</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>46242</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>Illenium</t>
+          <t>Diceys</t>
         </is>
       </c>
       <c r="C24" s="8" t="n">
-        <v>46058</v>
+        <v>46095</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46037</v>
+        <v>46038</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Pier 80 Warehouse</t>
+          <t>Diceys Dublin</t>
         </is>
       </c>
       <c r="G24" s="9" t="n">
-        <v>110.62</v>
+        <v>63.452</v>
       </c>
       <c r="H24" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="I24" s="9" t="n">
-        <v>221.24</v>
+        <v>634.52</v>
       </c>
       <c r="J24" s="8" t="n">
-        <v>46052</v>
+        <v>46083</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>Diceys</t>
+          <t>Odd Mob</t>
         </is>
       </c>
       <c r="C25" s="8" t="n">
-        <v>46095</v>
+        <v>46093</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>46038</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Diceys Dublin</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G25" s="9" t="n">
-        <v>63.452</v>
+        <v>50.72</v>
       </c>
       <c r="H25" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>634.52</v>
+        <v>304.32</v>
       </c>
       <c r="J25" s="8" t="n">
-        <v>46083</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>Odd Mob</t>
+          <t>Blondish</t>
         </is>
       </c>
       <c r="C26" s="8" t="n">
-        <v>46093</v>
+        <v>46073</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>46038</v>
+        <v>46043</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Belly Up Aspen</t>
         </is>
       </c>
       <c r="G26" s="9" t="n">
-        <v>50.72</v>
+        <v>168</v>
       </c>
       <c r="H26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I26" s="9" t="n">
-        <v>304.32</v>
+        <v>168</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>46093</v>
+        <v>46075</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
         <is>
-          <t>Blondish</t>
+          <t>Mau P</t>
         </is>
       </c>
       <c r="C27" s="8" t="n">
-        <v>46073</v>
+        <v>46074</v>
       </c>
       <c r="D27" s="8" t="n">
         <v>46043</v>
@@ -1303,13 +1311,13 @@
         </is>
       </c>
       <c r="G27" s="9" t="n">
-        <v>168</v>
+        <v>222</v>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27" s="9" t="n">
-        <v>168</v>
+        <v>444</v>
       </c>
       <c r="J27" s="8" t="n">
         <v>46075</v>
@@ -1318,58 +1326,58 @@
     <row r="28">
       <c r="B28" t="inlineStr">
         <is>
-          <t>Mau P</t>
+          <t>Hi Ibiza</t>
         </is>
       </c>
       <c r="C28" s="8" t="n">
-        <v>46074</v>
+        <v>46137</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>46043</v>
+        <v>46049</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Belly Up Aspen</t>
+          <t>Hi Ibiza</t>
         </is>
       </c>
       <c r="G28" s="9" t="n">
-        <v>222</v>
+        <v>73.33333333333333</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28" s="9" t="n">
-        <v>444</v>
+        <v>220</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>46075</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>Hi Ibiza</t>
+          <t>Alesso CO</t>
         </is>
       </c>
       <c r="C29" s="8" t="n">
         <v>46137</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>46049</v>
+        <v>46056</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Hi Ibiza</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G29" s="9" t="n">
-        <v>73.33333333333333</v>
+        <v>79.7</v>
       </c>
       <c r="H29" t="n">
         <v>3</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>220</v>
+        <v>239.1</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>46153</v>
@@ -1378,178 +1386,178 @@
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>Alesso CO</t>
+          <t>Chris Lorenzo DEN</t>
         </is>
       </c>
       <c r="C30" s="8" t="n">
-        <v>46137</v>
+        <v>46060</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>46056</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G30" s="9" t="n">
-        <v>79.7</v>
+        <v>54.63</v>
       </c>
       <c r="H30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>239.1</v>
+        <v>218.52</v>
       </c>
       <c r="J30" s="8" t="n">
-        <v>46153</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chris Lorenzo DEN</t>
+          <t>Discolines Boulder</t>
         </is>
       </c>
       <c r="C31" s="8" t="n">
-        <v>46060</v>
+        <v>46130</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Ferrand Field</t>
         </is>
       </c>
       <c r="G31" s="9" t="n">
-        <v>54.63</v>
+        <v>99</v>
       </c>
       <c r="H31" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I31" s="9" t="n">
-        <v>218.52</v>
+        <v>1188</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>46060</v>
+        <v>46130</v>
       </c>
     </row>
     <row r="32">
       <c r="B32" t="inlineStr">
         <is>
-          <t>Discolines Boulder</t>
+          <t>Its Murph UT</t>
         </is>
       </c>
       <c r="C32" s="8" t="n">
-        <v>46130</v>
+        <v>46151</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Ferrand Field</t>
+          <t>BoxPac</t>
         </is>
       </c>
       <c r="G32" s="9" t="n">
-        <v>99</v>
+        <v>55.505</v>
       </c>
       <c r="H32" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I32" s="9" t="n">
-        <v>1188</v>
+        <v>222.02</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>46130</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
         <is>
-          <t>Its Murph UT</t>
+          <t>Yukimatsu DEN</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>46151</v>
+        <v>46115</v>
       </c>
       <c r="D33" s="8" t="n">
         <v>46058</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>BoxPac</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G33" s="9" t="n">
-        <v>55.505</v>
+        <v>38.38</v>
       </c>
       <c r="H33" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I33" s="9" t="n">
-        <v>222.02</v>
+        <v>38.38</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>46153</v>
+        <v>46117</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yukimatsu DEN</t>
+          <t>Factory Town MMW 3/29</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>46115</v>
+        <v>46110</v>
       </c>
       <c r="D34" s="8" t="n">
         <v>46058</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Factory Town</t>
         </is>
       </c>
       <c r="G34" s="9" t="n">
-        <v>38.38</v>
+        <v>75</v>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I34" s="9" t="n">
-        <v>38.38</v>
+        <v>375</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>46117</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>Factory Town MMW 3/29</t>
+          <t>Solid Grooves GA Before 1AM</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>46110</v>
+        <v>46108</v>
       </c>
       <c r="D35" s="8" t="n">
         <v>46058</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Factory Town</t>
+          <t>Space</t>
         </is>
       </c>
       <c r="G35" s="9" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I35" s="9" t="n">
-        <v>375</v>
+        <v>200</v>
       </c>
       <c r="J35" s="8" t="n">
         <v>46110</v>
@@ -1558,41 +1566,41 @@
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>Solid Grooves GA Before 1AM</t>
+          <t>Factory Town MMW 3/28</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>46058</v>
+        <v>45694</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Space</t>
+          <t>Factory Town</t>
         </is>
       </c>
       <c r="G36" s="9" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H36" t="n">
         <v>2</v>
       </c>
       <c r="I36" s="9" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="J36" s="8" t="n">
-        <v>46110</v>
+        <v>46108</v>
       </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
         <is>
-          <t>Factory Town MMW 3/28</t>
+          <t>Factory Town MMW 3/27</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>46109</v>
+        <v>46108</v>
       </c>
       <c r="D37" s="8" t="n">
         <v>45694</v>
@@ -1603,56 +1611,56 @@
         </is>
       </c>
       <c r="G37" s="9" t="n">
-        <v>75</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H37" t="n">
         <v>2</v>
       </c>
       <c r="I37" s="9" t="n">
-        <v>150</v>
+        <v>159.98</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>46108</v>
+        <v>46103</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>Factory Town MMW 3/27</t>
+          <t>Rufus Jun 5</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>46108</v>
+        <v>46178</v>
       </c>
       <c r="D38" s="8" t="n">
-        <v>45694</v>
+        <v>46063</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Factory Town</t>
+          <t>The Gorge</t>
         </is>
       </c>
       <c r="G38" s="9" t="n">
-        <v>79.98999999999999</v>
+        <v>253.48</v>
       </c>
       <c r="H38" t="n">
         <v>2</v>
       </c>
       <c r="I38" s="9" t="n">
-        <v>159.98</v>
+        <v>506.96</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>46103</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rufus Jun 5</t>
+          <t>Rufus Jun 6</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>46178</v>
+        <v>46179</v>
       </c>
       <c r="D39" s="8" t="n">
         <v>46063</v>
@@ -1666,10 +1674,10 @@
         <v>253.48</v>
       </c>
       <c r="H39" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39" s="9" t="n">
-        <v>506.96</v>
+        <v>1013.92</v>
       </c>
       <c r="J39" s="8" t="n">
         <v>46186</v>
@@ -1678,11 +1686,11 @@
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rufus Jun 6</t>
+          <t>Rufus 2 day</t>
         </is>
       </c>
       <c r="C40" s="8" t="n">
-        <v>46179</v>
+        <v>46178</v>
       </c>
       <c r="D40" s="8" t="n">
         <v>46063</v>
@@ -1693,103 +1701,103 @@
         </is>
       </c>
       <c r="G40" s="9" t="n">
-        <v>253.48</v>
+        <v>138.98</v>
       </c>
       <c r="H40" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40" s="9" t="n">
-        <v>1013.92</v>
+        <v>277.96</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>46186</v>
+        <v>46063</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rufus 2 day</t>
+          <t>Breakaway Atlanta Stands 26</t>
         </is>
       </c>
       <c r="C41" s="8" t="n">
-        <v>46178</v>
+        <v>46157</v>
       </c>
       <c r="D41" s="8" t="n">
-        <v>46063</v>
+        <v>46066</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>The Gorge</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="G41" s="9" t="n">
-        <v>138.98</v>
+        <v>127.3</v>
       </c>
       <c r="H41" t="n">
         <v>2</v>
       </c>
       <c r="I41" s="9" t="n">
-        <v>277.96</v>
+        <v>254.6</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>46063</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="inlineStr">
         <is>
-          <t>Breakaway Atlanta Stands 26</t>
+          <t>Josh Baker CO</t>
         </is>
       </c>
       <c r="C42" s="8" t="n">
-        <v>46157</v>
+        <v>46116</v>
       </c>
       <c r="D42" s="8" t="n">
         <v>46066</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>The Arch</t>
         </is>
       </c>
       <c r="G42" s="9" t="n">
-        <v>127.3</v>
+        <v>47.38</v>
       </c>
       <c r="H42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I42" s="9" t="n">
-        <v>254.6</v>
+        <v>47.38</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>46186</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>Josh Baker CO</t>
+          <t>Bullet Tooth</t>
         </is>
       </c>
       <c r="C43" s="8" t="n">
-        <v>46116</v>
+        <v>46100</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>46066</v>
+        <v>46067</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>The Arch</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G43" s="9" t="n">
-        <v>47.38</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="I43" s="9" t="n">
-        <v>47.38</v>
+        <v>0</v>
       </c>
       <c r="J43" s="8" t="n">
         <v>46242</v>
@@ -1798,127 +1806,124 @@
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bullet Tooth</t>
+          <t>Black book Records MMW</t>
         </is>
       </c>
       <c r="C44" s="8" t="n">
-        <v>46100</v>
+        <v>46108</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>46067</v>
+        <v>46070</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Toe Jam Backlot</t>
         </is>
       </c>
       <c r="G44" s="9" t="n">
-        <v>0</v>
+        <v>76.04000000000001</v>
       </c>
       <c r="H44" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I44" s="9" t="n">
-        <v>0</v>
+        <v>456.24</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>46242</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
         <is>
-          <t>Black book Records MMW</t>
+          <t>Kettama Detroit</t>
         </is>
       </c>
       <c r="C45" s="8" t="n">
-        <v>46108</v>
+        <v>46100</v>
       </c>
       <c r="D45" s="8" t="n">
         <v>46070</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Toe Jam Backlot</t>
+          <t>Expo Hall at Russell Industrial Center</t>
         </is>
       </c>
       <c r="G45" s="9" t="n">
-        <v>76.04000000000001</v>
+        <v>56</v>
       </c>
       <c r="H45" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="I45" s="9" t="n">
-        <v>456.24</v>
+        <v>1344</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>46110</v>
+        <v>46103</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>Kettama Detroit</t>
+          <t>Sammy Virji Austin</t>
         </is>
       </c>
       <c r="C46" s="8" t="n">
-        <v>46100</v>
+        <v>46151</v>
       </c>
       <c r="D46" s="8" t="n">
         <v>46070</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Expo Hall at Russell Industrial Center</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G46" s="9" t="n">
-        <v>56</v>
+        <v>94.29000000000001</v>
       </c>
       <c r="H46" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="I46" s="9" t="n">
-        <v>1344</v>
+        <v>565.74</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>46103</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sammy Virji Austin</t>
+          <t>Sammy Virji CO Center</t>
         </is>
       </c>
       <c r="C47" s="8" t="n">
-        <v>46151</v>
+        <v>46311</v>
       </c>
       <c r="D47" s="8" t="n">
         <v>46070</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G47" s="9" t="n">
-        <v>94.29000000000001</v>
+        <v>158.2</v>
       </c>
       <c r="H47" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I47" s="9" t="n">
-        <v>565.74</v>
-      </c>
-      <c r="J47" s="8" t="n">
-        <v>46153</v>
+        <v>632.8</v>
       </c>
     </row>
     <row r="48">
       <c r="B48" t="inlineStr">
         <is>
-          <t>Sammy Virji CO Center</t>
+          <t>Sammy Virji CO</t>
         </is>
       </c>
       <c r="C48" s="8" t="n">
@@ -1933,140 +1938,143 @@
         </is>
       </c>
       <c r="G48" s="9" t="n">
-        <v>158.2</v>
+        <v>90.5</v>
       </c>
       <c r="H48" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="I48" s="9" t="n">
-        <v>632.8</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>Sammy Virji CO</t>
+          <t>Obskur Sound</t>
         </is>
       </c>
       <c r="C49" s="8" t="n">
-        <v>46311</v>
+        <v>46101</v>
       </c>
       <c r="D49" s="8" t="n">
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="G49" s="9" t="n">
-        <v>90.5</v>
+        <v>33.99</v>
       </c>
       <c r="H49" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="I49" s="9" t="n">
-        <v>1086</v>
+        <v>203.94</v>
+      </c>
+      <c r="J49" s="8" t="n">
+        <v>46103</v>
       </c>
     </row>
     <row r="50">
       <c r="B50" t="inlineStr">
         <is>
-          <t>Obskur Sound</t>
+          <t>Louis the Child</t>
         </is>
       </c>
       <c r="C50" s="8" t="n">
-        <v>46101</v>
+        <v>46088</v>
       </c>
       <c r="D50" s="8" t="n">
-        <v>46072</v>
+        <v>46077</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Belly Up Aspen</t>
         </is>
       </c>
       <c r="G50" s="9" t="n">
-        <v>33.99</v>
+        <v>120.52</v>
       </c>
       <c r="H50" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I50" s="9" t="n">
-        <v>203.94</v>
+        <v>361.56</v>
       </c>
       <c r="J50" s="8" t="n">
-        <v>46103</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="51">
       <c r="B51" t="inlineStr">
         <is>
-          <t>Louis the Child</t>
+          <t>Rufus Du Sol Boulder Field</t>
         </is>
       </c>
       <c r="C51" s="8" t="n">
-        <v>46088</v>
+        <v>46256</v>
       </c>
       <c r="D51" s="8" t="n">
         <v>46077</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Belly Up Aspen</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="G51" s="9" t="n">
-        <v>120.52</v>
+        <v>208.125</v>
       </c>
       <c r="H51" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="I51" s="9" t="n">
-        <v>361.56</v>
+        <v>3330</v>
       </c>
       <c r="J51" s="8" t="n">
-        <v>46242</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Field</t>
+          <t>Rufus Du Sol NY Sec 115</t>
         </is>
       </c>
       <c r="C52" s="8" t="n">
-        <v>46256</v>
+        <v>46200</v>
       </c>
       <c r="D52" s="8" t="n">
         <v>46077</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>MSG</t>
         </is>
       </c>
       <c r="G52" s="9" t="n">
-        <v>208.125</v>
+        <v>284.5</v>
       </c>
       <c r="H52" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="I52" s="9" t="n">
-        <v>3330</v>
+        <v>569</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>46258</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>Rufus Du Sol NY Sec 115</t>
+          <t>Rufus Du Sol NY GA</t>
         </is>
       </c>
       <c r="C53" s="8" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="D53" s="8" t="n">
         <v>46077</v>
@@ -2077,13 +2085,13 @@
         </is>
       </c>
       <c r="G53" s="9" t="n">
-        <v>284.5</v>
+        <v>336.8</v>
       </c>
       <c r="H53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I53" s="9" t="n">
-        <v>569</v>
+        <v>336.8</v>
       </c>
       <c r="J53" s="8" t="n">
         <v>46209</v>
@@ -2092,148 +2100,148 @@
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>Rufus Du Sol NY GA</t>
+          <t>Rufus du sol Boulder Pit</t>
         </is>
       </c>
       <c r="C54" s="8" t="n">
-        <v>46201</v>
+        <v>46256</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>46077</v>
+        <v>46078</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>MSG</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="G54" s="9" t="n">
-        <v>336.8</v>
+        <v>232.8636363636364</v>
       </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I54" s="9" t="n">
-        <v>336.8</v>
+        <v>2561.5</v>
       </c>
       <c r="J54" s="8" t="n">
-        <v>46209</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>Rufus du sol Boulder Pit</t>
+          <t>Max Styler CO</t>
         </is>
       </c>
       <c r="C55" s="8" t="n">
-        <v>46256</v>
+        <v>46095</v>
       </c>
       <c r="D55" s="8" t="n">
-        <v>46078</v>
+        <v>46083</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G55" s="9" t="n">
-        <v>232.8636363636364</v>
+        <v>49.98999999999999</v>
       </c>
       <c r="H55" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="I55" s="9" t="n">
-        <v>2561.5</v>
+        <v>899.8199999999999</v>
       </c>
       <c r="J55" s="8" t="n">
-        <v>46258</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>Max Styler CO</t>
+          <t>Up in the Sky 2 day GA</t>
         </is>
       </c>
       <c r="C56" s="8" t="n">
-        <v>46095</v>
+        <v>46241</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Buttermilk</t>
         </is>
       </c>
       <c r="G56" s="9" t="n">
-        <v>49.98999999999999</v>
+        <v>378.62</v>
       </c>
       <c r="H56" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I56" s="9" t="n">
-        <v>899.8199999999999</v>
+        <v>757.24</v>
       </c>
       <c r="J56" s="8" t="n">
-        <v>46098</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
         <is>
-          <t>Up in the Sky 2 day GA</t>
+          <t>Disclosure Miami GA Any</t>
         </is>
       </c>
       <c r="C57" s="8" t="n">
-        <v>46241</v>
+        <v>46145</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>46085</v>
+        <v>46086</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Buttermilk</t>
+          <t>Space</t>
         </is>
       </c>
       <c r="G57" s="9" t="n">
-        <v>378.62</v>
+        <v>100</v>
       </c>
       <c r="H57" t="n">
         <v>2</v>
       </c>
       <c r="I57" s="9" t="n">
-        <v>757.24</v>
+        <v>200</v>
       </c>
       <c r="J57" s="8" t="n">
-        <v>46239</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
-          <t>Disclosure Miami GA Any</t>
+          <t>Disclosure Chicago</t>
         </is>
       </c>
       <c r="C58" s="8" t="n">
-        <v>46145</v>
+        <v>46150</v>
       </c>
       <c r="D58" s="8" t="n">
         <v>46086</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Space</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="G58" s="9" t="n">
-        <v>100</v>
+        <v>74.57000000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I58" s="9" t="n">
-        <v>200</v>
+        <v>223.71</v>
       </c>
       <c r="J58" s="8" t="n">
         <v>46153</v>
@@ -2242,88 +2250,88 @@
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>Disclosure Chicago</t>
+          <t>Josh Baker Austin</t>
         </is>
       </c>
       <c r="C59" s="8" t="n">
-        <v>46150</v>
+        <v>46199</v>
       </c>
       <c r="D59" s="8" t="n">
         <v>46086</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G59" s="9" t="n">
-        <v>74.57000000000001</v>
+        <v>36.77</v>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I59" s="9" t="n">
-        <v>223.71</v>
+        <v>220.62</v>
       </c>
       <c r="J59" s="8" t="n">
-        <v>46153</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
         <is>
-          <t>Josh Baker Austin</t>
+          <t>Silva Bumpa Nashville</t>
         </is>
       </c>
       <c r="C60" s="8" t="n">
-        <v>46199</v>
+        <v>46101</v>
       </c>
       <c r="D60" s="8" t="n">
-        <v>46086</v>
+        <v>46090</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Night We Met</t>
         </is>
       </c>
       <c r="G60" s="9" t="n">
-        <v>36.77</v>
+        <v>24.7</v>
       </c>
       <c r="H60" t="n">
         <v>6</v>
       </c>
       <c r="I60" s="9" t="n">
-        <v>220.62</v>
+        <v>148.2</v>
       </c>
       <c r="J60" s="8" t="n">
-        <v>46186</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>Silva Bumpa Nashville</t>
+          <t>Kanye Sofi</t>
         </is>
       </c>
       <c r="C61" s="8" t="n">
-        <v>46101</v>
+        <v>46115</v>
       </c>
       <c r="D61" s="8" t="n">
-        <v>46090</v>
+        <v>46091</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Night We Met</t>
+          <t>Sofi</t>
         </is>
       </c>
       <c r="G61" s="9" t="n">
-        <v>24.7</v>
+        <v>412</v>
       </c>
       <c r="H61" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I61" s="9" t="n">
-        <v>148.2</v>
+        <v>2884</v>
       </c>
       <c r="J61" s="8" t="n">
         <v>46242</v>
@@ -2332,125 +2340,125 @@
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>Kanye Sofi</t>
+          <t>Keinemusik</t>
         </is>
       </c>
       <c r="C62" s="8" t="n">
-        <v>46115</v>
+        <v>46149</v>
       </c>
       <c r="D62" s="8" t="n">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Sofi</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G62" s="9" t="n">
-        <v>412</v>
+        <v>102.48</v>
       </c>
       <c r="H62" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I62" s="9" t="n">
-        <v>2884</v>
+        <v>204.96</v>
       </c>
       <c r="J62" s="8" t="n">
-        <v>46242</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>Keinemusik</t>
+          <t>Levity RR</t>
         </is>
       </c>
       <c r="C63" s="8" t="n">
-        <v>46149</v>
+        <v>46297</v>
       </c>
       <c r="D63" s="8" t="n">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G63" s="9" t="n">
-        <v>102.48</v>
+        <v>92.3</v>
       </c>
       <c r="H63" t="n">
         <v>2</v>
       </c>
       <c r="I63" s="9" t="n">
-        <v>204.96</v>
-      </c>
-      <c r="J63" s="8" t="n">
-        <v>46153</v>
+        <v>184.6</v>
       </c>
     </row>
     <row r="64">
       <c r="B64" t="inlineStr">
         <is>
-          <t>Levity RR</t>
+          <t>Breakaway Utah 2026</t>
         </is>
       </c>
       <c r="C64" s="8" t="n">
         <v>46297</v>
       </c>
       <c r="D64" s="8" t="n">
-        <v>46093</v>
+        <v>46105</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Utah</t>
         </is>
       </c>
       <c r="G64" s="9" t="n">
-        <v>92.3</v>
+        <v>149</v>
       </c>
       <c r="H64" t="n">
         <v>2</v>
       </c>
       <c r="I64" s="9" t="n">
-        <v>184.6</v>
+        <v>298</v>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t>Breakaway Utah 2026</t>
+          <t>Obskur NYC</t>
         </is>
       </c>
       <c r="C65" s="8" t="n">
-        <v>46297</v>
+        <v>46221</v>
       </c>
       <c r="D65" s="8" t="n">
-        <v>46105</v>
+        <v>46107</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Sunset Park Rooftop</t>
         </is>
       </c>
       <c r="G65" s="9" t="n">
-        <v>149</v>
+        <v>54.8</v>
       </c>
       <c r="H65" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I65" s="9" t="n">
-        <v>298</v>
+        <v>164.4</v>
+      </c>
+      <c r="J65" s="8" t="n">
+        <v>46226</v>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t>Obskur NYC</t>
+          <t>Beltran NYC</t>
         </is>
       </c>
       <c r="C66" s="8" t="n">
-        <v>46221</v>
+        <v>46194</v>
       </c>
       <c r="D66" s="8" t="n">
         <v>46107</v>
@@ -2461,223 +2469,223 @@
         </is>
       </c>
       <c r="G66" s="9" t="n">
-        <v>54.8</v>
+        <v>66.75</v>
       </c>
       <c r="H66" t="n">
         <v>3</v>
       </c>
       <c r="I66" s="9" t="n">
-        <v>164.4</v>
+        <v>200.25</v>
       </c>
       <c r="J66" s="8" t="n">
-        <v>46226</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t>Beltran NYC</t>
+          <t>Kettama Nashville</t>
         </is>
       </c>
       <c r="C67" s="8" t="n">
-        <v>46194</v>
+        <v>46234</v>
       </c>
       <c r="D67" s="8" t="n">
-        <v>46107</v>
+        <v>46114</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Sunset Park Rooftop</t>
+          <t>The Pinnacle</t>
         </is>
       </c>
       <c r="G67" s="9" t="n">
-        <v>66.75</v>
+        <v>45.36</v>
       </c>
       <c r="H67" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="I67" s="9" t="n">
-        <v>200.25</v>
+        <v>816.48</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>46192</v>
+        <v>46216</v>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>Kettama Nashville</t>
+          <t>Its Murph July 4</t>
         </is>
       </c>
       <c r="C68" s="8" t="n">
-        <v>46234</v>
+        <v>46207</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>46114</v>
+        <v>46116</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>The Pinnacle</t>
+          <t>Lakefront Green</t>
         </is>
       </c>
       <c r="G68" s="9" t="n">
-        <v>45.36</v>
+        <v>68.01000000000001</v>
       </c>
       <c r="H68" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="I68" s="9" t="n">
-        <v>816.48</v>
+        <v>544.08</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>46216</v>
+        <v>46209</v>
       </c>
     </row>
     <row r="69">
       <c r="B69" t="inlineStr">
         <is>
-          <t>Its Murph July 4</t>
+          <t>John Summit RR</t>
         </is>
       </c>
       <c r="C69" s="8" t="n">
-        <v>46207</v>
+        <v>46120</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>46116</v>
+        <v>46117</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Lakefront Green</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G69" s="9" t="n">
-        <v>68.01000000000001</v>
+        <v>114.5</v>
       </c>
       <c r="H69" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I69" s="9" t="n">
-        <v>544.08</v>
+        <v>458</v>
       </c>
       <c r="J69" s="8" t="n">
-        <v>46209</v>
+        <v>46242</v>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>John Summit RR</t>
+          <t>Martin Garrix F1</t>
         </is>
       </c>
       <c r="C70" s="8" t="n">
-        <v>46120</v>
+        <v>46145</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>46117</v>
+        <v>46121</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Factory Town</t>
         </is>
       </c>
       <c r="G70" s="9" t="n">
-        <v>114.5</v>
+        <v>79.98999999999999</v>
       </c>
       <c r="H70" t="n">
         <v>4</v>
       </c>
       <c r="I70" s="9" t="n">
-        <v>458</v>
+        <v>319.96</v>
       </c>
       <c r="J70" s="8" t="n">
-        <v>46242</v>
+        <v>46153</v>
       </c>
     </row>
     <row r="71">
       <c r="B71" t="inlineStr">
         <is>
-          <t>Martin Garrix F1</t>
+          <t>Its Murph NYC</t>
         </is>
       </c>
       <c r="C71" s="8" t="n">
-        <v>46145</v>
+        <v>46262</v>
       </c>
       <c r="D71" s="8" t="n">
-        <v>46121</v>
+        <v>46135</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Factory Town</t>
+          <t>Under the K Bridge</t>
         </is>
       </c>
       <c r="G71" s="9" t="n">
-        <v>79.98999999999999</v>
+        <v>74.22153846153846</v>
       </c>
       <c r="H71" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="I71" s="9" t="n">
-        <v>319.96</v>
+        <v>964.88</v>
       </c>
       <c r="J71" s="8" t="n">
-        <v>46153</v>
+        <v>46262</v>
       </c>
     </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
-          <t>Its Murph NYC</t>
+          <t>Jeff Dunham</t>
         </is>
       </c>
       <c r="C72" s="8" t="n">
-        <v>46262</v>
+        <v>46180</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>46135</v>
+        <v>46153</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Under the K Bridge</t>
+          <t>Brea Improv</t>
         </is>
       </c>
       <c r="G72" s="9" t="n">
-        <v>74.22153846153846</v>
+        <v>35</v>
       </c>
       <c r="H72" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="I72" s="9" t="n">
-        <v>964.88</v>
+        <v>210</v>
       </c>
       <c r="J72" s="8" t="n">
-        <v>46262</v>
+        <v>46186</v>
       </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
         <is>
-          <t>Jeff Dunham</t>
+          <t>Dom Dolla Movement Afters</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
-        <v>46180</v>
+        <v>46167</v>
       </c>
       <c r="D73" s="8" t="n">
         <v>46153</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Brea Improv</t>
+          <t>Russell Industrial Center</t>
         </is>
       </c>
       <c r="G73" s="9" t="n">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="H73" t="n">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="I73" s="9" t="n">
-        <v>210</v>
+        <v>1980</v>
       </c>
       <c r="J73" s="8" t="n">
         <v>46186</v>
@@ -2686,95 +2694,92 @@
     <row r="74">
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dom Dolla Movement Afters</t>
+          <t>MPH DEN</t>
         </is>
       </c>
       <c r="C74" s="8" t="n">
-        <v>46167</v>
+        <v>46340</v>
       </c>
       <c r="D74" s="8" t="n">
-        <v>46153</v>
+        <v>46177</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Russell Industrial Center</t>
+          <t>Ogden Theater</t>
         </is>
       </c>
       <c r="G74" s="9" t="n">
-        <v>66</v>
+        <v>35.625</v>
       </c>
       <c r="H74" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="I74" s="9" t="n">
-        <v>1980</v>
-      </c>
-      <c r="J74" s="8" t="n">
-        <v>46186</v>
+        <v>285</v>
       </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
         <is>
-          <t>MPH DEN</t>
+          <t>Kettama Dallas</t>
         </is>
       </c>
       <c r="C75" s="8" t="n">
-        <v>46340</v>
+        <v>46318</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>46177</v>
+        <v>46186</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Ogden Theater</t>
+          <t>SILO</t>
         </is>
       </c>
       <c r="G75" s="9" t="n">
-        <v>35.625</v>
+        <v>59.41</v>
       </c>
       <c r="H75" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I75" s="9" t="n">
-        <v>285</v>
+        <v>237.64</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
         <is>
-          <t>Kettama Dallas</t>
+          <t>Kettama NYC Thursday</t>
         </is>
       </c>
       <c r="C76" s="8" t="n">
-        <v>46318</v>
+        <v>46303</v>
       </c>
       <c r="D76" s="8" t="n">
         <v>46186</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>SILO</t>
+          <t>Knockdown Center</t>
         </is>
       </c>
       <c r="G76" s="9" t="n">
-        <v>59.41</v>
+        <v>53.62</v>
       </c>
       <c r="H76" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I76" s="9" t="n">
-        <v>237.64</v>
+        <v>53.62</v>
       </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
         <is>
-          <t>Kettama NYC Thursday</t>
+          <t>Kettama NYC Friday</t>
         </is>
       </c>
       <c r="C77" s="8" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="D77" s="8" t="n">
         <v>46186</v>
@@ -2785,121 +2790,124 @@
         </is>
       </c>
       <c r="G77" s="9" t="n">
-        <v>53.62</v>
+        <v>69.06999999999999</v>
       </c>
       <c r="H77" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I77" s="9" t="n">
-        <v>53.62</v>
+        <v>276.28</v>
       </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
         <is>
-          <t>Kettama NYC Friday</t>
+          <t>Levity Mission Ballroom</t>
         </is>
       </c>
       <c r="C78" s="8" t="n">
-        <v>46304</v>
+        <v>46296</v>
       </c>
       <c r="D78" s="8" t="n">
         <v>46186</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Knockdown Center</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G78" s="9" t="n">
-        <v>69.06999999999999</v>
+        <v>90.67</v>
       </c>
       <c r="H78" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I78" s="9" t="n">
-        <v>276.28</v>
+        <v>906.7</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>Levity Mission Ballroom</t>
+          <t>Tape B RR Fri</t>
         </is>
       </c>
       <c r="C79" s="8" t="n">
-        <v>46296</v>
+        <v>46304</v>
       </c>
       <c r="D79" s="8" t="n">
-        <v>46186</v>
+        <v>46189</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G79" s="9" t="n">
-        <v>90.67</v>
+        <v>110</v>
       </c>
       <c r="H79" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I79" s="9" t="n">
-        <v>906.7</v>
+        <v>550</v>
       </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
         <is>
-          <t>Tape B RR Fri</t>
+          <t>Chris Lake LA</t>
         </is>
       </c>
       <c r="C80" s="8" t="n">
-        <v>46304</v>
+        <v>46192</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>46189</v>
+        <v>46192</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>LA state historic park</t>
         </is>
       </c>
       <c r="G80" s="9" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="H80" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I80" s="9" t="n">
-        <v>550</v>
+        <v>720</v>
+      </c>
+      <c r="J80" s="8" t="n">
+        <v>46209</v>
       </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
         <is>
-          <t>Chris Lake LA</t>
+          <t>Zeds Dead Mission</t>
         </is>
       </c>
       <c r="C81" s="8" t="n">
-        <v>46192</v>
+        <v>46207</v>
       </c>
       <c r="D81" s="8" t="n">
         <v>46192</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>LA state historic park</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G81" s="9" t="n">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="H81" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I81" s="9" t="n">
-        <v>720</v>
+        <v>700</v>
       </c>
       <c r="J81" s="8" t="n">
         <v>46209</v>
@@ -2908,14 +2916,14 @@
     <row r="82">
       <c r="B82" t="inlineStr">
         <is>
-          <t>Zeds Dead Mission</t>
+          <t>Level Up</t>
         </is>
       </c>
       <c r="C82" s="8" t="n">
-        <v>46207</v>
+        <v>46346</v>
       </c>
       <c r="D82" s="8" t="n">
-        <v>46192</v>
+        <v>46197</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -2923,233 +2931,233 @@
         </is>
       </c>
       <c r="G82" s="9" t="n">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="H82" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I82" s="9" t="n">
-        <v>700</v>
-      </c>
-      <c r="J82" s="8" t="n">
-        <v>46209</v>
+        <v>232</v>
       </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
         <is>
-          <t>Level Up</t>
+          <t>Eternal NYE</t>
         </is>
       </c>
       <c r="C83" s="8" t="n">
-        <v>46346</v>
+        <v>46386</v>
       </c>
       <c r="D83" s="8" t="n">
-        <v>46197</v>
+        <v>46203</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Orlando Amphitheater</t>
         </is>
       </c>
       <c r="G83" s="9" t="n">
-        <v>29</v>
+        <v>190.94</v>
       </c>
       <c r="H83" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I83" s="9" t="n">
-        <v>232</v>
+        <v>1145.64</v>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>Eternal NYE</t>
+          <t>HARD Afters Mau p</t>
         </is>
       </c>
       <c r="C84" s="8" t="n">
-        <v>46386</v>
+        <v>46235</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Orlando Amphitheater</t>
+          <t>Ace Mission Studios</t>
         </is>
       </c>
       <c r="G84" s="9" t="n">
-        <v>190.94</v>
+        <v>94.87</v>
       </c>
       <c r="H84" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I84" s="9" t="n">
-        <v>1145.64</v>
+        <v>379.48</v>
+      </c>
+      <c r="J84" s="8" t="n">
+        <v>46239</v>
       </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>HARD Afters Mau p</t>
+          <t>The Chainsmokers SJ</t>
         </is>
       </c>
       <c r="C85" s="8" t="n">
-        <v>46235</v>
+        <v>46269</v>
       </c>
       <c r="D85" s="8" t="n">
-        <v>46202</v>
+        <v>46209</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Ace Mission Studios</t>
+          <t>Discovery Meadow</t>
         </is>
       </c>
       <c r="G85" s="9" t="n">
-        <v>94.87</v>
+        <v>55.5</v>
       </c>
       <c r="H85" t="n">
         <v>4</v>
       </c>
       <c r="I85" s="9" t="n">
-        <v>379.48</v>
+        <v>222</v>
       </c>
       <c r="J85" s="8" t="n">
-        <v>46239</v>
+        <v>46269</v>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>The Chainsmokers SJ</t>
+          <t>Dom Dolla Belly Up</t>
         </is>
       </c>
       <c r="C86" s="8" t="n">
-        <v>46269</v>
+        <v>46242</v>
       </c>
       <c r="D86" s="8" t="n">
-        <v>46209</v>
+        <v>46210</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Discovery Meadow</t>
+          <t>Belly Up Aspen</t>
         </is>
       </c>
       <c r="G86" s="9" t="n">
-        <v>55.5</v>
+        <v>310.5</v>
       </c>
       <c r="H86" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I86" s="9" t="n">
-        <v>222</v>
+        <v>1863</v>
       </c>
       <c r="J86" s="8" t="n">
-        <v>46269</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dom Dolla Belly Up</t>
+          <t>Louis the Child Lolla Afters</t>
         </is>
       </c>
       <c r="C87" s="8" t="n">
-        <v>46242</v>
+        <v>46235</v>
       </c>
       <c r="D87" s="8" t="n">
         <v>46210</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Belly Up Aspen</t>
+          <t>Tao Chicago</t>
         </is>
       </c>
       <c r="G87" s="9" t="n">
-        <v>310.5</v>
+        <v>75</v>
       </c>
       <c r="H87" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I87" s="9" t="n">
-        <v>1863</v>
+        <v>600</v>
       </c>
       <c r="J87" s="8" t="n">
-        <v>46250</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
         <is>
-          <t>Louis the Child Lolla Afters</t>
+          <t>Illenium RR</t>
         </is>
       </c>
       <c r="C88" s="8" t="n">
-        <v>46235</v>
+        <v>46253</v>
       </c>
       <c r="D88" s="8" t="n">
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Tao Chicago</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G88" s="9" t="n">
-        <v>75</v>
+        <v>103.4</v>
       </c>
       <c r="H88" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I88" s="9" t="n">
-        <v>600</v>
+        <v>517</v>
       </c>
       <c r="J88" s="8" t="n">
-        <v>46239</v>
+        <v>46250</v>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>Illenium RR</t>
+          <t>Bunt Pacha</t>
         </is>
       </c>
       <c r="C89" s="8" t="n">
-        <v>46253</v>
+        <v>46227</v>
       </c>
       <c r="D89" s="8" t="n">
-        <v>46212</v>
+        <v>46216</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="G89" s="9" t="n">
-        <v>103.4</v>
+        <v>180</v>
       </c>
       <c r="H89" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I89" s="9" t="n">
-        <v>517</v>
+        <v>1080</v>
       </c>
       <c r="J89" s="8" t="n">
-        <v>46250</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="90">
       <c r="B90" t="inlineStr">
         <is>
-          <t>Bunt Pacha</t>
+          <t>Francis Mercier Pacha</t>
         </is>
       </c>
       <c r="C90" s="8" t="n">
-        <v>46227</v>
+        <v>46306</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>46216</v>
+        <v>46225</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3157,53 +3165,50 @@
         </is>
       </c>
       <c r="G90" s="9" t="n">
-        <v>180</v>
+        <v>45</v>
       </c>
       <c r="H90" t="n">
         <v>6</v>
       </c>
       <c r="I90" s="9" t="n">
-        <v>1080</v>
-      </c>
-      <c r="J90" s="8" t="n">
-        <v>46239</v>
+        <v>270</v>
       </c>
     </row>
     <row r="91">
       <c r="B91" t="inlineStr">
         <is>
-          <t>Francis Mercier Pacha</t>
+          <t>Dom Dolla Nashville Fri</t>
         </is>
       </c>
       <c r="C91" s="8" t="n">
-        <v>46306</v>
+        <v>46318</v>
       </c>
       <c r="D91" s="8" t="n">
         <v>46225</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>The Pinnacle</t>
         </is>
       </c>
       <c r="G91" s="9" t="n">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="H91" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I91" s="9" t="n">
-        <v>270</v>
+        <v>86</v>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>Dom Dolla Nashville Fri</t>
+          <t>Dom Dolla Nashville Sat</t>
         </is>
       </c>
       <c r="C92" s="8" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="D92" s="8" t="n">
         <v>46225</v>
@@ -3214,46 +3219,49 @@
         </is>
       </c>
       <c r="G92" s="9" t="n">
-        <v>86</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="H92" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I92" s="9" t="n">
-        <v>86</v>
+        <v>367</v>
       </c>
     </row>
     <row r="93">
       <c r="B93" t="inlineStr">
         <is>
-          <t>Dom Dolla Nashville Sat</t>
+          <t>Max Dean B2B Luke Dean LA</t>
         </is>
       </c>
       <c r="C93" s="8" t="n">
-        <v>46319</v>
+        <v>46228</v>
       </c>
       <c r="D93" s="8" t="n">
         <v>46225</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>The Pinnacle</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="G93" s="9" t="n">
-        <v>73.40000000000001</v>
+        <v>58.58</v>
       </c>
       <c r="H93" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I93" s="9" t="n">
-        <v>367</v>
+        <v>58.58</v>
+      </c>
+      <c r="J93" s="8" t="n">
+        <v>46239</v>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>Max Dean B2B Luke Dean LA</t>
+          <t>Stranger Than House NY Afters</t>
         </is>
       </c>
       <c r="C94" s="8" t="n">
@@ -3264,117 +3272,117 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Industry City</t>
         </is>
       </c>
       <c r="G94" s="9" t="n">
-        <v>58.58</v>
+        <v>47.38</v>
       </c>
       <c r="H94" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I94" s="9" t="n">
-        <v>58.58</v>
+        <v>284.28</v>
       </c>
       <c r="J94" s="8" t="n">
-        <v>46239</v>
+        <v>46226</v>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>Stranger Than House NY Afters</t>
+          <t>Anotr LA</t>
         </is>
       </c>
       <c r="C95" s="8" t="n">
-        <v>46228</v>
+        <v>46325</v>
       </c>
       <c r="D95" s="8" t="n">
-        <v>46225</v>
+        <v>46226</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Industry City</t>
+          <t>Ace Mission Studios</t>
         </is>
       </c>
       <c r="G95" s="9" t="n">
-        <v>47.38</v>
+        <v>75.39</v>
       </c>
       <c r="H95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I95" s="9" t="n">
-        <v>284.28</v>
-      </c>
-      <c r="J95" s="8" t="n">
-        <v>46226</v>
+        <v>376.95</v>
       </c>
     </row>
     <row r="96">
       <c r="B96" t="inlineStr">
         <is>
-          <t>Anotr LA</t>
+          <t>John Summit Radius Lolla</t>
         </is>
       </c>
       <c r="C96" s="8" t="n">
-        <v>46325</v>
+        <v>46233</v>
       </c>
       <c r="D96" s="8" t="n">
-        <v>46226</v>
+        <v>46239</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Ace Mission Studios</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="G96" s="9" t="n">
-        <v>75.39</v>
+        <v>132</v>
       </c>
       <c r="H96" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I96" s="9" t="n">
-        <v>376.95</v>
+        <v>132</v>
+      </c>
+      <c r="J96" s="8" t="n">
+        <v>46239</v>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>John Summit Radius Lolla</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C97" s="8" t="n">
-        <v>46233</v>
+        <v>46290</v>
       </c>
       <c r="D97" s="8" t="n">
         <v>46239</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G97" s="9" t="n">
-        <v>132</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="H97" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="I97" s="9" t="n">
-        <v>132</v>
+        <v>983</v>
       </c>
       <c r="J97" s="8" t="n">
-        <v>46239</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
-          <t>Prospa Mission</t>
+          <t>Odd Mob Mission</t>
         </is>
       </c>
       <c r="C98" s="8" t="n">
-        <v>46290</v>
+        <v>46318</v>
       </c>
       <c r="D98" s="8" t="n">
         <v>46239</v>
@@ -3385,304 +3393,304 @@
         </is>
       </c>
       <c r="G98" s="9" t="n">
-        <v>54.61111111111111</v>
+        <v>44.0625</v>
       </c>
       <c r="H98" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I98" s="9" t="n">
-        <v>983</v>
-      </c>
-      <c r="J98" s="8" t="n">
-        <v>46276</v>
+        <v>705</v>
       </c>
     </row>
     <row r="99">
       <c r="B99" t="inlineStr">
         <is>
-          <t>Odd Mob Mission</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C99" s="8" t="n">
-        <v>46318</v>
+        <v>46270</v>
       </c>
       <c r="D99" s="8" t="n">
         <v>46239</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="G99" s="9" t="n">
-        <v>44.0625</v>
+        <v>120</v>
       </c>
       <c r="H99" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I99" s="9" t="n">
-        <v>705</v>
+        <v>960</v>
+      </c>
+      <c r="J99" s="8" t="n">
+        <v>46271</v>
       </c>
     </row>
     <row r="100">
       <c r="B100" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Carl Cox LA</t>
         </is>
       </c>
       <c r="C100" s="8" t="n">
-        <v>46270</v>
+        <v>46332</v>
       </c>
       <c r="D100" s="8" t="n">
-        <v>46239</v>
+        <v>46241</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Hollywood Palladium</t>
         </is>
       </c>
       <c r="G100" s="9" t="n">
-        <v>120</v>
+        <v>59</v>
       </c>
       <c r="H100" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I100" s="9" t="n">
-        <v>960</v>
-      </c>
-      <c r="J100" s="8" t="n">
-        <v>46271</v>
+        <v>354</v>
       </c>
     </row>
     <row r="101">
       <c r="B101" t="inlineStr">
         <is>
-          <t>Carl Cox LA</t>
+          <t>Rossi Concourse</t>
         </is>
       </c>
       <c r="C101" s="8" t="n">
-        <v>46332</v>
+        <v>46367</v>
       </c>
       <c r="D101" s="8" t="n">
         <v>46241</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Hollywood Palladium</t>
+          <t>The Councourse</t>
         </is>
       </c>
       <c r="G101" s="9" t="n">
-        <v>59</v>
+        <v>23.83333333333333</v>
       </c>
       <c r="H101" t="n">
         <v>6</v>
       </c>
       <c r="I101" s="9" t="n">
-        <v>354</v>
+        <v>143</v>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>Rossi Concourse</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C102" s="8" t="n">
-        <v>46367</v>
+        <v>46242</v>
       </c>
       <c r="D102" s="8" t="n">
         <v>46241</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>The Councourse</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="G102" s="9" t="n">
-        <v>23.83333333333333</v>
+        <v>47.59</v>
       </c>
       <c r="H102" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I102" s="9" t="n">
-        <v>143</v>
+        <v>190.36</v>
+      </c>
+      <c r="J102" s="8" t="n">
+        <v>46242</v>
       </c>
     </row>
     <row r="103">
       <c r="B103" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>TWINSICK TAO</t>
         </is>
       </c>
       <c r="C103" s="8" t="n">
-        <v>46242</v>
+        <v>46270</v>
       </c>
       <c r="D103" s="8" t="n">
         <v>46241</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Tao</t>
         </is>
       </c>
       <c r="G103" s="9" t="n">
-        <v>47.59</v>
+        <v>20</v>
       </c>
       <c r="H103" t="n">
         <v>4</v>
       </c>
       <c r="I103" s="9" t="n">
-        <v>190.36</v>
+        <v>80</v>
       </c>
       <c r="J103" s="8" t="n">
-        <v>46242</v>
+        <v>46271</v>
       </c>
     </row>
     <row r="104">
       <c r="B104" t="inlineStr">
         <is>
-          <t>TWINSICK TAO</t>
+          <t>Anotr Miami</t>
         </is>
       </c>
       <c r="C104" s="8" t="n">
-        <v>46270</v>
+        <v>46360</v>
       </c>
       <c r="D104" s="8" t="n">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Watson Island Park</t>
         </is>
       </c>
       <c r="G104" s="9" t="n">
-        <v>20</v>
+        <v>121.23</v>
       </c>
       <c r="H104" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I104" s="9" t="n">
-        <v>80</v>
-      </c>
-      <c r="J104" s="8" t="n">
-        <v>46271</v>
+        <v>242.46</v>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>Anotr Miami</t>
+          <t>Levity / Tape b K Bridge</t>
         </is>
       </c>
       <c r="C105" s="8" t="n">
-        <v>46360</v>
+        <v>46256</v>
       </c>
       <c r="D105" s="8" t="n">
-        <v>46247</v>
+        <v>46250</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>K bridge</t>
         </is>
       </c>
       <c r="G105" s="9" t="n">
-        <v>121.23</v>
+        <v>95</v>
       </c>
       <c r="H105" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="I105" s="9" t="n">
-        <v>242.46</v>
+        <v>1140</v>
+      </c>
+      <c r="J105" s="8" t="n">
+        <v>46258</v>
       </c>
     </row>
     <row r="106">
       <c r="B106" t="inlineStr">
         <is>
-          <t>Levity / Tape b K Bridge</t>
+          <t>Kaytranada Pacha</t>
         </is>
       </c>
       <c r="C106" s="8" t="n">
-        <v>46256</v>
+        <v>46325</v>
       </c>
       <c r="D106" s="8" t="n">
-        <v>46250</v>
+        <v>46253</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>K bridge</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="G106" s="9" t="n">
-        <v>95</v>
+        <v>134.5</v>
       </c>
       <c r="H106" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I106" s="9" t="n">
-        <v>1140</v>
-      </c>
-      <c r="J106" s="8" t="n">
-        <v>46258</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>Kaytranada Pacha</t>
+          <t>Bunt ACL</t>
         </is>
       </c>
       <c r="C107" s="8" t="n">
-        <v>46325</v>
+        <v>46297</v>
       </c>
       <c r="D107" s="8" t="n">
         <v>46253</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Emo's Austin</t>
         </is>
       </c>
       <c r="G107" s="9" t="n">
-        <v>134.5</v>
+        <v>57.65</v>
       </c>
       <c r="H107" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="I107" s="9" t="n">
-        <v>1345</v>
+        <v>230.6</v>
       </c>
     </row>
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>Bunt ACL</t>
+          <t>Parcels ACL</t>
         </is>
       </c>
       <c r="C108" s="8" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="D108" s="8" t="n">
         <v>46253</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Emo's Austin</t>
+          <t>Stubb's Waller Creek Amphitheater</t>
         </is>
       </c>
       <c r="G108" s="9" t="n">
-        <v>57.65</v>
+        <v>65.2</v>
       </c>
       <c r="H108" t="n">
         <v>4</v>
       </c>
       <c r="I108" s="9" t="n">
-        <v>230.6</v>
+        <v>260.8</v>
+      </c>
+      <c r="J108" s="8" t="n">
+        <v>46271</v>
       </c>
     </row>
     <row r="109">
       <c r="B109" t="inlineStr">
         <is>
-          <t>Parcels ACL</t>
+          <t>Levity ACL</t>
         </is>
       </c>
       <c r="C109" s="8" t="n">
@@ -3693,144 +3701,141 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Stubb's Waller Creek Amphitheater</t>
+          <t>Emo's Austin</t>
         </is>
       </c>
       <c r="G109" s="9" t="n">
-        <v>65.2</v>
+        <v>62.52</v>
       </c>
       <c r="H109" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I109" s="9" t="n">
-        <v>260.8</v>
-      </c>
-      <c r="J109" s="8" t="n">
-        <v>46271</v>
+        <v>500.16</v>
       </c>
     </row>
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>Levity ACL</t>
+          <t>Levity Tape B NYC afters</t>
         </is>
       </c>
       <c r="C110" s="8" t="n">
-        <v>46298</v>
+        <v>46256</v>
       </c>
       <c r="D110" s="8" t="n">
         <v>46253</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Emo's Austin</t>
+          <t>Brooklyn Steel</t>
         </is>
       </c>
       <c r="G110" s="9" t="n">
-        <v>62.52</v>
+        <v>62.37</v>
       </c>
       <c r="H110" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I110" s="9" t="n">
-        <v>500.16</v>
+        <v>249.48</v>
+      </c>
+      <c r="J110" s="8" t="n">
+        <v>46258</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>Levity Tape B NYC afters</t>
+          <t>Circoloco NYC Halloween</t>
         </is>
       </c>
       <c r="C111" s="8" t="n">
-        <v>46256</v>
+        <v>46325</v>
       </c>
       <c r="D111" s="8" t="n">
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Brooklyn Steel</t>
+          <t>Brooklyn Storehouse</t>
         </is>
       </c>
       <c r="G111" s="9" t="n">
-        <v>62.37</v>
+        <v>180.25</v>
       </c>
       <c r="H111" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I111" s="9" t="n">
-        <v>249.48</v>
-      </c>
-      <c r="J111" s="8" t="n">
-        <v>46258</v>
+        <v>360.5</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>Circoloco NYC Halloween</t>
+          <t>Arc Friday Pass 2026</t>
         </is>
       </c>
       <c r="C112" s="8" t="n">
-        <v>46325</v>
+        <v>46269</v>
       </c>
       <c r="D112" s="8" t="n">
         <v>46254</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Brooklyn Storehouse</t>
+          <t>Arc</t>
         </is>
       </c>
       <c r="G112" s="9" t="n">
-        <v>180.25</v>
+        <v>219</v>
       </c>
       <c r="H112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I112" s="9" t="n">
-        <v>360.5</v>
+        <v>219</v>
+      </c>
+      <c r="J112" s="8" t="n">
+        <v>46271</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" t="inlineStr">
         <is>
-          <t>Arc Friday Pass 2026</t>
+          <t>Bunt ACL Oct 9</t>
         </is>
       </c>
       <c r="C113" s="8" t="n">
-        <v>46269</v>
+        <v>46304</v>
       </c>
       <c r="D113" s="8" t="n">
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G113" s="9" t="n">
-        <v>219</v>
+        <v>69.39</v>
       </c>
       <c r="H113" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I113" s="9" t="n">
-        <v>219</v>
-      </c>
-      <c r="J113" s="8" t="n">
-        <v>46271</v>
+        <v>208.17</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>Bunt ACL Oct 9</t>
+          <t>its murph acl</t>
         </is>
       </c>
       <c r="C114" s="8" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="D114" s="8" t="n">
         <v>46255</v>
@@ -3841,23 +3846,23 @@
         </is>
       </c>
       <c r="G114" s="9" t="n">
-        <v>69.39</v>
+        <v>81.84</v>
       </c>
       <c r="H114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I114" s="9" t="n">
-        <v>208.17</v>
+        <v>327.36</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>its murph acl</t>
+          <t>Chainsmokers ACL</t>
         </is>
       </c>
       <c r="C115" s="8" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="D115" s="8" t="n">
         <v>46255</v>
@@ -3868,46 +3873,49 @@
         </is>
       </c>
       <c r="G115" s="9" t="n">
-        <v>81.84</v>
+        <v>94.28999999999999</v>
       </c>
       <c r="H115" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="I115" s="9" t="n">
-        <v>327.36</v>
+        <v>942.9</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>Chainsmokers ACL</t>
+          <t>Chris stussy Arc Afters</t>
         </is>
       </c>
       <c r="C116" s="8" t="n">
-        <v>46296</v>
+        <v>46269</v>
       </c>
       <c r="D116" s="8" t="n">
         <v>46255</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="G116" s="9" t="n">
-        <v>94.28999999999999</v>
+        <v>100.24</v>
       </c>
       <c r="H116" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I116" s="9" t="n">
-        <v>942.9</v>
+        <v>100.24</v>
+      </c>
+      <c r="J116" s="8" t="n">
+        <v>46271</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>Chris stussy Arc Afters</t>
+          <t>Max dean ARC afters</t>
         </is>
       </c>
       <c r="C117" s="8" t="n">
@@ -3918,17 +3926,17 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Concord Music Hall</t>
         </is>
       </c>
       <c r="G117" s="9" t="n">
-        <v>100.24</v>
+        <v>42.18</v>
       </c>
       <c r="H117" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I117" s="9" t="n">
-        <v>100.24</v>
+        <v>168.72</v>
       </c>
       <c r="J117" s="8" t="n">
         <v>46271</v>
@@ -3937,239 +3945,236 @@
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>Max dean ARC afters</t>
+          <t>Rufus Du Sol Boulder Bowl</t>
         </is>
       </c>
       <c r="C118" s="8" t="n">
-        <v>46269</v>
+        <v>46256</v>
       </c>
       <c r="D118" s="8" t="n">
-        <v>46255</v>
+        <v>46256</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Concord Music Hall</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="G118" s="9" t="n">
-        <v>42.18</v>
+        <v>110</v>
       </c>
       <c r="H118" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I118" s="9" t="n">
-        <v>168.72</v>
+        <v>220</v>
       </c>
       <c r="J118" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Bowl</t>
+          <t>Goose RR</t>
         </is>
       </c>
       <c r="C119" s="8" t="n">
-        <v>46256</v>
+        <v>46266</v>
       </c>
       <c r="D119" s="8" t="n">
-        <v>46256</v>
+        <v>46262</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="G119" s="9" t="n">
-        <v>110</v>
+        <v>45</v>
       </c>
       <c r="H119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I119" s="9" t="n">
-        <v>220</v>
+        <v>45</v>
       </c>
       <c r="J119" s="8" t="n">
-        <v>46258</v>
+        <v>46267</v>
       </c>
     </row>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
-          <t>Goose RR</t>
+          <t>Josh Baker Radius</t>
         </is>
       </c>
       <c r="C120" s="8" t="n">
-        <v>46266</v>
+        <v>46353</v>
       </c>
       <c r="D120" s="8" t="n">
         <v>46262</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="G120" s="9" t="n">
-        <v>45</v>
+        <v>74.51000000000001</v>
       </c>
       <c r="H120" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I120" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="J120" s="8" t="n">
-        <v>46267</v>
+        <v>223.53</v>
       </c>
     </row>
     <row r="121">
       <c r="B121" t="inlineStr">
         <is>
-          <t>Josh Baker Radius</t>
+          <t>Josh Baker Mission</t>
         </is>
       </c>
       <c r="C121" s="8" t="n">
-        <v>46353</v>
+        <v>46351</v>
       </c>
       <c r="D121" s="8" t="n">
         <v>46262</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="G121" s="9" t="n">
-        <v>74.51000000000001</v>
+        <v>37.5</v>
       </c>
       <c r="H121" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I121" s="9" t="n">
-        <v>223.53</v>
+        <v>225</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>Josh Baker Mission</t>
+          <t>Kaytranada</t>
         </is>
       </c>
       <c r="C122" s="8" t="n">
-        <v>46351</v>
+        <v>46298</v>
       </c>
       <c r="D122" s="8" t="n">
         <v>46262</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Reframe Studios Outdoors</t>
         </is>
       </c>
       <c r="G122" s="9" t="n">
-        <v>37.5</v>
+        <v>113.3</v>
       </c>
       <c r="H122" t="n">
         <v>6</v>
       </c>
       <c r="I122" s="9" t="n">
-        <v>225</v>
+        <v>679.8</v>
       </c>
     </row>
     <row r="123">
       <c r="B123" t="inlineStr">
         <is>
-          <t>Kaytranada</t>
+          <t>Jigitz Ogden</t>
         </is>
       </c>
       <c r="C123" s="8" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="D123" s="8" t="n">
-        <v>46262</v>
+        <v>46263</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Reframe Studios Outdoors</t>
+          <t>Ogden</t>
         </is>
       </c>
       <c r="G123" s="9" t="n">
-        <v>113.3</v>
+        <v>59.48999999999999</v>
       </c>
       <c r="H123" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="I123" s="9" t="n">
-        <v>679.8</v>
+        <v>1070.82</v>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>Jigitz Ogden</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C124" s="8" t="n">
-        <v>46305</v>
+        <v>46263</v>
       </c>
       <c r="D124" s="8" t="n">
         <v>46263</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Ogden</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="G124" s="9" t="n">
-        <v>59.48999999999999</v>
+        <v>151.76</v>
       </c>
       <c r="H124" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="I124" s="9" t="n">
-        <v>1070.82</v>
+        <v>303.52</v>
+      </c>
+      <c r="J124" s="8" t="n">
+        <v>46263</v>
       </c>
     </row>
     <row r="125">
       <c r="B125" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Music on Pacha</t>
         </is>
       </c>
       <c r="C125" s="8" t="n">
-        <v>46263</v>
+        <v>46311</v>
       </c>
       <c r="D125" s="8" t="n">
-        <v>46263</v>
+        <v>46267</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="G125" s="9" t="n">
-        <v>151.76</v>
+        <v>140</v>
       </c>
       <c r="H125" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I125" s="9" t="n">
-        <v>303.52</v>
-      </c>
-      <c r="J125" s="8" t="n">
-        <v>46263</v>
+        <v>840</v>
       </c>
     </row>
     <row r="126">
       <c r="B126" t="inlineStr">
         <is>
-          <t>Music on Pacha</t>
+          <t>Nervous Records Pacha</t>
         </is>
       </c>
       <c r="C126" s="8" t="n">
-        <v>46311</v>
+        <v>46333</v>
       </c>
       <c r="D126" s="8" t="n">
         <v>46267</v>
@@ -4180,103 +4185,103 @@
         </is>
       </c>
       <c r="G126" s="9" t="n">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="H126" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I126" s="9" t="n">
-        <v>840</v>
+        <v>400</v>
       </c>
     </row>
     <row r="127">
       <c r="B127" t="inlineStr">
         <is>
-          <t>Nervous Records Pacha</t>
+          <t>Ian Asher Concourse</t>
         </is>
       </c>
       <c r="C127" s="8" t="n">
-        <v>46333</v>
+        <v>46319</v>
       </c>
       <c r="D127" s="8" t="n">
         <v>46267</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G127" s="9" t="n">
-        <v>50</v>
+        <v>50.72</v>
       </c>
       <c r="H127" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I127" s="9" t="n">
-        <v>400</v>
+        <v>304.32</v>
       </c>
     </row>
     <row r="128">
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ian Asher Concourse</t>
+          <t>jamie xx NY</t>
         </is>
       </c>
       <c r="C128" s="8" t="n">
-        <v>46319</v>
+        <v>46269</v>
       </c>
       <c r="D128" s="8" t="n">
         <v>46267</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>Public Records</t>
         </is>
       </c>
       <c r="G128" s="9" t="n">
-        <v>50.72</v>
+        <v>49.44</v>
       </c>
       <c r="H128" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I128" s="9" t="n">
-        <v>304.32</v>
+        <v>49.44</v>
+      </c>
+      <c r="J128" s="8" t="n">
+        <v>46271</v>
       </c>
     </row>
     <row r="129">
       <c r="B129" t="inlineStr">
         <is>
-          <t>jamie xx NY</t>
+          <t>Franky Rizardo GA Concourse</t>
         </is>
       </c>
       <c r="C129" s="8" t="n">
-        <v>46269</v>
+        <v>46359</v>
       </c>
       <c r="D129" s="8" t="n">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Public Records</t>
+          <t>Councourse</t>
         </is>
       </c>
       <c r="G129" s="9" t="n">
-        <v>49.44</v>
+        <v>44.49</v>
       </c>
       <c r="H129" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I129" s="9" t="n">
-        <v>49.44</v>
-      </c>
-      <c r="J129" s="8" t="n">
-        <v>46271</v>
+        <v>266.94</v>
       </c>
     </row>
     <row r="130">
       <c r="B130" t="inlineStr">
         <is>
-          <t>Franky Rizardo GA Concourse</t>
+          <t>Franky Rizardo VIP Concourse</t>
         </is>
       </c>
       <c r="C130" s="8" t="n">
@@ -4287,84 +4292,84 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Councourse</t>
+          <t>Concourse</t>
         </is>
       </c>
       <c r="G130" s="9" t="n">
-        <v>44.49</v>
+        <v>81.84</v>
       </c>
       <c r="H130" t="n">
         <v>6</v>
       </c>
       <c r="I130" s="9" t="n">
-        <v>266.94</v>
+        <v>491.04</v>
       </c>
     </row>
     <row r="131">
       <c r="B131" t="inlineStr">
         <is>
-          <t>Franky Rizardo VIP Concourse</t>
+          <t>Mellow Circus LA</t>
         </is>
       </c>
       <c r="C131" s="8" t="n">
-        <v>46359</v>
+        <v>46326</v>
       </c>
       <c r="D131" s="8" t="n">
         <v>46268</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Concourse</t>
+          <t>TBA</t>
         </is>
       </c>
       <c r="G131" s="9" t="n">
-        <v>81.84</v>
+        <v>84.61</v>
       </c>
       <c r="H131" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I131" s="9" t="n">
-        <v>491.04</v>
+        <v>169.22</v>
       </c>
     </row>
     <row r="132">
       <c r="B132" t="inlineStr">
         <is>
-          <t>Mellow Circus LA</t>
+          <t>Prospa Miami Space</t>
         </is>
       </c>
       <c r="C132" s="8" t="n">
-        <v>46326</v>
+        <v>46357</v>
       </c>
       <c r="D132" s="8" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Space</t>
         </is>
       </c>
       <c r="G132" s="9" t="n">
-        <v>84.61</v>
+        <v>120</v>
       </c>
       <c r="H132" t="n">
         <v>2</v>
       </c>
       <c r="I132" s="9" t="n">
-        <v>169.22</v>
+        <v>240</v>
       </c>
     </row>
     <row r="133">
       <c r="B133" t="inlineStr">
         <is>
-          <t>Prospa Miami Space</t>
+          <t>Art Basel Miami 3am</t>
         </is>
       </c>
       <c r="C133" s="8" t="n">
-        <v>46357</v>
+        <v>46360</v>
       </c>
       <c r="D133" s="8" t="n">
-        <v>46269</v>
+        <v>46274</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -4372,207 +4377,180 @@
         </is>
       </c>
       <c r="G133" s="9" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="H133" t="n">
         <v>2</v>
       </c>
       <c r="I133" s="9" t="n">
-        <v>240</v>
+        <v>160</v>
       </c>
     </row>
     <row r="134">
       <c r="B134" t="inlineStr">
         <is>
-          <t>Art Basel Miami 3am</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C134" s="8" t="n">
-        <v>46360</v>
+        <v>46309</v>
       </c>
       <c r="D134" s="8" t="n">
         <v>46274</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Space</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="G134" s="9" t="n">
-        <v>80</v>
+        <v>59.99</v>
       </c>
       <c r="H134" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="I134" s="9" t="n">
-        <v>160</v>
+        <v>719.88</v>
       </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
         <is>
-          <t>Prospa Wednesday LA</t>
+          <t>Cloonee Belly Up</t>
         </is>
       </c>
       <c r="C135" s="8" t="n">
-        <v>46309</v>
+        <v>46382</v>
       </c>
       <c r="D135" s="8" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Shrine</t>
+          <t>Belly up</t>
         </is>
       </c>
       <c r="G135" s="9" t="n">
-        <v>59.99</v>
+        <v>198</v>
       </c>
       <c r="H135" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I135" s="9" t="n">
-        <v>719.88</v>
+        <v>396</v>
       </c>
     </row>
     <row r="136">
       <c r="B136" t="inlineStr">
         <is>
-          <t>Cloonee Belly Up</t>
+          <t>Adriatique B2B Cloonee</t>
         </is>
       </c>
       <c r="C136" s="8" t="n">
-        <v>46382</v>
+        <v>46361</v>
       </c>
       <c r="D136" s="8" t="n">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Belly up</t>
+          <t>Watson Island Park</t>
         </is>
       </c>
       <c r="G136" s="9" t="n">
-        <v>198</v>
+        <v>103.05</v>
       </c>
       <c r="H136" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I136" s="9" t="n">
-        <v>396</v>
+        <v>412.2</v>
+      </c>
+      <c r="J136" s="8" t="n">
+        <v>46276</v>
       </c>
     </row>
     <row r="137">
       <c r="B137" t="inlineStr">
         <is>
-          <t>Adriatique B2B Cloonee</t>
+          <t>Pawsa LA</t>
         </is>
       </c>
       <c r="C137" s="8" t="n">
-        <v>46361</v>
+        <v>46312</v>
       </c>
       <c r="D137" s="8" t="n">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>Historic Sers Building</t>
         </is>
       </c>
       <c r="G137" s="9" t="n">
-        <v>103.05</v>
+        <v>108</v>
       </c>
       <c r="H137" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I137" s="9" t="n">
-        <v>412.2</v>
-      </c>
-      <c r="J137" s="8" t="n">
-        <v>46276</v>
+        <v>648</v>
       </c>
     </row>
     <row r="138">
       <c r="B138" t="inlineStr">
         <is>
-          <t>Pawsa LA</t>
+          <t>Ben Sterling Afters Sound</t>
         </is>
       </c>
       <c r="C138" s="8" t="n">
-        <v>46312</v>
+        <v>46277</v>
       </c>
       <c r="D138" s="8" t="n">
         <v>46279</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Historic Sers Building</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="G138" s="9" t="n">
-        <v>108</v>
+        <v>47.59</v>
       </c>
       <c r="H138" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I138" s="9" t="n">
-        <v>648</v>
+        <v>190.36</v>
+      </c>
+      <c r="J138" s="8" t="n">
+        <v>46279</v>
       </c>
     </row>
     <row r="139">
       <c r="B139" t="inlineStr">
         <is>
-          <t>Ben Sterling Afters Sound</t>
+          <t>CircoLoco Miami Sat</t>
         </is>
       </c>
       <c r="C139" s="8" t="n">
-        <v>46277</v>
+        <v>46361</v>
       </c>
       <c r="D139" s="8" t="n">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Factory Town</t>
         </is>
       </c>
       <c r="G139" s="9" t="n">
-        <v>47.59</v>
+        <v>174.99</v>
       </c>
       <c r="H139" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I139" s="9" t="n">
-        <v>190.36</v>
-      </c>
-      <c r="J139" s="8" t="n">
-        <v>46279</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>CircoLoco Miami Sat</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="n">
-        <v>46361</v>
-      </c>
-      <c r="D140" s="8" t="n">
-        <v>46283</v>
-      </c>
-      <c r="F140" t="inlineStr">
-        <is>
-          <t>Factory Town</t>
-        </is>
-      </c>
-      <c r="G140" s="9" t="n">
-        <v>174.99</v>
-      </c>
-      <c r="H140" t="n">
-        <v>2</v>
-      </c>
-      <c r="I140" s="9" t="n">
         <v>349.98</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Pending sheet to Excel export and matching dashboard section
export.py now writes a third Pending sheet alongside BL/SL, listing
scraped-but-unpromoted (source='email') transactions. It's purely
informational and never feeds Net Profit/ROI. dashboard.py gets a
matching "Pending purchases" table below the existing pending-review
notice, additive to the existing excel-sourced metrics section.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet name="BL" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pending" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -14420,4 +14421,110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Venue</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Event Date</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Purchase Date</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Quantity</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Price per Ticket</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Total Price</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Review Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GRiZ - Free Shows for the People</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JUNKYARD — Denver, CO</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>46292</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>46283</v>
+      </c>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Ticketmaster</t>
+        </is>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: pipeline run 2026-09-21 (13 new transactions, 188 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14429,7 +14429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14524,6 +14524,529 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>46286.08380787037</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46286.06381944445</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46286.02076388889</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>220</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>418</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46286.01179398148</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46286.00988425926</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>220</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>660</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46286.00737268518</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>600</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PACHA NEW YORK</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>total_price missing from email content</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PACHA NEW YORK</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46285.98454861111</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>total_price and price_per_ticket not stated in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PACHA NEW YORK</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46285.79740740741</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>total_price and currency missing from confirmation email</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>46285.79673611111</v>
+      </c>
+      <c r="F13" t="n">
+        <v>6</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>1128</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>46285.79628472222</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>1128</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>46285.79575231481</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>1128</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J15" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-21 (3 new transactions, 188 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14429,7 +14429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15047,6 +15047,116 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>46286.80615740741</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>1200</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Circoloco Halloween (Friday)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Brooklyn Storehouse</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>46286.80028935185</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>770</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Experts Only Festival After Party - Sunday</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>46286.13207175926</v>
+      </c>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Text content not supported for this email, quantity and price cannot be extracted</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-22 (3 new transactions, 188 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14429,7 +14429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15157,6 +15157,127 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Four Tet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>46287.79021990741</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Four Tet - Admissions</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>46287.79016203704</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="9" t="n"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>total_price missing from ticket transfer notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Four Tet</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>52.43</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>52.43</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-23 (13 new transactions, 188 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14429,7 +14429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15278,6 +15278,481 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Prospa - Admissions</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>46288.86873842592</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="9" t="n"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="9" t="n"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Quantity and pricing details not provided in listing deletion email</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>46288.82011574074</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver, CO</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver, CO</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="9" t="n"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>46288.76680555556</v>
+      </c>
+      <c r="G28" s="9" t="n"/>
+      <c r="H28" s="9" t="n"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>quantity and pricing not stated in email body</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>46288.76528935185</v>
+      </c>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="9" t="n"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J30" t="b">
+        <v>1</v>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>quantity and pricing not stated for deleted ticket listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>jigitz - Admissions</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>46288.73217592593</v>
+      </c>
+      <c r="F31" t="n">
+        <v>6</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>116.55</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>699.3</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>46288.72925925926</v>
+      </c>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J32" t="b">
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>quantity and pricing not stated in email body</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>46288.72884259259</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="H33" s="9" t="n"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>total_price not applicable for a ticket listing confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>46288.72767361111</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="9" t="n"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: re-ingest 13 rows broken by platform/HTML/listing bugs
Deleted email rows 497-506, 512, 522, 526 and re-extracted uids 67, 85,
86, 87-91, 93-95, 177, 183 with the fixed pipeline: 10 rows saved
(ids 529-538), 3 listing-only emails (87, 89, 93) correctly skipped.
Re-ran match.py and export.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14429,7 +14429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14527,7 +14527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14544,16 +14544,16 @@
         <v>46285</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>46286.08380787037</v>
+        <v>46285.79673611111</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>230</v>
+        <v>1128</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -14567,7 +14567,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -14584,16 +14584,16 @@
         <v>46285</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46286.06381944445</v>
+        <v>46285.79628472222</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>230</v>
+        <v>1128</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -14607,7 +14607,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -14624,16 +14624,16 @@
         <v>46285</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>46286.02076388889</v>
+        <v>46285.79575231481</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>418</v>
+        <v>1128</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -14652,28 +14652,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Pawsa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Historic Sears Building</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46285</v>
+        <v>46312</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>46286.01179398148</v>
+        <v>46286.80615740741</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G6" s="9" t="n">
         <v>200</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>200</v>
+        <v>1200</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -14692,28 +14692,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Circoloco Halloween (Friday)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Brooklyn Storehouse</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46285</v>
+        <v>46325</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>46286.00988425926</v>
+        <v>46286.80028935185</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>220</v>
+        <v>400</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>660</v>
+        <v>770</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -14727,37 +14727,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Four Tet</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46286.00737268518</v>
+        <v>46287.79021990741</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>200</v>
+        <v>41.4</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>400</v>
+        <v>41.4</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J8" t="b">
@@ -14767,41 +14767,42 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Four Tet - Admissions</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom, Denver , CO</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46285</v>
+        <v>46287.79016203704</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>600</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J9" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>total_price missing from ticket transfer notification</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -14812,60 +14813,59 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Four Tet</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46285</v>
+        <v>46287</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
+      <c r="G10" s="9" t="n">
+        <v>52.43</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>52.43</v>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J10" t="b">
-        <v>1</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>total_price missing from email content</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa - Admissions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Mission Ballroom, Denver , CO</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>46285</v>
+        <v>46290</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46285.98454861111</v>
+        <v>46288.86873842592</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -14874,39 +14874,34 @@
       <c r="H11" s="9" t="n"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J11" t="b">
-        <v>1</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>total_price and price_per_ticket not stated in email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D12" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46285.79740740741</v>
+        <v>46288</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -14915,92 +14910,85 @@
       <c r="H12" s="9" t="n"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J12" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>total_price and currency missing from confirmation email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>46285.79673611111</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>180</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>1128</v>
-      </c>
+        <v>46288</v>
+      </c>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J13" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Quantity and pricing details not provided in listing deletion email</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>46285.79628472222</v>
+        <v>46288.82011574074</v>
       </c>
       <c r="F14" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>180</v>
+        <v>100.65</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>1128</v>
+        <v>100.65</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J14" t="b">
@@ -15010,37 +14998,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom, Denver, CO</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>46285</v>
+        <v>46290</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46285.79575231481</v>
+        <v>46288</v>
       </c>
       <c r="F15" t="n">
-        <v>6</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>180</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>1128</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J15" t="b">
@@ -15055,32 +15039,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Pawsa</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Historic Sears Building</t>
+          <t>Mission Ballroom, Denver, CO</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>46312</v>
+        <v>46290</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>46286.80615740741</v>
+        <v>46288</v>
       </c>
       <c r="F16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>1200</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J16" t="b">
@@ -15095,32 +15075,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Circoloco Halloween (Friday)</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Brooklyn Storehouse</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>46325</v>
+        <v>46309</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46286.80028935185</v>
+        <v>46288</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>770</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J17" t="b">
@@ -15135,17 +15111,25 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Experts Only Festival After Party - Sunday</t>
-        </is>
+          <t>Prospa present Prophecy - Admissions</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>46309</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>46286.13207175926</v>
+        <v>46288.76528935185</v>
       </c>
       <c r="G18" s="9" t="n"/>
       <c r="H18" s="9" t="n"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J18" t="b">
@@ -15153,44 +15137,44 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Text content not supported for this email, quantity and price cannot be extracted</t>
+          <t>quantity and pricing not stated for deleted ticket listing</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Four Tet</t>
+          <t>jigitz - Admissions</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Ogden Theatre</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>46289</v>
+        <v>46305</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>46287.79021990741</v>
+        <v>46288.73217592593</v>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>41.4</v>
+        <v>116.55</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>41.4</v>
+        <v>699.3</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J19" t="b">
@@ -15200,29 +15184,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Four Tet - Admissions</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver , CO</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>46289</v>
+        <v>46309</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46287.79016203704</v>
+        <v>46288.72884259259</v>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" s="9" t="n"/>
+        <v>5</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>100.65</v>
+      </c>
       <c r="H20" s="9" t="n"/>
       <c r="I20" t="inlineStr">
         <is>
@@ -15234,44 +15220,40 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>total_price missing from ticket transfer notification</t>
+          <t>total_price not applicable for a ticket listing confirmation</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Four Tet</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>46289</v>
+        <v>46309</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>46287</v>
+        <v>46288.72767361111</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="9" t="n">
-        <v>52.43</v>
-      </c>
-      <c r="H21" s="9" t="n">
-        <v>52.43</v>
-      </c>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -15281,33 +15263,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Prospa - Admissions</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver , CO</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>46290</v>
+        <v>46285</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>46288.86873842592</v>
+        <v>46285</v>
       </c>
       <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
+      <c r="G22" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>326</v>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J22" t="b">
@@ -15317,33 +15303,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>46288</v>
+        <v>46285</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="9" t="n"/>
-      <c r="H23" s="9" t="n"/>
+      <c r="G23" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>326</v>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -15353,39 +15343,41 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="G24" s="9" t="n"/>
-      <c r="H24" s="9" t="n"/>
+        <v>46285.98454861111</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>326</v>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J24" t="b">
-        <v>1</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Quantity and pricing details not provided in listing deletion email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -15396,32 +15388,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>46288.82011574074</v>
+        <v>46286</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>100.65</v>
+        <v>200</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>100.65</v>
+        <v>400</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J25" t="b">
@@ -15436,28 +15428,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver, CO</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D26" s="8" t="n">
-        <v>46290</v>
+        <v>46285</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>46288</v>
+        <v>46286.01179398148</v>
       </c>
       <c r="F26" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="9" t="n"/>
-      <c r="H26" s="9" t="n"/>
+      <c r="G26" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>200</v>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J26" t="b">
@@ -15472,28 +15468,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver, CO</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D27" s="8" t="n">
-        <v>46290</v>
+        <v>46285</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" s="9" t="n"/>
-      <c r="H27" s="9" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>220</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>440</v>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J27" t="b">
@@ -15508,26 +15508,36 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Prospa</t>
-        </is>
+          <t>Experts Only (Sunday Afters)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>46285</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>46288.76680555556</v>
-      </c>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="9" t="n"/>
+        <v>46286.08380787037</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>230</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>230</v>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J28" t="b">
-        <v>1</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>quantity and pricing not stated in email body</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -15538,28 +15548,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival After Party - Sunday</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Pacha New York</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="F29" t="n">
-        <v>4</v>
-      </c>
-      <c r="G29" s="9" t="n"/>
-      <c r="H29" s="9" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>319.48</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>638.96</v>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J29" t="b">
@@ -15574,34 +15588,36 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
         <v>46309</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>46288.76528935185</v>
-      </c>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
+        <v>46288.72925925926</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>quantity and pricing not stated for deleted ticket listing</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -15612,144 +15628,35 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>jigitz - Admissions</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ogden Theatre</t>
+          <t>Shrine Auditorium and Expo Hall</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>46305</v>
+        <v>46309</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>46288.73217592593</v>
+        <v>46288.76680555556</v>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>116.55</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>699.3</v>
+        <v>372.4</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J31" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>46288.72925925926</v>
-      </c>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="J32" t="b">
-        <v>1</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>quantity and pricing not stated in email body</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Prospa present Prophecy - Admissions</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E33" s="8" t="n">
-        <v>46288.72884259259</v>
-      </c>
-      <c r="F33" t="n">
-        <v>5</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <v>100.65</v>
-      </c>
-      <c r="H33" s="9" t="n"/>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>AXS</t>
-        </is>
-      </c>
-      <c r="J33" t="b">
-        <v>1</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>total_price not applicable for a ticket listing confirmation</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Prospa present Prophecy - Admissions</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E34" s="8" t="n">
-        <v>46288.72767361111</v>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>AXS</t>
-        </is>
-      </c>
-      <c r="J34" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-24 (3 new transactions, 196 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N139"/>
+  <dimension ref="A1:N143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3373,7 +3373,7 @@
         <v>983</v>
       </c>
       <c r="J97" s="8" t="n">
-        <v>46276</v>
+        <v>46288</v>
       </c>
     </row>
     <row r="98">
@@ -4413,6 +4413,9 @@
       <c r="I134" s="9" t="n">
         <v>719.88</v>
       </c>
+      <c r="J134" s="8" t="n">
+        <v>46288</v>
+      </c>
     </row>
     <row r="135">
       <c r="B135" t="inlineStr">
@@ -4553,6 +4556,120 @@
       </c>
       <c r="I139" s="9" t="n">
         <v>349.98</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Griz Free Show 7PM</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="n">
+        <v>46292</v>
+      </c>
+      <c r="D140" s="8" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Junkyard</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="n">
+        <v>2</v>
+      </c>
+      <c r="I140" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Griz Free Show 1Pm</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="n">
+        <v>46292</v>
+      </c>
+      <c r="D141" s="8" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Junkyard</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="n">
+        <v>1</v>
+      </c>
+      <c r="I141" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C142" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D142" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="H142" t="n">
+        <v>6</v>
+      </c>
+      <c r="I142" s="9" t="n">
+        <v>1128</v>
+      </c>
+      <c r="J142" s="8" t="n">
+        <v>46288</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="D143" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="G143" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H143" t="n">
+        <v>3</v>
+      </c>
+      <c r="I143" s="9" t="n">
+        <v>978</v>
+      </c>
+      <c r="J143" s="8" t="n">
+        <v>46288</v>
       </c>
     </row>
   </sheetData>
@@ -4566,7 +4683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O189"/>
+  <dimension ref="A1:O197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5093,7 +5210,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -5145,7 +5262,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -5197,7 +5314,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -5301,7 +5418,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -5353,7 +5470,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -5457,7 +5574,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -5509,7 +5626,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -5561,7 +5678,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -5613,7 +5730,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -5665,7 +5782,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -5717,7 +5834,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -5769,7 +5886,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -5821,7 +5938,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -5873,7 +5990,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -5925,7 +6042,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -5977,7 +6094,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -6133,7 +6250,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -6185,7 +6302,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -6445,7 +6562,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -6497,7 +6614,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -6549,7 +6666,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -6653,7 +6770,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -6809,7 +6926,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -6861,7 +6978,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -6913,7 +7030,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -6965,7 +7082,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -7017,7 +7134,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -7069,7 +7186,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -7121,7 +7238,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -7485,7 +7602,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -7537,7 +7654,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -7589,7 +7706,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Stubuhb</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -8109,7 +8226,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -8941,7 +9058,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -9461,7 +9578,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Crowd Volt</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -9617,7 +9734,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -9669,7 +9786,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -10861,7 +10978,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -11017,7 +11134,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -11121,7 +11238,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -11745,7 +11862,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>crowdvolt</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -11849,7 +11966,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -12421,7 +12538,7 @@
       </c>
       <c r="J151" t="inlineStr">
         <is>
-          <t>Lysed</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K151" t="inlineStr">
@@ -12733,7 +12850,7 @@
       </c>
       <c r="J157" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K157" t="inlineStr">
@@ -12837,7 +12954,7 @@
       </c>
       <c r="J159" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K159" t="inlineStr">
@@ -13149,7 +13266,7 @@
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
@@ -13436,32 +13553,32 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D171" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E171" s="8" t="n">
-        <v>46271</v>
+        <v>46288</v>
       </c>
       <c r="G171" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H171" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I171" s="9" t="n">
-        <v>87.5</v>
+        <v>121.72</v>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>Crowdvolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
@@ -13470,16 +13587,16 @@
         </is>
       </c>
       <c r="L171" s="9" t="n">
-        <v>350</v>
+        <v>243.44</v>
       </c>
       <c r="M171" s="9" t="n">
-        <v>350</v>
+        <v>243.44</v>
       </c>
       <c r="N171" s="9" t="n">
-        <v>-130</v>
+        <v>134.2177777777778</v>
       </c>
       <c r="O171" s="7" t="n">
-        <v>-0.2708333333333333</v>
+        <v>1.228850457782299</v>
       </c>
     </row>
     <row r="172">
@@ -13509,11 +13626,11 @@
         <v>120</v>
       </c>
       <c r="I172" s="9" t="n">
-        <v>92.41500000000001</v>
+        <v>87.5</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -13522,16 +13639,16 @@
         </is>
       </c>
       <c r="L172" s="9" t="n">
-        <v>369.66</v>
+        <v>350</v>
       </c>
       <c r="M172" s="9" t="n">
-        <v>369.66</v>
+        <v>350</v>
       </c>
       <c r="N172" s="9" t="n">
-        <v>-110.34</v>
+        <v>-130</v>
       </c>
       <c r="O172" s="7" t="n">
-        <v>-0.2298749999999999</v>
+        <v>-0.2708333333333333</v>
       </c>
     </row>
     <row r="173">
@@ -13540,32 +13657,32 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D173" s="8" t="n">
-        <v>46242</v>
+        <v>46270</v>
       </c>
       <c r="E173" s="8" t="n">
-        <v>46242</v>
+        <v>46271</v>
       </c>
       <c r="G173" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H173" s="9" t="n">
-        <v>47.59</v>
+        <v>120</v>
       </c>
       <c r="I173" s="9" t="n">
-        <v>52</v>
+        <v>92.41500000000001</v>
       </c>
       <c r="J173" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K173" t="inlineStr">
@@ -13574,16 +13691,16 @@
         </is>
       </c>
       <c r="L173" s="9" t="n">
-        <v>52</v>
+        <v>369.66</v>
       </c>
       <c r="M173" s="9" t="n">
-        <v>52</v>
+        <v>369.66</v>
       </c>
       <c r="N173" s="9" t="n">
-        <v>4.409999999999997</v>
+        <v>-110.34</v>
       </c>
       <c r="O173" s="7" t="n">
-        <v>0.09266652658121446</v>
+        <v>-0.2298749999999999</v>
       </c>
     </row>
     <row r="174">
@@ -13613,11 +13730,11 @@
         <v>47.59</v>
       </c>
       <c r="I174" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -13626,16 +13743,16 @@
         </is>
       </c>
       <c r="L174" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M174" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="N174" s="9" t="n">
-        <v>7.409999999999997</v>
+        <v>4.409999999999997</v>
       </c>
       <c r="O174" s="7" t="n">
-        <v>0.155704980037823</v>
+        <v>0.09266652658121446</v>
       </c>
     </row>
     <row r="175">
@@ -13659,17 +13776,17 @@
         <v>46242</v>
       </c>
       <c r="G175" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H175" s="9" t="n">
         <v>47.59</v>
       </c>
       <c r="I175" s="9" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -13678,16 +13795,16 @@
         </is>
       </c>
       <c r="L175" s="9" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="M175" s="9" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="N175" s="9" t="n">
-        <v>-9.180000000000007</v>
+        <v>7.409999999999997</v>
       </c>
       <c r="O175" s="7" t="n">
-        <v>-0.09644883378861112</v>
+        <v>0.155704980037823</v>
       </c>
     </row>
     <row r="176">
@@ -13696,32 +13813,32 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>TWINSICK TAO</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D176" s="8" t="n">
-        <v>46270</v>
+        <v>46242</v>
       </c>
       <c r="E176" s="8" t="n">
-        <v>46271</v>
+        <v>46242</v>
       </c>
       <c r="G176" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H176" s="9" t="n">
-        <v>20</v>
+        <v>47.59</v>
       </c>
       <c r="I176" s="9" t="n">
-        <v>27.05</v>
+        <v>43</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -13730,16 +13847,16 @@
         </is>
       </c>
       <c r="L176" s="9" t="n">
-        <v>108.2</v>
+        <v>86</v>
       </c>
       <c r="M176" s="9" t="n">
-        <v>108.2</v>
+        <v>86</v>
       </c>
       <c r="N176" s="9" t="n">
-        <v>28.2</v>
+        <v>-9.180000000000007</v>
       </c>
       <c r="O176" s="7" t="n">
-        <v>0.3525</v>
+        <v>-0.09644883378861112</v>
       </c>
     </row>
     <row r="177">
@@ -13748,32 +13865,32 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Levity / Tape b K Bridge</t>
+          <t>TWINSICK TAO</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>K bridge</t>
+          <t>Tao</t>
         </is>
       </c>
       <c r="D177" s="8" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="E177" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G177" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H177" s="9" t="n">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="I177" s="9" t="n">
-        <v>90</v>
+        <v>27.05</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K177" t="inlineStr">
@@ -13782,16 +13899,16 @@
         </is>
       </c>
       <c r="L177" s="9" t="n">
-        <v>1080</v>
+        <v>108.2</v>
       </c>
       <c r="M177" s="9" t="n">
-        <v>1080</v>
+        <v>108.2</v>
       </c>
       <c r="N177" s="9" t="n">
-        <v>-60</v>
+        <v>28.2</v>
       </c>
       <c r="O177" s="7" t="n">
-        <v>-0.05263157894736842</v>
+        <v>0.3525</v>
       </c>
     </row>
     <row r="178">
@@ -13800,32 +13917,32 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Parcels ACL</t>
+          <t>Levity / Tape b K Bridge</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Stubb's Waller Creek Amphitheater</t>
+          <t>K bridge</t>
         </is>
       </c>
       <c r="D178" s="8" t="n">
-        <v>46298</v>
+        <v>46256</v>
       </c>
       <c r="E178" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
       <c r="G178" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H178" s="9" t="n">
-        <v>65.2</v>
+        <v>95</v>
       </c>
       <c r="I178" s="9" t="n">
-        <v>54.1</v>
+        <v>90</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -13834,16 +13951,16 @@
         </is>
       </c>
       <c r="L178" s="9" t="n">
-        <v>54.1</v>
+        <v>1080</v>
       </c>
       <c r="M178" s="9" t="n">
-        <v>54.1</v>
+        <v>1080</v>
       </c>
       <c r="N178" s="9" t="n">
-        <v>-11.1</v>
+        <v>-60</v>
       </c>
       <c r="O178" s="7" t="n">
-        <v>-0.1702453987730062</v>
+        <v>-0.05263157894736842</v>
       </c>
     </row>
     <row r="179">
@@ -13852,32 +13969,32 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Levity Tape B NYC afters</t>
+          <t>Parcels ACL</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Brooklyn Steel</t>
+          <t>Stubb's Waller Creek Amphitheater</t>
         </is>
       </c>
       <c r="D179" s="8" t="n">
-        <v>46256</v>
+        <v>46298</v>
       </c>
       <c r="E179" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G179" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H179" s="9" t="n">
-        <v>62.37</v>
+        <v>65.2</v>
       </c>
       <c r="I179" s="9" t="n">
-        <v>44.25</v>
+        <v>54.1</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>crowdvolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -13886,16 +14003,16 @@
         </is>
       </c>
       <c r="L179" s="9" t="n">
-        <v>177</v>
+        <v>54.1</v>
       </c>
       <c r="M179" s="9" t="n">
-        <v>177</v>
+        <v>54.1</v>
       </c>
       <c r="N179" s="9" t="n">
-        <v>-72.47999999999999</v>
+        <v>-11.1</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>-0.2905242905242905</v>
+        <v>-0.1702453987730062</v>
       </c>
     </row>
     <row r="180">
@@ -13904,32 +14021,32 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Arc Friday Pass 2026</t>
+          <t>Levity Tape B NYC afters</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Brooklyn Steel</t>
         </is>
       </c>
       <c r="D180" s="8" t="n">
-        <v>46269</v>
+        <v>46256</v>
       </c>
       <c r="E180" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
       <c r="G180" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H180" s="9" t="n">
-        <v>219</v>
+        <v>62.37</v>
       </c>
       <c r="I180" s="9" t="n">
-        <v>162.28</v>
+        <v>44.25</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -13938,16 +14055,16 @@
         </is>
       </c>
       <c r="L180" s="9" t="n">
-        <v>162.28</v>
+        <v>177</v>
       </c>
       <c r="M180" s="9" t="n">
-        <v>162.28</v>
+        <v>177</v>
       </c>
       <c r="N180" s="9" t="n">
-        <v>-56.72</v>
+        <v>-72.47999999999999</v>
       </c>
       <c r="O180" s="7" t="n">
-        <v>-0.2589954337899543</v>
+        <v>-0.2905242905242905</v>
       </c>
     </row>
     <row r="181">
@@ -13956,12 +14073,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Chris stussy Arc Afters</t>
+          <t>Arc Friday Pass 2026</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Arc</t>
         </is>
       </c>
       <c r="D181" s="8" t="n">
@@ -13974,10 +14091,10 @@
         <v>1</v>
       </c>
       <c r="H181" s="9" t="n">
-        <v>100.24</v>
+        <v>219</v>
       </c>
       <c r="I181" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
@@ -13990,16 +14107,16 @@
         </is>
       </c>
       <c r="L181" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="M181" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="N181" s="9" t="n">
-        <v>16.97</v>
+        <v>-56.72</v>
       </c>
       <c r="O181" s="7" t="n">
-        <v>0.169293695131684</v>
+        <v>-0.2589954337899543</v>
       </c>
     </row>
     <row r="182">
@@ -14008,12 +14125,12 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Max dean ARC afters</t>
+          <t>Chris stussy Arc Afters</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Concord Music Hall</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="D182" s="8" t="n">
@@ -14023,13 +14140,13 @@
         <v>46271</v>
       </c>
       <c r="G182" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H182" s="9" t="n">
-        <v>42.18</v>
+        <v>100.24</v>
       </c>
       <c r="I182" s="9" t="n">
-        <v>63.1125</v>
+        <v>117.21</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
@@ -14042,16 +14159,16 @@
         </is>
       </c>
       <c r="L182" s="9" t="n">
-        <v>252.45</v>
+        <v>117.21</v>
       </c>
       <c r="M182" s="9" t="n">
-        <v>252.45</v>
+        <v>117.21</v>
       </c>
       <c r="N182" s="9" t="n">
-        <v>83.72999999999999</v>
+        <v>16.97</v>
       </c>
       <c r="O182" s="7" t="n">
-        <v>0.4962660028449501</v>
+        <v>0.169293695131684</v>
       </c>
     </row>
     <row r="183">
@@ -14060,28 +14177,28 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Bowl</t>
+          <t>Max dean ARC afters</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>Concord Music Hall</t>
         </is>
       </c>
       <c r="D183" s="8" t="n">
-        <v>46256</v>
+        <v>46269</v>
       </c>
       <c r="E183" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G183" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H183" s="9" t="n">
-        <v>110</v>
+        <v>42.18</v>
       </c>
       <c r="I183" s="9" t="n">
-        <v>243.43</v>
+        <v>63.1125</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -14094,16 +14211,16 @@
         </is>
       </c>
       <c r="L183" s="9" t="n">
-        <v>486.86</v>
+        <v>252.45</v>
       </c>
       <c r="M183" s="9" t="n">
-        <v>486.86</v>
+        <v>252.45</v>
       </c>
       <c r="N183" s="9" t="n">
-        <v>266.86</v>
+        <v>83.72999999999999</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>1.213</v>
+        <v>0.4962660028449501</v>
       </c>
     </row>
     <row r="184">
@@ -14112,32 +14229,32 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Goose RR</t>
+          <t>Rufus Du Sol Boulder Bowl</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="D184" s="8" t="n">
-        <v>46266</v>
+        <v>46256</v>
       </c>
       <c r="E184" s="8" t="n">
-        <v>46267</v>
+        <v>46258</v>
       </c>
       <c r="G184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H184" s="9" t="n">
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="I184" s="9" t="n">
-        <v>0</v>
+        <v>243.43</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -14146,16 +14263,16 @@
         </is>
       </c>
       <c r="L184" s="9" t="n">
-        <v>0</v>
+        <v>486.86</v>
       </c>
       <c r="M184" s="9" t="n">
-        <v>0</v>
+        <v>486.86</v>
       </c>
       <c r="N184" s="9" t="n">
-        <v>-45</v>
+        <v>266.86</v>
       </c>
       <c r="O184" s="7" t="n">
-        <v>-1</v>
+        <v>1.213</v>
       </c>
     </row>
     <row r="185">
@@ -14164,32 +14281,32 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Goose RR</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="D185" s="8" t="n">
-        <v>46263</v>
+        <v>46266</v>
       </c>
       <c r="E185" s="8" t="n">
-        <v>46263</v>
+        <v>46267</v>
       </c>
       <c r="G185" t="n">
         <v>1</v>
       </c>
       <c r="H185" s="9" t="n">
-        <v>151.76</v>
+        <v>45</v>
       </c>
       <c r="I185" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -14198,16 +14315,16 @@
         </is>
       </c>
       <c r="L185" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="M185" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="N185" s="9" t="n">
-        <v>71.75</v>
+        <v>-45</v>
       </c>
       <c r="O185" s="7" t="n">
-        <v>0.4727859778597786</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="186">
@@ -14237,7 +14354,7 @@
         <v>151.76</v>
       </c>
       <c r="I186" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -14250,16 +14367,16 @@
         </is>
       </c>
       <c r="L186" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="M186" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="N186" s="9" t="n">
-        <v>78.24000000000001</v>
+        <v>71.75</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>0.5155508697944123</v>
+        <v>0.4727859778597786</v>
       </c>
     </row>
     <row r="187">
@@ -14268,32 +14385,32 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>jamie xx NY</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Public Records</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D187" s="8" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="E187" s="8" t="n">
-        <v>46271</v>
+        <v>46263</v>
       </c>
       <c r="G187" t="n">
         <v>1</v>
       </c>
       <c r="H187" s="9" t="n">
-        <v>49.44</v>
+        <v>151.76</v>
       </c>
       <c r="I187" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -14302,16 +14419,16 @@
         </is>
       </c>
       <c r="L187" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="M187" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="N187" s="9" t="n">
-        <v>-49.44</v>
+        <v>78.24000000000001</v>
       </c>
       <c r="O187" s="7" t="n">
-        <v>-1</v>
+        <v>0.5155508697944123</v>
       </c>
     </row>
     <row r="188">
@@ -14320,32 +14437,32 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Adriatique B2B Cloonee</t>
+          <t>jamie xx NY</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>Public Records</t>
         </is>
       </c>
       <c r="D188" s="8" t="n">
-        <v>46361</v>
+        <v>46269</v>
       </c>
       <c r="E188" s="8" t="n">
-        <v>46276</v>
+        <v>46271</v>
       </c>
       <c r="G188" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H188" s="9" t="n">
-        <v>103.05</v>
+        <v>49.44</v>
       </c>
       <c r="I188" s="9" t="n">
-        <v>103.05</v>
+        <v>0</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -14354,16 +14471,16 @@
         </is>
       </c>
       <c r="L188" s="9" t="n">
-        <v>412.2</v>
+        <v>0</v>
       </c>
       <c r="M188" s="9" t="n">
-        <v>412.2</v>
+        <v>0</v>
       </c>
       <c r="N188" s="9" t="n">
-        <v>0</v>
+        <v>-49.44</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="189">
@@ -14372,50 +14489,466 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
+          <t>Prospa Wednesday LA</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Shrine</t>
+        </is>
+      </c>
+      <c r="D189" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E189" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G189" t="n">
+        <v>5</v>
+      </c>
+      <c r="H189" s="9" t="n">
+        <v>59.98999999999999</v>
+      </c>
+      <c r="I189" s="9" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L189" s="9" t="n">
+        <v>428</v>
+      </c>
+      <c r="M189" s="9" t="n">
+        <v>428</v>
+      </c>
+      <c r="N189" s="9" t="n">
+        <v>128.05</v>
+      </c>
+      <c r="O189" s="7" t="n">
+        <v>0.4269044840806802</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Adriatique B2B Cloonee</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Watson Island Park</t>
+        </is>
+      </c>
+      <c r="D190" s="8" t="n">
+        <v>46361</v>
+      </c>
+      <c r="E190" s="8" t="n">
+        <v>46276</v>
+      </c>
+      <c r="G190" t="n">
+        <v>4</v>
+      </c>
+      <c r="H190" s="9" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="I190" s="9" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>Refund</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L190" s="9" t="n">
+        <v>412.2</v>
+      </c>
+      <c r="M190" s="9" t="n">
+        <v>412.2</v>
+      </c>
+      <c r="N190" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O190" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
           <t>Ben Sterling Afters Sound</t>
         </is>
       </c>
-      <c r="C189" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>Sound</t>
         </is>
       </c>
-      <c r="D189" s="8" t="n">
+      <c r="D191" s="8" t="n">
         <v>46277</v>
       </c>
-      <c r="E189" s="8" t="n">
+      <c r="E191" s="8" t="n">
         <v>46279</v>
       </c>
-      <c r="G189" t="n">
+      <c r="G191" t="n">
         <v>4</v>
       </c>
-      <c r="H189" s="9" t="n">
+      <c r="H191" s="9" t="n">
         <v>47.59</v>
       </c>
-      <c r="I189" s="9" t="n">
+      <c r="I191" s="9" t="n">
         <v>75.5</v>
       </c>
-      <c r="J189" t="inlineStr">
+      <c r="J191" t="inlineStr">
         <is>
           <t>CrowdVolt</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L189" s="9" t="n">
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L191" s="9" t="n">
         <v>302</v>
       </c>
-      <c r="M189" s="9" t="n">
+      <c r="M191" s="9" t="n">
         <v>302</v>
       </c>
-      <c r="N189" s="9" t="n">
+      <c r="N191" s="9" t="n">
         <v>111.64</v>
       </c>
-      <c r="O189" s="7" t="n">
+      <c r="O191" s="7" t="n">
         <v>0.586467745324648</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D192" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E192" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G192" t="n">
+        <v>1</v>
+      </c>
+      <c r="H192" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I192" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L192" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="M192" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="N192" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="O192" s="7" t="n">
+        <v>0.1595744680851064</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D193" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E193" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G193" t="n">
+        <v>2</v>
+      </c>
+      <c r="H193" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I193" s="9" t="n">
+        <v>209</v>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L193" s="9" t="n">
+        <v>418</v>
+      </c>
+      <c r="M193" s="9" t="n">
+        <v>418</v>
+      </c>
+      <c r="N193" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="O193" s="7" t="n">
+        <v>0.1117021276595745</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D194" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E194" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G194" t="n">
+        <v>1</v>
+      </c>
+      <c r="H194" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I194" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L194" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="M194" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="N194" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O194" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D195" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E195" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G195" t="n">
+        <v>2</v>
+      </c>
+      <c r="H195" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I195" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L195" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="M195" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="N195" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O195" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D196" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E196" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G196" t="n">
+        <v>2</v>
+      </c>
+      <c r="H196" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="I196" s="9" t="n">
+        <v>293.92</v>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L196" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="M196" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="N196" s="9" t="n">
+        <v>-64.15999999999997</v>
+      </c>
+      <c r="O196" s="7" t="n">
+        <v>-0.09840490797546007</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D197" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E197" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G197" t="n">
+        <v>1</v>
+      </c>
+      <c r="H197" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="I197" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L197" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="M197" s="9" t="n">
+        <v>253</v>
+      </c>
+      <c r="N197" s="9" t="n">
+        <v>-73</v>
+      </c>
+      <c r="O197" s="7" t="n">
+        <v>-0.2239263803680982</v>
       </c>
     </row>
   </sheetData>
@@ -14429,7 +14962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15660,6 +16193,126 @@
         <v>0</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: re-ingest 9 rows broken by listing/platform/duplicate-order bugs
Deleted unpromoted email rows 507-511, 519, 524, 525, 527 (none in
matches) and re-extracted uids 64-66, 113, 114, 176, 178, 181, 188 with
the fixed pipeline (9ce9de4), in ascending uid order:
- uid 64 saved as id 554: CrowdVolt buy, order T97962, Experts Only
  (Sunday Afters) at Pacha 2026-09-20 22:00, 6 x GA @ $180, $1128 total
  after fees -- verified against the email text
- uids 65, 66 ("tickets delivered" for T97962) skipped as duplicate order
- uid 181 (AXS "you deleted your ticket listing") skipped as delisting
- uids 113, 114, 176, 178, 188 (listing confirmations) skipped as listings
Re-ran match.py (unchanged: 196 pairs, $9,627.92) and export.py
(Pending 33 -> 25 rows).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14962,7 +14962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15065,32 +15065,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Four Tet</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>46285.79673611111</v>
+        <v>46287.79021990741</v>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>180</v>
+        <v>41.4</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>1128</v>
+        <v>41.4</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J3" t="b">
@@ -15105,36 +15105,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Four Tet - Admissions</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom, Denver , CO</t>
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46285.79628472222</v>
+        <v>46287.79016203704</v>
       </c>
       <c r="F4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" s="9" t="n">
-        <v>180</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>1128</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>total_price missing from ticket transfer notification</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -15145,32 +15146,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Four Tet</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46285</v>
+        <v>46289</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>46285.79575231481</v>
+        <v>46287</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>180</v>
+        <v>52.43</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>1128</v>
+        <v>52.43</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J5" t="b">
@@ -15185,32 +15186,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pawsa</t>
+          <t>Prospa - Admissions</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Historic Sears Building</t>
+          <t>Mission Ballroom, Denver , CO</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46312</v>
+        <v>46290</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>46286.80615740741</v>
+        <v>46288.86873842592</v>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>1200</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J6" t="b">
@@ -15225,32 +15222,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Circoloco Halloween (Friday)</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Brooklyn Storehouse</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46325</v>
+        <v>46309</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>46286.80028935185</v>
+        <v>46288</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>770</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J7" t="b">
@@ -15260,64 +15253,62 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Four Tet</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>46289</v>
+        <v>46309</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46287.79021990741</v>
-      </c>
-      <c r="F8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
         <v>1</v>
       </c>
-      <c r="G8" s="9" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>41.4</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>StubHub</t>
-        </is>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Quantity and pricing details not provided in listing deletion email</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Four Tet - Admissions</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver , CO</t>
+          <t>Mission Ballroom, Denver, CO</t>
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46287.79016203704</v>
+        <v>46288</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
@@ -15330,48 +15321,39 @@
         </is>
       </c>
       <c r="J9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>total_price missing from ticket transfer notification</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Four Tet</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Mission Ballroom, Denver, CO</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
-      <c r="G10" s="9" t="n">
-        <v>52.43</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>52.43</v>
-      </c>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J10" t="b">
@@ -15386,22 +15368,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Prospa - Admissions</t>
+          <t>Prospa present Prophecy - Admissions</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver , CO</t>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>46290</v>
+        <v>46309</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46288.86873842592</v>
+        <v>46288</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G11" s="9" t="n"/>
       <c r="H11" s="9" t="n"/>
@@ -15434,7 +15416,7 @@
         <v>46309</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>46288</v>
+        <v>46288.72767361111</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -15453,75 +15435,77 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
+        <v>46285</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>326</v>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J13" t="b">
-        <v>1</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Quantity and pricing details not provided in listing deletion email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D14" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>46288.82011574074</v>
+        <v>46285</v>
       </c>
       <c r="F14" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>100.65</v>
+        <v>326</v>
       </c>
       <c r="H14" s="9" t="n">
-        <v>100.65</v>
+        <v>326</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J14" t="b">
@@ -15531,33 +15515,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>Experts Only Festival Afterparty</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver, CO</t>
+          <t>PACHA NEW YORK</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>46290</v>
+        <v>46285</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46288</v>
+        <v>46285.98454861111</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
+      <c r="G15" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>326</v>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Fourvenues</t>
         </is>
       </c>
       <c r="J15" t="b">
@@ -15572,28 +15560,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mission Ballroom, Denver, CO</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D16" s="8" t="n">
-        <v>46290</v>
+        <v>46285</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>46288</v>
+        <v>46286</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="9" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>400</v>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J16" t="b">
@@ -15608,28 +15600,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46288</v>
+        <v>46286.01179398148</v>
       </c>
       <c r="F17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="9" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H17" s="9" t="n">
+        <v>200</v>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J17" t="b">
@@ -15644,34 +15640,36 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>46288.76528935185</v>
-      </c>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
+        <v>46286</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>220</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>440</v>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>quantity and pricing not stated for deleted ticket listing</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -15682,32 +15680,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>jigitz - Admissions</t>
+          <t>Experts Only (Sunday Afters)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ogden Theatre</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>46305</v>
+        <v>46285</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>46288.73217592593</v>
+        <v>46286.08380787037</v>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>116.55</v>
+        <v>230</v>
       </c>
       <c r="H19" s="9" t="n">
-        <v>699.3</v>
+        <v>230</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J19" t="b">
@@ -15722,39 +15720,36 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Experts Only Festival After Party - Sunday</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Pacha New York</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>46309</v>
+        <v>46285</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46288.72884259259</v>
+        <v>46286</v>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>100.65</v>
-      </c>
-      <c r="H20" s="9" t="n"/>
+        <v>319.48</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>638.96</v>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>total_price not applicable for a ticket listing confirmation</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -15765,28 +15760,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Prospa present Prophecy - Admissions</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Shrine Expo Hall, Los Angeles, CA</t>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
         <v>46309</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>46288.72767361111</v>
+        <v>46288.72925925926</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
+      <c r="G21" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -15796,37 +15795,37 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Shrine Auditorium and Expo Hall</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>46285</v>
+        <v>46288.76680555556</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>326</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>326</v>
+        <v>372.4</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Fourvenues</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J22" t="b">
@@ -15836,37 +15835,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Shrine Auditorium and Expo Hall</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="F23" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>326</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>326</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Fourvenues</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -15876,37 +15875,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D24" s="8" t="n">
-        <v>46285</v>
+        <v>46290</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>46285.98454861111</v>
+        <v>46288</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>326</v>
+        <v>132.3</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>326</v>
+        <v>132.3</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Fourvenues</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J24" t="b">
@@ -15921,32 +15920,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters)</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>46285</v>
+        <v>46290</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>200</v>
+        <v>132.3</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>400</v>
+        <v>132.3</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J25" t="b">
@@ -15956,7 +15955,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -15973,16 +15972,16 @@
         <v>46285</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>46286.01179398148</v>
+        <v>46285.79575231481</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>200</v>
+        <v>1128</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -15990,326 +15989,6 @@
         </is>
       </c>
       <c r="J26" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E27" s="8" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>220</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <v>440</v>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J27" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E28" s="8" t="n">
-        <v>46286.08380787037</v>
-      </c>
-      <c r="F28" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>230</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>230</v>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J28" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Experts Only Festival After Party - Sunday</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Pacha New York</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>319.48</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>638.96</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J29" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>46288.72925925926</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J30" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E31" s="8" t="n">
-        <v>46288.76680555556</v>
-      </c>
-      <c r="F31" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H31" s="9" t="n">
-        <v>372.4</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J31" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E32" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J32" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E33" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="H33" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J33" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E34" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J34" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Export: leave rows already recorded in Excel out of the Pending sheet
export.load_data now filters unpromoted email rows through
crosscheck.find_excel_matches, the same check the dashboard uses, so the
Pending sheet in EmailScrape.xlsx lists only rows that still need
action. The summary prints how many were left out.

Re-exported: Pending 16 -> 3 rows (GRiZ free show, Four Tet $52.43,
Prospa $93.10), 13 left out as already in Excel; BL and SL sheets have
identical cell values to before.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14962,7 +14962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15100,560 +15100,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PACHA NEW YORK</t>
+          <t>Shrine Auditorium and Expo Hall</t>
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46285</v>
+        <v>46288</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>326</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>326</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Fourvenues</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Experts Only Festival Afterparty</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>PACHA NEW YORK</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Fourvenues</t>
-        </is>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Experts Only Festival Afterparty</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>PACHA NEW YORK</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>46285.98454861111</v>
-      </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Fourvenues</t>
-        </is>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>400</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>46286.01179398148</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>200</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F9" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>220</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>440</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>46286.08380787037</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>230</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>230</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Experts Only Festival After Party - Sunday</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Pacha New York</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>46286</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>319.48</v>
-      </c>
-      <c r="H11" s="9" t="n">
-        <v>638.96</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>46288.72925925926</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H12" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E13" s="8" t="n">
-        <v>46288.76680555556</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H13" s="9" t="n">
-        <v>372.4</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Shrine Auditorium and Expo Hall</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="n">
-        <v>46309</v>
-      </c>
-      <c r="E14" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H14" s="9" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J14" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E15" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="H15" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>46288</v>
-      </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="H16" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Experts Only (Sunday Afters)</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Pacha</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>46285</v>
-      </c>
-      <c r="E17" s="8" t="n">
-        <v>46285.79575231481</v>
-      </c>
-      <c r="F17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" s="9" t="n">
-        <v>180</v>
-      </c>
-      <c r="H17" s="9" t="n">
-        <v>1128</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J17" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-24 (8 new transactions, 5 skipped, 196 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14962,7 +14962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15137,6 +15137,286 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GRiZMAS 2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Masonic Temple Theatre</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46374</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46289.59476851852</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>52.22</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>567.84</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MGMT (DJ Set)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46289.42085648148</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>153.08</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MGMT (DJ Set)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46289.42576388889</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>153.08</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46289.75697916667</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>132.3</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>133.28</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>133.28</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46289.81953703704</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>136.22</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>136.22</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>139.16</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>139.16</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-24 (1 new transactions, 1 skipped, 196 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15025,32 +15025,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GRiZ - Free Shows for the People</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JUNKYARD — Denver, CO</t>
+          <t>Shrine Auditorium and Expo Hall</t>
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46292</v>
+        <v>46309</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>46283</v>
-      </c>
-      <c r="G2" s="9" t="n"/>
+        <v>46288</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
       <c r="H2" s="9" t="n">
-        <v>0</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Ticketmaster</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J2" t="b">
@@ -15065,32 +15070,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Four Tet</t>
+          <t>GRiZMAS 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Masonic Temple Theatre</t>
         </is>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46289</v>
+        <v>46374</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>46287</v>
+        <v>46289.59476851852</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>52.43</v>
+        <v>52.22</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>52.43</v>
+        <v>567.84</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J3" t="b">
@@ -15100,37 +15105,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>MGMT (DJ Set)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Shrine Auditorium and Expo Hall</t>
+          <t>The Concourse Project</t>
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>46309</v>
+        <v>46312</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46288</v>
+        <v>46289.42085648148</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>93.09999999999999</v>
+        <v>30</v>
       </c>
       <c r="H4" s="9" t="n">
-        <v>93.09999999999999</v>
+        <v>153.08</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>See Tickets</t>
         </is>
       </c>
       <c r="J4" t="b">
@@ -15145,32 +15150,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>GRiZMAS 2026</t>
+          <t>MGMT (DJ Set)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Masonic Temple Theatre</t>
+          <t>The Concourse Project</t>
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>46374</v>
+        <v>46312</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>46289.59476851852</v>
+        <v>46289.42576388889</v>
       </c>
       <c r="F5" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>52.22</v>
+        <v>30</v>
       </c>
       <c r="H5" s="9" t="n">
-        <v>567.84</v>
+        <v>153.08</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>See Tickets</t>
         </is>
       </c>
       <c r="J5" t="b">
@@ -15180,37 +15185,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MGMT (DJ Set)</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The Concourse Project</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>46312</v>
+        <v>46290</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>46289.42085648148</v>
+        <v>46289.75697916667</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>30</v>
+        <v>132.3</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>153.08</v>
+        <v>132.3</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>See Tickets</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J6" t="b">
@@ -15220,37 +15225,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MGMT (DJ Set)</t>
+          <t>Prospa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The Concourse Project</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>46312</v>
+        <v>46290</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>46289.42576388889</v>
+        <v>46289</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>30</v>
+        <v>133.28</v>
       </c>
       <c r="H7" s="9" t="n">
-        <v>153.08</v>
+        <v>133.28</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>See Tickets</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J7" t="b">
@@ -15277,16 +15282,16 @@
         <v>46290</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46289.75697916667</v>
+        <v>46289.81953703704</v>
       </c>
       <c r="F8" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>132.3</v>
+        <v>136.22</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>132.3</v>
+        <v>136.22</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -15317,16 +15322,16 @@
         <v>46290</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46289</v>
+        <v>46289.82378472222</v>
       </c>
       <c r="F9" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>133.28</v>
+        <v>139.16</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>133.28</v>
+        <v>139.16</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -15357,16 +15362,16 @@
         <v>46290</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>46289.81953703704</v>
+        <v>46289</v>
       </c>
       <c r="F10" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>136.22</v>
+        <v>139.16</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>136.22</v>
+        <v>139.16</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -15397,7 +15402,7 @@
         <v>46290</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>46289</v>
+        <v>46289.84034722222</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-25 (1 new transactions, 1 skipped, 196 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -14962,7 +14962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15422,6 +15422,31 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46290.59245370371</v>
+      </c>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>quantity not stated and event details missing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sync workbook into DB (19 added, 7 updated, 202 matched pairs)
import_excel.py --apply, after backup transactions.backup-20260925-140339-pre-excel-sync.db:
- BL added rows 145-157: 12 Harry Styles buys (AZ/Dallas/Chicago 2027)
  and Four Tet Missionballroom, $9,214.99 total
- SL added SIDs 200-205: Prospa Mission 9/25 sales ($132.30-$139.16)
- BL row 124 Jigitz Ogden: qty 18 -> 12, total $1,070.82 -> $740.82
  (edited in the sheet after import; no matches used this buy)
- platform casing to match the sheet: BL rows 14, 38, 43 DICE -> Dice,
  83 Axs -> AXS; SL SIDs 47, 62 Stubhub -> StubHub
No rows removed; no email rows touched.

Excel buys now total $78,538.62, equal to the workbook's Expenses.
match.py: 196 -> 202 pairs, net profit $9,627.92 -> $10,054.01.
export.py: Pending 5 rows (Prospa email sales 558-563 now auto-match).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N143"/>
+  <dimension ref="A1:N156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3373,7 +3373,7 @@
         <v>983</v>
       </c>
       <c r="J97" s="8" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="98">
@@ -4102,13 +4102,13 @@
         </is>
       </c>
       <c r="G123" s="9" t="n">
-        <v>59.48999999999999</v>
+        <v>61.73499999999999</v>
       </c>
       <c r="H123" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="I123" s="9" t="n">
-        <v>1070.82</v>
+        <v>740.8199999999999</v>
       </c>
     </row>
     <row r="124">
@@ -4670,6 +4670,357 @@
       </c>
       <c r="J143" s="8" t="n">
         <v>46288</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Harry Styles AZ Fri Sec 421 Row 10</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="n">
+        <v>46479</v>
+      </c>
+      <c r="D144" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>State Farm Stadium</t>
+        </is>
+      </c>
+      <c r="G144" s="9" t="n">
+        <v>91.45999999999999</v>
+      </c>
+      <c r="H144" t="n">
+        <v>5</v>
+      </c>
+      <c r="I144" s="9" t="n">
+        <v>457.3</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Harry Styles AZ Sat 4/3/27 Sec 409 Row 10</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="n">
+        <v>46480</v>
+      </c>
+      <c r="D145" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>State Farm Stadium</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="n">
+        <v>91.45999999999999</v>
+      </c>
+      <c r="H145" t="n">
+        <v>2</v>
+      </c>
+      <c r="I145" s="9" t="n">
+        <v>182.92</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Harry Styles AZ Sat 4/3/27 GA Rear</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="n">
+        <v>46480</v>
+      </c>
+      <c r="D146" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>State farm Statidum</t>
+        </is>
+      </c>
+      <c r="G146" s="9" t="n">
+        <v>245.21</v>
+      </c>
+      <c r="H146" t="n">
+        <v>1</v>
+      </c>
+      <c r="I146" s="9" t="n">
+        <v>245.21</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/9 Dallas Sec 426</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="n">
+        <v>46486</v>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G147" s="9" t="n">
+        <v>166.13</v>
+      </c>
+      <c r="H147" t="n">
+        <v>2</v>
+      </c>
+      <c r="I147" s="9" t="n">
+        <v>332.26</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/9 Dallas Sec C212</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="n">
+        <v>46486</v>
+      </c>
+      <c r="D148" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G148" s="9" t="n">
+        <v>332.24</v>
+      </c>
+      <c r="H148" t="n">
+        <v>4</v>
+      </c>
+      <c r="I148" s="9" t="n">
+        <v>1328.96</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/10 Dallas Sec C213</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="n">
+        <v>46487</v>
+      </c>
+      <c r="D149" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G149" s="9" t="n">
+        <v>332.24</v>
+      </c>
+      <c r="H149" t="n">
+        <v>2</v>
+      </c>
+      <c r="I149" s="9" t="n">
+        <v>664.48</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/16 Dallas Sec 123</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="n">
+        <v>46493</v>
+      </c>
+      <c r="D150" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G150" s="9" t="n">
+        <v>332.24</v>
+      </c>
+      <c r="H150" t="n">
+        <v>2</v>
+      </c>
+      <c r="I150" s="9" t="n">
+        <v>664.48</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/16 Dallas Sec 413</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="n">
+        <v>46493</v>
+      </c>
+      <c r="D151" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G151" s="9" t="n">
+        <v>79.73999999999999</v>
+      </c>
+      <c r="H151" t="n">
+        <v>2</v>
+      </c>
+      <c r="I151" s="9" t="n">
+        <v>159.48</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/16 Dallas Sec C134</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="n">
+        <v>46493</v>
+      </c>
+      <c r="D152" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G152" s="9" t="n">
+        <v>398.69</v>
+      </c>
+      <c r="H152" t="n">
+        <v>6</v>
+      </c>
+      <c r="I152" s="9" t="n">
+        <v>2392.14</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Harry Styles 4/16 Dallas Sec FLRGA3</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="n">
+        <v>46493</v>
+      </c>
+      <c r="D153" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G153" s="9" t="n">
+        <v>265.79</v>
+      </c>
+      <c r="H153" t="n">
+        <v>5</v>
+      </c>
+      <c r="I153" s="9" t="n">
+        <v>1328.95</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Harry Styles 6/4 Chicago Sec 332</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="n">
+        <v>46542</v>
+      </c>
+      <c r="D154" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Soldier Field</t>
+        </is>
+      </c>
+      <c r="G154" s="9" t="n">
+        <v>157.49</v>
+      </c>
+      <c r="H154" t="n">
+        <v>1</v>
+      </c>
+      <c r="I154" s="9" t="n">
+        <v>157.49</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Harry Styles 6/5 Chicago Sec 134</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="n">
+        <v>46543</v>
+      </c>
+      <c r="D155" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Soldier Field</t>
+        </is>
+      </c>
+      <c r="G155" s="9" t="n">
+        <v>314.98</v>
+      </c>
+      <c r="H155" t="n">
+        <v>4</v>
+      </c>
+      <c r="I155" s="9" t="n">
+        <v>1259.92</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Four Tet Missionballroom</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="D156" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="G156" s="9" t="n">
+        <v>41.4</v>
+      </c>
+      <c r="H156" t="n">
+        <v>1</v>
+      </c>
+      <c r="I156" s="9" t="n">
+        <v>41.4</v>
       </c>
     </row>
   </sheetData>
@@ -4683,7 +5034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O197"/>
+  <dimension ref="A1:O203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6146,7 +6497,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -11550,7 +11901,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>Stubhub</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -13605,32 +13956,32 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D172" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E172" s="8" t="n">
-        <v>46271</v>
+        <v>46289</v>
       </c>
       <c r="G172" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H172" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I172" s="9" t="n">
-        <v>87.5</v>
+        <v>128.03</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K172" t="inlineStr">
@@ -13639,16 +13990,16 @@
         </is>
       </c>
       <c r="L172" s="9" t="n">
-        <v>350</v>
+        <v>128.03</v>
       </c>
       <c r="M172" s="9" t="n">
-        <v>350</v>
+        <v>128.03</v>
       </c>
       <c r="N172" s="9" t="n">
-        <v>-130</v>
+        <v>73.41888888888889</v>
       </c>
       <c r="O172" s="7" t="n">
-        <v>-0.2708333333333333</v>
+        <v>1.34439471007121</v>
       </c>
     </row>
     <row r="173">
@@ -13657,28 +14008,28 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D173" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E173" s="8" t="n">
-        <v>46271</v>
+        <v>46289</v>
       </c>
       <c r="G173" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H173" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I173" s="9" t="n">
-        <v>92.41500000000001</v>
+        <v>128.03</v>
       </c>
       <c r="J173" t="inlineStr">
         <is>
@@ -13691,16 +14042,16 @@
         </is>
       </c>
       <c r="L173" s="9" t="n">
-        <v>369.66</v>
+        <v>128.03</v>
       </c>
       <c r="M173" s="9" t="n">
-        <v>369.66</v>
+        <v>128.03</v>
       </c>
       <c r="N173" s="9" t="n">
-        <v>-110.34</v>
+        <v>73.41888888888889</v>
       </c>
       <c r="O173" s="7" t="n">
-        <v>-0.2298749999999999</v>
+        <v>1.34439471007121</v>
       </c>
     </row>
     <row r="174">
@@ -13709,32 +14060,32 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D174" s="8" t="n">
-        <v>46242</v>
+        <v>46290</v>
       </c>
       <c r="E174" s="8" t="n">
-        <v>46242</v>
+        <v>46289</v>
       </c>
       <c r="G174" t="n">
         <v>1</v>
       </c>
       <c r="H174" s="9" t="n">
-        <v>47.59</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I174" s="9" t="n">
-        <v>52</v>
+        <v>128.03</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K174" t="inlineStr">
@@ -13743,16 +14094,16 @@
         </is>
       </c>
       <c r="L174" s="9" t="n">
-        <v>52</v>
+        <v>128.03</v>
       </c>
       <c r="M174" s="9" t="n">
-        <v>52</v>
+        <v>128.03</v>
       </c>
       <c r="N174" s="9" t="n">
-        <v>4.409999999999997</v>
+        <v>73.41888888888889</v>
       </c>
       <c r="O174" s="7" t="n">
-        <v>0.09266652658121446</v>
+        <v>1.34439471007121</v>
       </c>
     </row>
     <row r="175">
@@ -13761,32 +14112,32 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D175" s="8" t="n">
-        <v>46242</v>
+        <v>46290</v>
       </c>
       <c r="E175" s="8" t="n">
-        <v>46242</v>
+        <v>46289</v>
       </c>
       <c r="G175" t="n">
         <v>1</v>
       </c>
       <c r="H175" s="9" t="n">
-        <v>47.59</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I175" s="9" t="n">
-        <v>55</v>
+        <v>125.32</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K175" t="inlineStr">
@@ -13795,16 +14146,16 @@
         </is>
       </c>
       <c r="L175" s="9" t="n">
-        <v>55</v>
+        <v>125.32</v>
       </c>
       <c r="M175" s="9" t="n">
-        <v>55</v>
+        <v>125.32</v>
       </c>
       <c r="N175" s="9" t="n">
-        <v>7.409999999999997</v>
+        <v>70.70888888888888</v>
       </c>
       <c r="O175" s="7" t="n">
-        <v>0.155704980037823</v>
+        <v>1.294771108850457</v>
       </c>
     </row>
     <row r="176">
@@ -13813,32 +14164,32 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D176" s="8" t="n">
-        <v>46242</v>
+        <v>46290</v>
       </c>
       <c r="E176" s="8" t="n">
-        <v>46242</v>
+        <v>46289</v>
       </c>
       <c r="G176" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H176" s="9" t="n">
-        <v>47.59</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I176" s="9" t="n">
-        <v>43</v>
+        <v>122.62</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K176" t="inlineStr">
@@ -13847,16 +14198,16 @@
         </is>
       </c>
       <c r="L176" s="9" t="n">
-        <v>86</v>
+        <v>122.62</v>
       </c>
       <c r="M176" s="9" t="n">
-        <v>86</v>
+        <v>122.62</v>
       </c>
       <c r="N176" s="9" t="n">
-        <v>-9.180000000000007</v>
+        <v>68.00888888888889</v>
       </c>
       <c r="O176" s="7" t="n">
-        <v>-0.09644883378861112</v>
+        <v>1.245330620549339</v>
       </c>
     </row>
     <row r="177">
@@ -13865,28 +14216,28 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>TWINSICK TAO</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D177" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E177" s="8" t="n">
-        <v>46271</v>
+        <v>46289</v>
       </c>
       <c r="G177" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H177" s="9" t="n">
-        <v>20</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I177" s="9" t="n">
-        <v>27.05</v>
+        <v>121.72</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -13899,16 +14250,16 @@
         </is>
       </c>
       <c r="L177" s="9" t="n">
-        <v>108.2</v>
+        <v>121.72</v>
       </c>
       <c r="M177" s="9" t="n">
-        <v>108.2</v>
+        <v>121.72</v>
       </c>
       <c r="N177" s="9" t="n">
-        <v>28.2</v>
+        <v>67.10888888888888</v>
       </c>
       <c r="O177" s="7" t="n">
-        <v>0.3525</v>
+        <v>1.228850457782299</v>
       </c>
     </row>
     <row r="178">
@@ -13917,32 +14268,32 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Levity / Tape b K Bridge</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>K bridge</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D178" s="8" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="E178" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G178" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H178" s="9" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="I178" s="9" t="n">
-        <v>90</v>
+        <v>87.5</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -13951,16 +14302,16 @@
         </is>
       </c>
       <c r="L178" s="9" t="n">
-        <v>1080</v>
+        <v>350</v>
       </c>
       <c r="M178" s="9" t="n">
-        <v>1080</v>
+        <v>350</v>
       </c>
       <c r="N178" s="9" t="n">
-        <v>-60</v>
+        <v>-130</v>
       </c>
       <c r="O178" s="7" t="n">
-        <v>-0.05263157894736842</v>
+        <v>-0.2708333333333333</v>
       </c>
     </row>
     <row r="179">
@@ -13969,28 +14320,28 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Parcels ACL</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Stubb's Waller Creek Amphitheater</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D179" s="8" t="n">
-        <v>46298</v>
+        <v>46270</v>
       </c>
       <c r="E179" s="8" t="n">
         <v>46271</v>
       </c>
       <c r="G179" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H179" s="9" t="n">
-        <v>65.2</v>
+        <v>120</v>
       </c>
       <c r="I179" s="9" t="n">
-        <v>54.1</v>
+        <v>92.41500000000001</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
@@ -14003,16 +14354,16 @@
         </is>
       </c>
       <c r="L179" s="9" t="n">
-        <v>54.1</v>
+        <v>369.66</v>
       </c>
       <c r="M179" s="9" t="n">
-        <v>54.1</v>
+        <v>369.66</v>
       </c>
       <c r="N179" s="9" t="n">
-        <v>-11.1</v>
+        <v>-110.34</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>-0.1702453987730062</v>
+        <v>-0.2298749999999999</v>
       </c>
     </row>
     <row r="180">
@@ -14021,28 +14372,28 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Levity Tape B NYC afters</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Brooklyn Steel</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D180" s="8" t="n">
-        <v>46256</v>
+        <v>46242</v>
       </c>
       <c r="E180" s="8" t="n">
-        <v>46258</v>
+        <v>46242</v>
       </c>
       <c r="G180" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H180" s="9" t="n">
-        <v>62.37</v>
+        <v>47.59</v>
       </c>
       <c r="I180" s="9" t="n">
-        <v>44.25</v>
+        <v>52</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
@@ -14055,16 +14406,16 @@
         </is>
       </c>
       <c r="L180" s="9" t="n">
-        <v>177</v>
+        <v>52</v>
       </c>
       <c r="M180" s="9" t="n">
-        <v>177</v>
+        <v>52</v>
       </c>
       <c r="N180" s="9" t="n">
-        <v>-72.47999999999999</v>
+        <v>4.409999999999997</v>
       </c>
       <c r="O180" s="7" t="n">
-        <v>-0.2905242905242905</v>
+        <v>0.09266652658121446</v>
       </c>
     </row>
     <row r="181">
@@ -14073,32 +14424,32 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Arc Friday Pass 2026</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D181" s="8" t="n">
-        <v>46269</v>
+        <v>46242</v>
       </c>
       <c r="E181" s="8" t="n">
-        <v>46271</v>
+        <v>46242</v>
       </c>
       <c r="G181" t="n">
         <v>1</v>
       </c>
       <c r="H181" s="9" t="n">
-        <v>219</v>
+        <v>47.59</v>
       </c>
       <c r="I181" s="9" t="n">
-        <v>162.28</v>
+        <v>55</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -14107,16 +14458,16 @@
         </is>
       </c>
       <c r="L181" s="9" t="n">
-        <v>162.28</v>
+        <v>55</v>
       </c>
       <c r="M181" s="9" t="n">
-        <v>162.28</v>
+        <v>55</v>
       </c>
       <c r="N181" s="9" t="n">
-        <v>-56.72</v>
+        <v>7.409999999999997</v>
       </c>
       <c r="O181" s="7" t="n">
-        <v>-0.2589954337899543</v>
+        <v>0.155704980037823</v>
       </c>
     </row>
     <row r="182">
@@ -14125,32 +14476,32 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Chris stussy Arc Afters</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D182" s="8" t="n">
-        <v>46269</v>
+        <v>46242</v>
       </c>
       <c r="E182" s="8" t="n">
-        <v>46271</v>
+        <v>46242</v>
       </c>
       <c r="G182" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H182" s="9" t="n">
-        <v>100.24</v>
+        <v>47.59</v>
       </c>
       <c r="I182" s="9" t="n">
-        <v>117.21</v>
+        <v>43</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -14159,16 +14510,16 @@
         </is>
       </c>
       <c r="L182" s="9" t="n">
-        <v>117.21</v>
+        <v>86</v>
       </c>
       <c r="M182" s="9" t="n">
-        <v>117.21</v>
+        <v>86</v>
       </c>
       <c r="N182" s="9" t="n">
-        <v>16.97</v>
+        <v>-9.180000000000007</v>
       </c>
       <c r="O182" s="7" t="n">
-        <v>0.169293695131684</v>
+        <v>-0.09644883378861112</v>
       </c>
     </row>
     <row r="183">
@@ -14177,16 +14528,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Max dean ARC afters</t>
+          <t>TWINSICK TAO</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Concord Music Hall</t>
+          <t>Tao</t>
         </is>
       </c>
       <c r="D183" s="8" t="n">
-        <v>46269</v>
+        <v>46270</v>
       </c>
       <c r="E183" s="8" t="n">
         <v>46271</v>
@@ -14195,10 +14546,10 @@
         <v>4</v>
       </c>
       <c r="H183" s="9" t="n">
-        <v>42.18</v>
+        <v>20</v>
       </c>
       <c r="I183" s="9" t="n">
-        <v>63.1125</v>
+        <v>27.05</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -14211,16 +14562,16 @@
         </is>
       </c>
       <c r="L183" s="9" t="n">
-        <v>252.45</v>
+        <v>108.2</v>
       </c>
       <c r="M183" s="9" t="n">
-        <v>252.45</v>
+        <v>108.2</v>
       </c>
       <c r="N183" s="9" t="n">
-        <v>83.72999999999999</v>
+        <v>28.2</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>0.4962660028449501</v>
+        <v>0.3525</v>
       </c>
     </row>
     <row r="184">
@@ -14229,12 +14580,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Bowl</t>
+          <t>Levity / Tape b K Bridge</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>K bridge</t>
         </is>
       </c>
       <c r="D184" s="8" t="n">
@@ -14244,17 +14595,17 @@
         <v>46258</v>
       </c>
       <c r="G184" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H184" s="9" t="n">
-        <v>110</v>
+        <v>95</v>
       </c>
       <c r="I184" s="9" t="n">
-        <v>243.43</v>
+        <v>90</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -14263,16 +14614,16 @@
         </is>
       </c>
       <c r="L184" s="9" t="n">
-        <v>486.86</v>
+        <v>1080</v>
       </c>
       <c r="M184" s="9" t="n">
-        <v>486.86</v>
+        <v>1080</v>
       </c>
       <c r="N184" s="9" t="n">
-        <v>266.86</v>
+        <v>-60</v>
       </c>
       <c r="O184" s="7" t="n">
-        <v>1.213</v>
+        <v>-0.05263157894736842</v>
       </c>
     </row>
     <row r="185">
@@ -14281,32 +14632,32 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Goose RR</t>
+          <t>Parcels ACL</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Stubb's Waller Creek Amphitheater</t>
         </is>
       </c>
       <c r="D185" s="8" t="n">
-        <v>46266</v>
+        <v>46298</v>
       </c>
       <c r="E185" s="8" t="n">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="G185" t="n">
         <v>1</v>
       </c>
       <c r="H185" s="9" t="n">
-        <v>45</v>
+        <v>65.2</v>
       </c>
       <c r="I185" s="9" t="n">
-        <v>0</v>
+        <v>54.1</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -14315,16 +14666,16 @@
         </is>
       </c>
       <c r="L185" s="9" t="n">
-        <v>0</v>
+        <v>54.1</v>
       </c>
       <c r="M185" s="9" t="n">
-        <v>0</v>
+        <v>54.1</v>
       </c>
       <c r="N185" s="9" t="n">
-        <v>-45</v>
+        <v>-11.1</v>
       </c>
       <c r="O185" s="7" t="n">
-        <v>-1</v>
+        <v>-0.1702453987730062</v>
       </c>
     </row>
     <row r="186">
@@ -14333,32 +14684,32 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Levity Tape B NYC afters</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Brooklyn Steel</t>
         </is>
       </c>
       <c r="D186" s="8" t="n">
-        <v>46263</v>
+        <v>46256</v>
       </c>
       <c r="E186" s="8" t="n">
-        <v>46263</v>
+        <v>46258</v>
       </c>
       <c r="G186" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H186" s="9" t="n">
-        <v>151.76</v>
+        <v>62.37</v>
       </c>
       <c r="I186" s="9" t="n">
-        <v>223.51</v>
+        <v>44.25</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -14367,16 +14718,16 @@
         </is>
       </c>
       <c r="L186" s="9" t="n">
-        <v>223.51</v>
+        <v>177</v>
       </c>
       <c r="M186" s="9" t="n">
-        <v>223.51</v>
+        <v>177</v>
       </c>
       <c r="N186" s="9" t="n">
-        <v>71.75</v>
+        <v>-72.47999999999999</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>0.4727859778597786</v>
+        <v>-0.2905242905242905</v>
       </c>
     </row>
     <row r="187">
@@ -14385,32 +14736,32 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Arc Friday Pass 2026</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Arc</t>
         </is>
       </c>
       <c r="D187" s="8" t="n">
-        <v>46263</v>
+        <v>46269</v>
       </c>
       <c r="E187" s="8" t="n">
-        <v>46263</v>
+        <v>46271</v>
       </c>
       <c r="G187" t="n">
         <v>1</v>
       </c>
       <c r="H187" s="9" t="n">
-        <v>151.76</v>
+        <v>219</v>
       </c>
       <c r="I187" s="9" t="n">
-        <v>230</v>
+        <v>162.28</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -14419,16 +14770,16 @@
         </is>
       </c>
       <c r="L187" s="9" t="n">
-        <v>230</v>
+        <v>162.28</v>
       </c>
       <c r="M187" s="9" t="n">
-        <v>230</v>
+        <v>162.28</v>
       </c>
       <c r="N187" s="9" t="n">
-        <v>78.24000000000001</v>
+        <v>-56.72</v>
       </c>
       <c r="O187" s="7" t="n">
-        <v>0.5155508697944123</v>
+        <v>-0.2589954337899543</v>
       </c>
     </row>
     <row r="188">
@@ -14437,12 +14788,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>jamie xx NY</t>
+          <t>Chris stussy Arc Afters</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Public Records</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="D188" s="8" t="n">
@@ -14455,14 +14806,14 @@
         <v>1</v>
       </c>
       <c r="H188" s="9" t="n">
-        <v>49.44</v>
+        <v>100.24</v>
       </c>
       <c r="I188" s="9" t="n">
-        <v>0</v>
+        <v>117.21</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K188" t="inlineStr">
@@ -14471,16 +14822,16 @@
         </is>
       </c>
       <c r="L188" s="9" t="n">
-        <v>0</v>
+        <v>117.21</v>
       </c>
       <c r="M188" s="9" t="n">
-        <v>0</v>
+        <v>117.21</v>
       </c>
       <c r="N188" s="9" t="n">
-        <v>-49.44</v>
+        <v>16.97</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>-1</v>
+        <v>0.169293695131684</v>
       </c>
     </row>
     <row r="189">
@@ -14489,28 +14840,28 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Prospa Wednesday LA</t>
+          <t>Max dean ARC afters</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Shrine</t>
+          <t>Concord Music Hall</t>
         </is>
       </c>
       <c r="D189" s="8" t="n">
-        <v>46309</v>
+        <v>46269</v>
       </c>
       <c r="E189" s="8" t="n">
-        <v>46288</v>
+        <v>46271</v>
       </c>
       <c r="G189" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H189" s="9" t="n">
-        <v>59.98999999999999</v>
+        <v>42.18</v>
       </c>
       <c r="I189" s="9" t="n">
-        <v>85.59999999999999</v>
+        <v>63.1125</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -14523,16 +14874,16 @@
         </is>
       </c>
       <c r="L189" s="9" t="n">
-        <v>428</v>
+        <v>252.45</v>
       </c>
       <c r="M189" s="9" t="n">
-        <v>428</v>
+        <v>252.45</v>
       </c>
       <c r="N189" s="9" t="n">
-        <v>128.05</v>
+        <v>83.72999999999999</v>
       </c>
       <c r="O189" s="7" t="n">
-        <v>0.4269044840806802</v>
+        <v>0.4962660028449501</v>
       </c>
     </row>
     <row r="190">
@@ -14541,32 +14892,32 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Adriatique B2B Cloonee</t>
+          <t>Rufus Du Sol Boulder Bowl</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="D190" s="8" t="n">
-        <v>46361</v>
+        <v>46256</v>
       </c>
       <c r="E190" s="8" t="n">
-        <v>46276</v>
+        <v>46258</v>
       </c>
       <c r="G190" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H190" s="9" t="n">
-        <v>103.05</v>
+        <v>110</v>
       </c>
       <c r="I190" s="9" t="n">
-        <v>103.05</v>
+        <v>243.43</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K190" t="inlineStr">
@@ -14575,16 +14926,16 @@
         </is>
       </c>
       <c r="L190" s="9" t="n">
-        <v>412.2</v>
+        <v>486.86</v>
       </c>
       <c r="M190" s="9" t="n">
-        <v>412.2</v>
+        <v>486.86</v>
       </c>
       <c r="N190" s="9" t="n">
-        <v>0</v>
+        <v>266.86</v>
       </c>
       <c r="O190" s="7" t="n">
-        <v>0</v>
+        <v>1.213</v>
       </c>
     </row>
     <row r="191">
@@ -14593,32 +14944,32 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Ben Sterling Afters Sound</t>
+          <t>Goose RR</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="D191" s="8" t="n">
-        <v>46277</v>
+        <v>46266</v>
       </c>
       <c r="E191" s="8" t="n">
-        <v>46279</v>
+        <v>46267</v>
       </c>
       <c r="G191" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H191" s="9" t="n">
-        <v>47.59</v>
+        <v>45</v>
       </c>
       <c r="I191" s="9" t="n">
-        <v>75.5</v>
+        <v>0</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -14627,16 +14978,16 @@
         </is>
       </c>
       <c r="L191" s="9" t="n">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="M191" s="9" t="n">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="N191" s="9" t="n">
-        <v>111.64</v>
+        <v>-45</v>
       </c>
       <c r="O191" s="7" t="n">
-        <v>0.586467745324648</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="192">
@@ -14645,32 +14996,32 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D192" s="8" t="n">
-        <v>46285</v>
+        <v>46263</v>
       </c>
       <c r="E192" s="8" t="n">
-        <v>46288</v>
+        <v>46263</v>
       </c>
       <c r="G192" t="n">
         <v>1</v>
       </c>
       <c r="H192" s="9" t="n">
-        <v>188</v>
+        <v>151.76</v>
       </c>
       <c r="I192" s="9" t="n">
-        <v>218</v>
+        <v>223.51</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -14679,16 +15030,16 @@
         </is>
       </c>
       <c r="L192" s="9" t="n">
-        <v>218</v>
+        <v>223.51</v>
       </c>
       <c r="M192" s="9" t="n">
-        <v>218</v>
+        <v>223.51</v>
       </c>
       <c r="N192" s="9" t="n">
-        <v>30</v>
+        <v>71.75</v>
       </c>
       <c r="O192" s="7" t="n">
-        <v>0.1595744680851064</v>
+        <v>0.4727859778597786</v>
       </c>
     </row>
     <row r="193">
@@ -14697,32 +15048,32 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D193" s="8" t="n">
-        <v>46285</v>
+        <v>46263</v>
       </c>
       <c r="E193" s="8" t="n">
-        <v>46288</v>
+        <v>46263</v>
       </c>
       <c r="G193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H193" s="9" t="n">
-        <v>188</v>
+        <v>151.76</v>
       </c>
       <c r="I193" s="9" t="n">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -14731,16 +15082,16 @@
         </is>
       </c>
       <c r="L193" s="9" t="n">
-        <v>418</v>
+        <v>230</v>
       </c>
       <c r="M193" s="9" t="n">
-        <v>418</v>
+        <v>230</v>
       </c>
       <c r="N193" s="9" t="n">
-        <v>42</v>
+        <v>78.24000000000001</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>0.1117021276595745</v>
+        <v>0.5155508697944123</v>
       </c>
     </row>
     <row r="194">
@@ -14749,32 +15100,32 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>jamie xx NY</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Public Records</t>
         </is>
       </c>
       <c r="D194" s="8" t="n">
-        <v>46285</v>
+        <v>46269</v>
       </c>
       <c r="E194" s="8" t="n">
-        <v>46288</v>
+        <v>46271</v>
       </c>
       <c r="G194" t="n">
         <v>1</v>
       </c>
       <c r="H194" s="9" t="n">
-        <v>188</v>
+        <v>49.44</v>
       </c>
       <c r="I194" s="9" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -14783,16 +15134,16 @@
         </is>
       </c>
       <c r="L194" s="9" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="M194" s="9" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="N194" s="9" t="n">
-        <v>2</v>
+        <v>-49.44</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="195">
@@ -14801,32 +15152,32 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="D195" s="8" t="n">
-        <v>46285</v>
+        <v>46309</v>
       </c>
       <c r="E195" s="8" t="n">
         <v>46288</v>
       </c>
       <c r="G195" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H195" s="9" t="n">
-        <v>188</v>
+        <v>59.98999999999999</v>
       </c>
       <c r="I195" s="9" t="n">
-        <v>190</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -14835,16 +15186,16 @@
         </is>
       </c>
       <c r="L195" s="9" t="n">
-        <v>380</v>
+        <v>428</v>
       </c>
       <c r="M195" s="9" t="n">
-        <v>380</v>
+        <v>428</v>
       </c>
       <c r="N195" s="9" t="n">
-        <v>4</v>
+        <v>128.05</v>
       </c>
       <c r="O195" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>0.4269044840806802</v>
       </c>
     </row>
     <row r="196">
@@ -14853,32 +15204,32 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+          <t>Adriatique B2B Cloonee</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Watson Island Park</t>
         </is>
       </c>
       <c r="D196" s="8" t="n">
-        <v>46285</v>
+        <v>46361</v>
       </c>
       <c r="E196" s="8" t="n">
-        <v>46288</v>
+        <v>46276</v>
       </c>
       <c r="G196" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H196" s="9" t="n">
-        <v>326</v>
+        <v>103.05</v>
       </c>
       <c r="I196" s="9" t="n">
-        <v>293.92</v>
+        <v>103.05</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -14887,16 +15238,16 @@
         </is>
       </c>
       <c r="L196" s="9" t="n">
-        <v>587.84</v>
+        <v>412.2</v>
       </c>
       <c r="M196" s="9" t="n">
-        <v>587.84</v>
+        <v>412.2</v>
       </c>
       <c r="N196" s="9" t="n">
-        <v>-64.15999999999997</v>
+        <v>0</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>-0.09840490797546007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="197">
@@ -14905,49 +15256,361 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
+          <t>Ben Sterling Afters Sound</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Sound</t>
+        </is>
+      </c>
+      <c r="D197" s="8" t="n">
+        <v>46277</v>
+      </c>
+      <c r="E197" s="8" t="n">
+        <v>46279</v>
+      </c>
+      <c r="G197" t="n">
+        <v>4</v>
+      </c>
+      <c r="H197" s="9" t="n">
+        <v>47.59</v>
+      </c>
+      <c r="I197" s="9" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L197" s="9" t="n">
+        <v>302</v>
+      </c>
+      <c r="M197" s="9" t="n">
+        <v>302</v>
+      </c>
+      <c r="N197" s="9" t="n">
+        <v>111.64</v>
+      </c>
+      <c r="O197" s="7" t="n">
+        <v>0.586467745324648</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D198" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E198" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G198" t="n">
+        <v>1</v>
+      </c>
+      <c r="H198" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I198" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L198" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="M198" s="9" t="n">
+        <v>218</v>
+      </c>
+      <c r="N198" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="O198" s="7" t="n">
+        <v>0.1595744680851064</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D199" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E199" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G199" t="n">
+        <v>2</v>
+      </c>
+      <c r="H199" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I199" s="9" t="n">
+        <v>209</v>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L199" s="9" t="n">
+        <v>418</v>
+      </c>
+      <c r="M199" s="9" t="n">
+        <v>418</v>
+      </c>
+      <c r="N199" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="O199" s="7" t="n">
+        <v>0.1117021276595745</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D200" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E200" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G200" t="n">
+        <v>1</v>
+      </c>
+      <c r="H200" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I200" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L200" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="M200" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="N200" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="O200" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D201" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E201" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G201" t="n">
+        <v>2</v>
+      </c>
+      <c r="H201" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I201" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L201" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="M201" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="N201" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O201" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
           <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C202" t="inlineStr">
         <is>
           <t>Pacha</t>
         </is>
       </c>
-      <c r="D197" s="8" t="n">
+      <c r="D202" s="8" t="n">
         <v>46285</v>
       </c>
-      <c r="E197" s="8" t="n">
+      <c r="E202" s="8" t="n">
         <v>46288</v>
       </c>
-      <c r="G197" t="n">
+      <c r="G202" t="n">
+        <v>2</v>
+      </c>
+      <c r="H202" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="I202" s="9" t="n">
+        <v>293.92</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L202" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="M202" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="N202" s="9" t="n">
+        <v>-64.15999999999997</v>
+      </c>
+      <c r="O202" s="7" t="n">
+        <v>-0.09840490797546007</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D203" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E203" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G203" t="n">
         <v>1</v>
       </c>
-      <c r="H197" s="9" t="n">
+      <c r="H203" s="9" t="n">
         <v>326</v>
       </c>
-      <c r="I197" s="9" t="n">
+      <c r="I203" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="J197" t="inlineStr">
+      <c r="J203" t="inlineStr">
         <is>
           <t>CrowdVolt</t>
         </is>
       </c>
-      <c r="K197" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L197" s="9" t="n">
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L203" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="M197" s="9" t="n">
+      <c r="M203" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="N197" s="9" t="n">
+      <c r="N203" s="9" t="n">
         <v>-73</v>
       </c>
-      <c r="O197" s="7" t="n">
+      <c r="O203" s="7" t="n">
         <v>-0.2239263803680982</v>
       </c>
     </row>
@@ -14962,7 +15625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15185,263 +15848,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>46290</v>
+          <t>buy</t>
+        </is>
       </c>
       <c r="E6" s="8" t="n">
-        <v>46289.75697916667</v>
-      </c>
-      <c r="F6" t="n">
+        <v>46290.59245370371</v>
+      </c>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J6" t="b">
         <v>1</v>
       </c>
-      <c r="G6" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>132.3</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>46289</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>133.28</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>133.28</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>46289.81953703704</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>136.22</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>136.22</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>46289.82378472222</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>46289</v>
-      </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>46289.84034722222</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="H11" s="9" t="n">
-        <v>139.16</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>46290.59245370371</v>
-      </c>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>AXS</t>
-        </is>
-      </c>
-      <c r="J12" t="b">
-        <v>1</v>
-      </c>
-      <c r="K12" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>quantity not stated and event details missing</t>
         </is>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-25 (5 new transactions, 7 skipped, 202 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15625,7 +15625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15870,6 +15870,206 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46290.50342592593</v>
+      </c>
+      <c r="F7" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H7" s="9" t="n">
+        <v>378.96</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46290.50458333334</v>
+      </c>
+      <c r="F8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>378.96</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46290.50798611111</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="H9" s="9" t="n">
+        <v>640.38</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46290.51108796296</v>
+      </c>
+      <c r="F10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>416.34</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>See Tickets</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46290.76260416667</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>166.6</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>333.2</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sync workbook into DB (Prospa +2, Four Tet price fix)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -3373,7 +3373,7 @@
         <v>983</v>
       </c>
       <c r="J97" s="8" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="98">
@@ -4414,7 +4414,7 @@
         <v>719.88</v>
       </c>
       <c r="J134" s="8" t="n">
-        <v>46288</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="135">
@@ -5014,13 +5014,13 @@
         </is>
       </c>
       <c r="G156" s="9" t="n">
-        <v>41.4</v>
+        <v>52.43</v>
       </c>
       <c r="H156" t="n">
         <v>1</v>
       </c>
       <c r="I156" s="9" t="n">
-        <v>41.4</v>
+        <v>52.43</v>
       </c>
     </row>
   </sheetData>
@@ -5034,7 +5034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O203"/>
+  <dimension ref="A1:O205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14268,32 +14268,32 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D178" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E178" s="8" t="n">
-        <v>46271</v>
+        <v>46290</v>
       </c>
       <c r="G178" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H178" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I178" s="9" t="n">
-        <v>87.5</v>
+        <v>153.27</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K178" t="inlineStr">
@@ -14302,16 +14302,16 @@
         </is>
       </c>
       <c r="L178" s="9" t="n">
-        <v>350</v>
+        <v>306.54</v>
       </c>
       <c r="M178" s="9" t="n">
-        <v>350</v>
+        <v>306.54</v>
       </c>
       <c r="N178" s="9" t="n">
-        <v>-130</v>
+        <v>197.3177777777778</v>
       </c>
       <c r="O178" s="7" t="n">
-        <v>-0.2708333333333333</v>
+        <v>1.806571719226857</v>
       </c>
     </row>
     <row r="179">
@@ -14341,11 +14341,11 @@
         <v>120</v>
       </c>
       <c r="I179" s="9" t="n">
-        <v>92.41500000000001</v>
+        <v>87.5</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -14354,16 +14354,16 @@
         </is>
       </c>
       <c r="L179" s="9" t="n">
-        <v>369.66</v>
+        <v>350</v>
       </c>
       <c r="M179" s="9" t="n">
-        <v>369.66</v>
+        <v>350</v>
       </c>
       <c r="N179" s="9" t="n">
-        <v>-110.34</v>
+        <v>-130</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>-0.2298749999999999</v>
+        <v>-0.2708333333333333</v>
       </c>
     </row>
     <row r="180">
@@ -14372,32 +14372,32 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D180" s="8" t="n">
-        <v>46242</v>
+        <v>46270</v>
       </c>
       <c r="E180" s="8" t="n">
-        <v>46242</v>
+        <v>46271</v>
       </c>
       <c r="G180" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H180" s="9" t="n">
-        <v>47.59</v>
+        <v>120</v>
       </c>
       <c r="I180" s="9" t="n">
-        <v>52</v>
+        <v>92.41500000000001</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -14406,16 +14406,16 @@
         </is>
       </c>
       <c r="L180" s="9" t="n">
-        <v>52</v>
+        <v>369.66</v>
       </c>
       <c r="M180" s="9" t="n">
-        <v>52</v>
+        <v>369.66</v>
       </c>
       <c r="N180" s="9" t="n">
-        <v>4.409999999999997</v>
+        <v>-110.34</v>
       </c>
       <c r="O180" s="7" t="n">
-        <v>0.09266652658121446</v>
+        <v>-0.2298749999999999</v>
       </c>
     </row>
     <row r="181">
@@ -14445,11 +14445,11 @@
         <v>47.59</v>
       </c>
       <c r="I181" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K181" t="inlineStr">
@@ -14458,16 +14458,16 @@
         </is>
       </c>
       <c r="L181" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M181" s="9" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="N181" s="9" t="n">
-        <v>7.409999999999997</v>
+        <v>4.409999999999997</v>
       </c>
       <c r="O181" s="7" t="n">
-        <v>0.155704980037823</v>
+        <v>0.09266652658121446</v>
       </c>
     </row>
     <row r="182">
@@ -14491,17 +14491,17 @@
         <v>46242</v>
       </c>
       <c r="G182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H182" s="9" t="n">
         <v>47.59</v>
       </c>
       <c r="I182" s="9" t="n">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -14510,16 +14510,16 @@
         </is>
       </c>
       <c r="L182" s="9" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="M182" s="9" t="n">
-        <v>86</v>
+        <v>55</v>
       </c>
       <c r="N182" s="9" t="n">
-        <v>-9.180000000000007</v>
+        <v>7.409999999999997</v>
       </c>
       <c r="O182" s="7" t="n">
-        <v>-0.09644883378861112</v>
+        <v>0.155704980037823</v>
       </c>
     </row>
     <row r="183">
@@ -14528,32 +14528,32 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>TWINSICK TAO</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D183" s="8" t="n">
-        <v>46270</v>
+        <v>46242</v>
       </c>
       <c r="E183" s="8" t="n">
-        <v>46271</v>
+        <v>46242</v>
       </c>
       <c r="G183" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H183" s="9" t="n">
-        <v>20</v>
+        <v>47.59</v>
       </c>
       <c r="I183" s="9" t="n">
-        <v>27.05</v>
+        <v>43</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K183" t="inlineStr">
@@ -14562,16 +14562,16 @@
         </is>
       </c>
       <c r="L183" s="9" t="n">
-        <v>108.2</v>
+        <v>86</v>
       </c>
       <c r="M183" s="9" t="n">
-        <v>108.2</v>
+        <v>86</v>
       </c>
       <c r="N183" s="9" t="n">
-        <v>28.2</v>
+        <v>-9.180000000000007</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>0.3525</v>
+        <v>-0.09644883378861112</v>
       </c>
     </row>
     <row r="184">
@@ -14580,32 +14580,32 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Levity / Tape b K Bridge</t>
+          <t>TWINSICK TAO</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>K bridge</t>
+          <t>Tao</t>
         </is>
       </c>
       <c r="D184" s="8" t="n">
-        <v>46256</v>
+        <v>46270</v>
       </c>
       <c r="E184" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G184" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H184" s="9" t="n">
-        <v>95</v>
+        <v>20</v>
       </c>
       <c r="I184" s="9" t="n">
-        <v>90</v>
+        <v>27.05</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -14614,16 +14614,16 @@
         </is>
       </c>
       <c r="L184" s="9" t="n">
-        <v>1080</v>
+        <v>108.2</v>
       </c>
       <c r="M184" s="9" t="n">
-        <v>1080</v>
+        <v>108.2</v>
       </c>
       <c r="N184" s="9" t="n">
-        <v>-60</v>
+        <v>28.2</v>
       </c>
       <c r="O184" s="7" t="n">
-        <v>-0.05263157894736842</v>
+        <v>0.3525</v>
       </c>
     </row>
     <row r="185">
@@ -14632,32 +14632,32 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Parcels ACL</t>
+          <t>Levity / Tape b K Bridge</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Stubb's Waller Creek Amphitheater</t>
+          <t>K bridge</t>
         </is>
       </c>
       <c r="D185" s="8" t="n">
-        <v>46298</v>
+        <v>46256</v>
       </c>
       <c r="E185" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
       <c r="G185" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H185" s="9" t="n">
-        <v>65.2</v>
+        <v>95</v>
       </c>
       <c r="I185" s="9" t="n">
-        <v>54.1</v>
+        <v>90</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -14666,16 +14666,16 @@
         </is>
       </c>
       <c r="L185" s="9" t="n">
-        <v>54.1</v>
+        <v>1080</v>
       </c>
       <c r="M185" s="9" t="n">
-        <v>54.1</v>
+        <v>1080</v>
       </c>
       <c r="N185" s="9" t="n">
-        <v>-11.1</v>
+        <v>-60</v>
       </c>
       <c r="O185" s="7" t="n">
-        <v>-0.1702453987730062</v>
+        <v>-0.05263157894736842</v>
       </c>
     </row>
     <row r="186">
@@ -14684,32 +14684,32 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Levity Tape B NYC afters</t>
+          <t>Parcels ACL</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Brooklyn Steel</t>
+          <t>Stubb's Waller Creek Amphitheater</t>
         </is>
       </c>
       <c r="D186" s="8" t="n">
-        <v>46256</v>
+        <v>46298</v>
       </c>
       <c r="E186" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G186" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H186" s="9" t="n">
-        <v>62.37</v>
+        <v>65.2</v>
       </c>
       <c r="I186" s="9" t="n">
-        <v>44.25</v>
+        <v>54.1</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -14718,16 +14718,16 @@
         </is>
       </c>
       <c r="L186" s="9" t="n">
-        <v>177</v>
+        <v>54.1</v>
       </c>
       <c r="M186" s="9" t="n">
-        <v>177</v>
+        <v>54.1</v>
       </c>
       <c r="N186" s="9" t="n">
-        <v>-72.47999999999999</v>
+        <v>-11.1</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>-0.2905242905242905</v>
+        <v>-0.1702453987730062</v>
       </c>
     </row>
     <row r="187">
@@ -14736,32 +14736,32 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Arc Friday Pass 2026</t>
+          <t>Levity Tape B NYC afters</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Brooklyn Steel</t>
         </is>
       </c>
       <c r="D187" s="8" t="n">
-        <v>46269</v>
+        <v>46256</v>
       </c>
       <c r="E187" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
       <c r="G187" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H187" s="9" t="n">
-        <v>219</v>
+        <v>62.37</v>
       </c>
       <c r="I187" s="9" t="n">
-        <v>162.28</v>
+        <v>44.25</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -14770,16 +14770,16 @@
         </is>
       </c>
       <c r="L187" s="9" t="n">
-        <v>162.28</v>
+        <v>177</v>
       </c>
       <c r="M187" s="9" t="n">
-        <v>162.28</v>
+        <v>177</v>
       </c>
       <c r="N187" s="9" t="n">
-        <v>-56.72</v>
+        <v>-72.47999999999999</v>
       </c>
       <c r="O187" s="7" t="n">
-        <v>-0.2589954337899543</v>
+        <v>-0.2905242905242905</v>
       </c>
     </row>
     <row r="188">
@@ -14788,12 +14788,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Chris stussy Arc Afters</t>
+          <t>Arc Friday Pass 2026</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Arc</t>
         </is>
       </c>
       <c r="D188" s="8" t="n">
@@ -14806,10 +14806,10 @@
         <v>1</v>
       </c>
       <c r="H188" s="9" t="n">
-        <v>100.24</v>
+        <v>219</v>
       </c>
       <c r="I188" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -14822,16 +14822,16 @@
         </is>
       </c>
       <c r="L188" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="M188" s="9" t="n">
-        <v>117.21</v>
+        <v>162.28</v>
       </c>
       <c r="N188" s="9" t="n">
-        <v>16.97</v>
+        <v>-56.72</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>0.169293695131684</v>
+        <v>-0.2589954337899543</v>
       </c>
     </row>
     <row r="189">
@@ -14840,12 +14840,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Max dean ARC afters</t>
+          <t>Chris stussy Arc Afters</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Concord Music Hall</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="D189" s="8" t="n">
@@ -14855,13 +14855,13 @@
         <v>46271</v>
       </c>
       <c r="G189" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H189" s="9" t="n">
-        <v>42.18</v>
+        <v>100.24</v>
       </c>
       <c r="I189" s="9" t="n">
-        <v>63.1125</v>
+        <v>117.21</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -14874,16 +14874,16 @@
         </is>
       </c>
       <c r="L189" s="9" t="n">
-        <v>252.45</v>
+        <v>117.21</v>
       </c>
       <c r="M189" s="9" t="n">
-        <v>252.45</v>
+        <v>117.21</v>
       </c>
       <c r="N189" s="9" t="n">
-        <v>83.72999999999999</v>
+        <v>16.97</v>
       </c>
       <c r="O189" s="7" t="n">
-        <v>0.4962660028449501</v>
+        <v>0.169293695131684</v>
       </c>
     </row>
     <row r="190">
@@ -14892,28 +14892,28 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Bowl</t>
+          <t>Max dean ARC afters</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>Concord Music Hall</t>
         </is>
       </c>
       <c r="D190" s="8" t="n">
-        <v>46256</v>
+        <v>46269</v>
       </c>
       <c r="E190" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G190" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H190" s="9" t="n">
-        <v>110</v>
+        <v>42.18</v>
       </c>
       <c r="I190" s="9" t="n">
-        <v>243.43</v>
+        <v>63.1125</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -14926,16 +14926,16 @@
         </is>
       </c>
       <c r="L190" s="9" t="n">
-        <v>486.86</v>
+        <v>252.45</v>
       </c>
       <c r="M190" s="9" t="n">
-        <v>486.86</v>
+        <v>252.45</v>
       </c>
       <c r="N190" s="9" t="n">
-        <v>266.86</v>
+        <v>83.72999999999999</v>
       </c>
       <c r="O190" s="7" t="n">
-        <v>1.213</v>
+        <v>0.4962660028449501</v>
       </c>
     </row>
     <row r="191">
@@ -14944,32 +14944,32 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Goose RR</t>
+          <t>Rufus Du Sol Boulder Bowl</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="D191" s="8" t="n">
-        <v>46266</v>
+        <v>46256</v>
       </c>
       <c r="E191" s="8" t="n">
-        <v>46267</v>
+        <v>46258</v>
       </c>
       <c r="G191" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H191" s="9" t="n">
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="I191" s="9" t="n">
-        <v>0</v>
+        <v>243.43</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K191" t="inlineStr">
@@ -14978,16 +14978,16 @@
         </is>
       </c>
       <c r="L191" s="9" t="n">
-        <v>0</v>
+        <v>486.86</v>
       </c>
       <c r="M191" s="9" t="n">
-        <v>0</v>
+        <v>486.86</v>
       </c>
       <c r="N191" s="9" t="n">
-        <v>-45</v>
+        <v>266.86</v>
       </c>
       <c r="O191" s="7" t="n">
-        <v>-1</v>
+        <v>1.213</v>
       </c>
     </row>
     <row r="192">
@@ -14996,32 +14996,32 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Goose RR</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="D192" s="8" t="n">
-        <v>46263</v>
+        <v>46266</v>
       </c>
       <c r="E192" s="8" t="n">
-        <v>46263</v>
+        <v>46267</v>
       </c>
       <c r="G192" t="n">
         <v>1</v>
       </c>
       <c r="H192" s="9" t="n">
-        <v>151.76</v>
+        <v>45</v>
       </c>
       <c r="I192" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -15030,16 +15030,16 @@
         </is>
       </c>
       <c r="L192" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="M192" s="9" t="n">
-        <v>223.51</v>
+        <v>0</v>
       </c>
       <c r="N192" s="9" t="n">
-        <v>71.75</v>
+        <v>-45</v>
       </c>
       <c r="O192" s="7" t="n">
-        <v>0.4727859778597786</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="193">
@@ -15069,7 +15069,7 @@
         <v>151.76</v>
       </c>
       <c r="I193" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -15082,16 +15082,16 @@
         </is>
       </c>
       <c r="L193" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="M193" s="9" t="n">
-        <v>230</v>
+        <v>223.51</v>
       </c>
       <c r="N193" s="9" t="n">
-        <v>78.24000000000001</v>
+        <v>71.75</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>0.5155508697944123</v>
+        <v>0.4727859778597786</v>
       </c>
     </row>
     <row r="194">
@@ -15100,32 +15100,32 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>jamie xx NY</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Public Records</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D194" s="8" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="E194" s="8" t="n">
-        <v>46271</v>
+        <v>46263</v>
       </c>
       <c r="G194" t="n">
         <v>1</v>
       </c>
       <c r="H194" s="9" t="n">
-        <v>49.44</v>
+        <v>151.76</v>
       </c>
       <c r="I194" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -15134,16 +15134,16 @@
         </is>
       </c>
       <c r="L194" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="M194" s="9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="N194" s="9" t="n">
-        <v>-49.44</v>
+        <v>78.24000000000001</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>-1</v>
+        <v>0.5155508697944123</v>
       </c>
     </row>
     <row r="195">
@@ -15152,32 +15152,32 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Prospa Wednesday LA</t>
+          <t>jamie xx NY</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Shrine</t>
+          <t>Public Records</t>
         </is>
       </c>
       <c r="D195" s="8" t="n">
-        <v>46309</v>
+        <v>46269</v>
       </c>
       <c r="E195" s="8" t="n">
-        <v>46288</v>
+        <v>46271</v>
       </c>
       <c r="G195" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H195" s="9" t="n">
-        <v>59.98999999999999</v>
+        <v>49.44</v>
       </c>
       <c r="I195" s="9" t="n">
-        <v>85.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -15186,16 +15186,16 @@
         </is>
       </c>
       <c r="L195" s="9" t="n">
-        <v>428</v>
+        <v>0</v>
       </c>
       <c r="M195" s="9" t="n">
-        <v>428</v>
+        <v>0</v>
       </c>
       <c r="N195" s="9" t="n">
-        <v>128.05</v>
+        <v>-49.44</v>
       </c>
       <c r="O195" s="7" t="n">
-        <v>0.4269044840806802</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="196">
@@ -15204,32 +15204,32 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Adriatique B2B Cloonee</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="D196" s="8" t="n">
-        <v>46361</v>
+        <v>46309</v>
       </c>
       <c r="E196" s="8" t="n">
-        <v>46276</v>
+        <v>46288</v>
       </c>
       <c r="G196" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H196" s="9" t="n">
-        <v>103.05</v>
+        <v>59.98999999999999</v>
       </c>
       <c r="I196" s="9" t="n">
-        <v>103.05</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -15238,16 +15238,16 @@
         </is>
       </c>
       <c r="L196" s="9" t="n">
-        <v>412.2</v>
+        <v>428</v>
       </c>
       <c r="M196" s="9" t="n">
-        <v>412.2</v>
+        <v>428</v>
       </c>
       <c r="N196" s="9" t="n">
-        <v>0</v>
+        <v>128.05</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>0</v>
+        <v>0.4269044840806802</v>
       </c>
     </row>
     <row r="197">
@@ -15256,32 +15256,32 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Ben Sterling Afters Sound</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="D197" s="8" t="n">
-        <v>46277</v>
+        <v>46309</v>
       </c>
       <c r="E197" s="8" t="n">
-        <v>46279</v>
+        <v>46290</v>
       </c>
       <c r="G197" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H197" s="9" t="n">
-        <v>47.59</v>
+        <v>59.99</v>
       </c>
       <c r="I197" s="9" t="n">
-        <v>75.5</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -15290,16 +15290,16 @@
         </is>
       </c>
       <c r="L197" s="9" t="n">
-        <v>302</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="M197" s="9" t="n">
-        <v>302</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="N197" s="9" t="n">
-        <v>111.64</v>
+        <v>25.66</v>
       </c>
       <c r="O197" s="7" t="n">
-        <v>0.586467745324648</v>
+        <v>0.4277379563260544</v>
       </c>
     </row>
     <row r="198">
@@ -15308,32 +15308,32 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Adriatique B2B Cloonee</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Watson Island Park</t>
         </is>
       </c>
       <c r="D198" s="8" t="n">
-        <v>46285</v>
+        <v>46361</v>
       </c>
       <c r="E198" s="8" t="n">
-        <v>46288</v>
+        <v>46276</v>
       </c>
       <c r="G198" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H198" s="9" t="n">
-        <v>188</v>
+        <v>103.05</v>
       </c>
       <c r="I198" s="9" t="n">
-        <v>218</v>
+        <v>103.05</v>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -15342,16 +15342,16 @@
         </is>
       </c>
       <c r="L198" s="9" t="n">
-        <v>218</v>
+        <v>412.2</v>
       </c>
       <c r="M198" s="9" t="n">
-        <v>218</v>
+        <v>412.2</v>
       </c>
       <c r="N198" s="9" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="O198" s="7" t="n">
-        <v>0.1595744680851064</v>
+        <v>0</v>
       </c>
     </row>
     <row r="199">
@@ -15360,28 +15360,28 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Ben Sterling Afters Sound</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D199" s="8" t="n">
-        <v>46285</v>
+        <v>46277</v>
       </c>
       <c r="E199" s="8" t="n">
-        <v>46288</v>
+        <v>46279</v>
       </c>
       <c r="G199" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H199" s="9" t="n">
-        <v>188</v>
+        <v>47.59</v>
       </c>
       <c r="I199" s="9" t="n">
-        <v>209</v>
+        <v>75.5</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -15394,16 +15394,16 @@
         </is>
       </c>
       <c r="L199" s="9" t="n">
-        <v>418</v>
+        <v>302</v>
       </c>
       <c r="M199" s="9" t="n">
-        <v>418</v>
+        <v>302</v>
       </c>
       <c r="N199" s="9" t="n">
-        <v>42</v>
+        <v>111.64</v>
       </c>
       <c r="O199" s="7" t="n">
-        <v>0.1117021276595745</v>
+        <v>0.586467745324648</v>
       </c>
     </row>
     <row r="200">
@@ -15433,7 +15433,7 @@
         <v>188</v>
       </c>
       <c r="I200" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
@@ -15446,16 +15446,16 @@
         </is>
       </c>
       <c r="L200" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="M200" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="N200" s="9" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="O200" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>0.1595744680851064</v>
       </c>
     </row>
     <row r="201">
@@ -15485,7 +15485,7 @@
         <v>188</v>
       </c>
       <c r="I201" s="9" t="n">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="J201" t="inlineStr">
         <is>
@@ -15498,16 +15498,16 @@
         </is>
       </c>
       <c r="L201" s="9" t="n">
-        <v>380</v>
+        <v>418</v>
       </c>
       <c r="M201" s="9" t="n">
-        <v>380</v>
+        <v>418</v>
       </c>
       <c r="N201" s="9" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="O201" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>0.1117021276595745</v>
       </c>
     </row>
     <row r="202">
@@ -15516,7 +15516,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -15531,35 +15531,35 @@
         <v>46288</v>
       </c>
       <c r="G202" t="n">
+        <v>1</v>
+      </c>
+      <c r="H202" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I202" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L202" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="M202" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="N202" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H202" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="I202" s="9" t="n">
-        <v>293.92</v>
-      </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="K202" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L202" s="9" t="n">
-        <v>587.84</v>
-      </c>
-      <c r="M202" s="9" t="n">
-        <v>587.84</v>
-      </c>
-      <c r="N202" s="9" t="n">
-        <v>-64.15999999999997</v>
-      </c>
       <c r="O202" s="7" t="n">
-        <v>-0.09840490797546007</v>
+        <v>0.01063829787234043</v>
       </c>
     </row>
     <row r="203">
@@ -15568,7 +15568,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -15583,34 +15583,138 @@
         <v>46288</v>
       </c>
       <c r="G203" t="n">
+        <v>2</v>
+      </c>
+      <c r="H203" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I203" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L203" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="M203" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="N203" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O203" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D204" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E204" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G204" t="n">
+        <v>2</v>
+      </c>
+      <c r="H204" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="I204" s="9" t="n">
+        <v>293.92</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L204" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="M204" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="N204" s="9" t="n">
+        <v>-64.15999999999997</v>
+      </c>
+      <c r="O204" s="7" t="n">
+        <v>-0.09840490797546007</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D205" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E205" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G205" t="n">
         <v>1</v>
       </c>
-      <c r="H203" s="9" t="n">
+      <c r="H205" s="9" t="n">
         <v>326</v>
       </c>
-      <c r="I203" s="9" t="n">
+      <c r="I205" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="J203" t="inlineStr">
+      <c r="J205" t="inlineStr">
         <is>
           <t>CrowdVolt</t>
         </is>
       </c>
-      <c r="K203" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L203" s="9" t="n">
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L205" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="M203" s="9" t="n">
+      <c r="M205" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="N203" s="9" t="n">
+      <c r="N205" s="9" t="n">
         <v>-73</v>
       </c>
-      <c r="O203" s="7" t="n">
+      <c r="O205" s="7" t="n">
         <v>-0.2239263803680982</v>
       </c>
     </row>
@@ -15625,7 +15729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15688,37 +15792,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Prospa</t>
+          <t>GRiZMAS 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Shrine Auditorium and Expo Hall</t>
+          <t>Masonic Temple Theatre</t>
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>46309</v>
+        <v>46374</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>46288</v>
+        <v>46289.59476851852</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>93.09999999999999</v>
+        <v>52.22</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>93.09999999999999</v>
+        <v>567.84</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J2" t="b">
@@ -15733,32 +15837,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GRiZMAS 2026</t>
+          <t>MGMT (DJ Set)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Masonic Temple Theatre</t>
+          <t>The Concourse Project</t>
         </is>
       </c>
       <c r="D3" s="8" t="n">
-        <v>46374</v>
+        <v>46312</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>46289.59476851852</v>
+        <v>46289.42085648148</v>
       </c>
       <c r="F3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>52.22</v>
+        <v>30</v>
       </c>
       <c r="H3" s="9" t="n">
-        <v>567.84</v>
+        <v>153.08</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>See Tickets</t>
         </is>
       </c>
       <c r="J3" t="b">
@@ -15785,7 +15889,7 @@
         <v>46312</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46289.42085648148</v>
+        <v>46289.42576388889</v>
       </c>
       <c r="F4" t="n">
         <v>4</v>
@@ -15811,38 +15915,23 @@
           <t>buy</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MGMT (DJ Set)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="n">
-        <v>46312</v>
-      </c>
       <c r="E5" s="8" t="n">
-        <v>46289.42576388889</v>
-      </c>
-      <c r="F5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="H5" s="9" t="n">
-        <v>153.08</v>
-      </c>
+        <v>46290.59245370371</v>
+      </c>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>See Tickets</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J5" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>quantity not stated and event details missing</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -15851,23 +15940,38 @@
           <t>buy</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46389</v>
+      </c>
       <c r="E6" s="8" t="n">
-        <v>46290.59245370371</v>
-      </c>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
+        <v>46290.50342592593</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>378.96</v>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>See Tickets</t>
         </is>
       </c>
       <c r="J6" t="b">
-        <v>1</v>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>quantity not stated and event details missing</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -15890,7 +15994,7 @@
         <v>46389</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>46290.50342592593</v>
+        <v>46290.50458333334</v>
       </c>
       <c r="F7" t="n">
         <v>6</v>
@@ -15930,16 +16034,16 @@
         <v>46389</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>46290.50458333334</v>
+        <v>46290.50798611111</v>
       </c>
       <c r="F8" t="n">
         <v>6</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>378.96</v>
+        <v>640.38</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -15970,16 +16074,16 @@
         <v>46389</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>46290.50798611111</v>
+        <v>46290.51108796296</v>
       </c>
       <c r="F9" t="n">
         <v>6</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="H9" s="9" t="n">
-        <v>640.38</v>
+        <v>416.34</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -15987,86 +16091,6 @@
         </is>
       </c>
       <c r="J9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Max Dean b2b Luke Dean</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>46389</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>46290.51108796296</v>
-      </c>
-      <c r="F10" t="n">
-        <v>6</v>
-      </c>
-      <c r="G10" s="9" t="n">
-        <v>55</v>
-      </c>
-      <c r="H10" s="9" t="n">
-        <v>416.34</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Prospa</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="E11" s="8" t="n">
-        <v>46290.76260416667</v>
-      </c>
-      <c r="F11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="9" t="n">
-        <v>166.6</v>
-      </c>
-      <c r="H11" s="9" t="n">
-        <v>333.2</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J11" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sync workbook into DB (7 added, 206 matched pairs); manual mark uid 266
import_excel.py --apply, after backup transactions.backup-20260925-160233-pre-excel-sync.db:
- BL added rows 158-162: MGMT Concourse (8, $306.16); Grizmas 12/18 and
  12/19 (4 each, $283.92; the sheet's split of the 8-ticket GRiZMAS buy,
  event year corrected to 2026 in the sheet before sync); Max Dean b2b
  Luke Dean Concourse (18, $1,174.26) and VIP Concourse (6, $640.38)
- SL added SIDs 208-209: Prospa Mission 9/25 ($166.49, $162.49)
No rows updated or removed; no email rows touched.

match.py: 204 -> 206 pairs, net profit $10,470.58.
export.py: Pending 1 row (GRiZMAS email 555: one 8-ticket email vs two
4-ticket sheet rows, which auto-match doesn't combine).

manual_marks.csv: uid 266 (AXS email from 9/25 with no event, date,
qty or price), marked from the dashboard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N156"/>
+  <dimension ref="A1:N161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5021,6 +5021,141 @@
       </c>
       <c r="I156" s="9" t="n">
         <v>52.43</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>MGMT Concourse</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Concourse</t>
+        </is>
+      </c>
+      <c r="G157" s="9" t="n">
+        <v>38.27</v>
+      </c>
+      <c r="H157" t="n">
+        <v>8</v>
+      </c>
+      <c r="I157" s="9" t="n">
+        <v>306.16</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Grizmas 12/18</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="n">
+        <v>46374</v>
+      </c>
+      <c r="D158" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Masonic Temple Theater</t>
+        </is>
+      </c>
+      <c r="G158" s="9" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="H158" t="n">
+        <v>4</v>
+      </c>
+      <c r="I158" s="9" t="n">
+        <v>283.92</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Grizmas 12/19</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="n">
+        <v>46375</v>
+      </c>
+      <c r="D159" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Masonic Temple Theater</t>
+        </is>
+      </c>
+      <c r="G159" s="9" t="n">
+        <v>70.98</v>
+      </c>
+      <c r="H159" t="n">
+        <v>4</v>
+      </c>
+      <c r="I159" s="9" t="n">
+        <v>283.92</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean Concourse</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="D160" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Concourse</t>
+        </is>
+      </c>
+      <c r="G160" s="9" t="n">
+        <v>65.23666666666666</v>
+      </c>
+      <c r="H160" t="n">
+        <v>18</v>
+      </c>
+      <c r="I160" s="9" t="n">
+        <v>1174.26</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Max Dean b2b Luke Dean VIP Concourse</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="n">
+        <v>46389</v>
+      </c>
+      <c r="D161" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Concourse</t>
+        </is>
+      </c>
+      <c r="G161" s="9" t="n">
+        <v>106.73</v>
+      </c>
+      <c r="H161" t="n">
+        <v>6</v>
+      </c>
+      <c r="I161" s="9" t="n">
+        <v>640.38</v>
       </c>
     </row>
   </sheetData>
@@ -5034,7 +5169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O205"/>
+  <dimension ref="A1:O207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14320,32 +14455,32 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D179" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E179" s="8" t="n">
-        <v>46271</v>
+        <v>46290</v>
       </c>
       <c r="G179" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H179" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I179" s="9" t="n">
-        <v>87.5</v>
+        <v>153.31</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K179" t="inlineStr">
@@ -14354,16 +14489,16 @@
         </is>
       </c>
       <c r="L179" s="9" t="n">
-        <v>350</v>
+        <v>153.31</v>
       </c>
       <c r="M179" s="9" t="n">
-        <v>350</v>
+        <v>153.31</v>
       </c>
       <c r="N179" s="9" t="n">
-        <v>-130</v>
+        <v>98.69888888888889</v>
       </c>
       <c r="O179" s="7" t="n">
-        <v>-0.2708333333333333</v>
+        <v>1.807304170905392</v>
       </c>
     </row>
     <row r="180">
@@ -14372,32 +14507,32 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Justice Pacha</t>
+          <t>Prospa Mission</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D180" s="8" t="n">
-        <v>46270</v>
+        <v>46290</v>
       </c>
       <c r="E180" s="8" t="n">
-        <v>46271</v>
+        <v>46290</v>
       </c>
       <c r="G180" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H180" s="9" t="n">
-        <v>120</v>
+        <v>54.61111111111111</v>
       </c>
       <c r="I180" s="9" t="n">
-        <v>92.41500000000001</v>
+        <v>149.51</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K180" t="inlineStr">
@@ -14406,16 +14541,16 @@
         </is>
       </c>
       <c r="L180" s="9" t="n">
-        <v>369.66</v>
+        <v>149.51</v>
       </c>
       <c r="M180" s="9" t="n">
-        <v>369.66</v>
+        <v>149.51</v>
       </c>
       <c r="N180" s="9" t="n">
-        <v>-110.34</v>
+        <v>94.89888888888888</v>
       </c>
       <c r="O180" s="7" t="n">
-        <v>-0.2298749999999999</v>
+        <v>1.737721261444557</v>
       </c>
     </row>
     <row r="181">
@@ -14424,28 +14559,28 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D181" s="8" t="n">
-        <v>46242</v>
+        <v>46270</v>
       </c>
       <c r="E181" s="8" t="n">
-        <v>46242</v>
+        <v>46271</v>
       </c>
       <c r="G181" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H181" s="9" t="n">
-        <v>47.59</v>
+        <v>120</v>
       </c>
       <c r="I181" s="9" t="n">
-        <v>52</v>
+        <v>87.5</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
@@ -14458,16 +14593,16 @@
         </is>
       </c>
       <c r="L181" s="9" t="n">
-        <v>52</v>
+        <v>350</v>
       </c>
       <c r="M181" s="9" t="n">
-        <v>52</v>
+        <v>350</v>
       </c>
       <c r="N181" s="9" t="n">
-        <v>4.409999999999997</v>
+        <v>-130</v>
       </c>
       <c r="O181" s="7" t="n">
-        <v>0.09266652658121446</v>
+        <v>-0.2708333333333333</v>
       </c>
     </row>
     <row r="182">
@@ -14476,32 +14611,32 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Carlita Sound</t>
+          <t>Justice Pacha</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Pacha</t>
         </is>
       </c>
       <c r="D182" s="8" t="n">
-        <v>46242</v>
+        <v>46270</v>
       </c>
       <c r="E182" s="8" t="n">
-        <v>46242</v>
+        <v>46271</v>
       </c>
       <c r="G182" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H182" s="9" t="n">
-        <v>47.59</v>
+        <v>120</v>
       </c>
       <c r="I182" s="9" t="n">
-        <v>55</v>
+        <v>92.41500000000001</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K182" t="inlineStr">
@@ -14510,16 +14645,16 @@
         </is>
       </c>
       <c r="L182" s="9" t="n">
-        <v>55</v>
+        <v>369.66</v>
       </c>
       <c r="M182" s="9" t="n">
-        <v>55</v>
+        <v>369.66</v>
       </c>
       <c r="N182" s="9" t="n">
-        <v>7.409999999999997</v>
+        <v>-110.34</v>
       </c>
       <c r="O182" s="7" t="n">
-        <v>0.155704980037823</v>
+        <v>-0.2298749999999999</v>
       </c>
     </row>
     <row r="183">
@@ -14543,13 +14678,13 @@
         <v>46242</v>
       </c>
       <c r="G183" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H183" s="9" t="n">
         <v>47.59</v>
       </c>
       <c r="I183" s="9" t="n">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -14562,16 +14697,16 @@
         </is>
       </c>
       <c r="L183" s="9" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="M183" s="9" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="N183" s="9" t="n">
-        <v>-9.180000000000007</v>
+        <v>4.409999999999997</v>
       </c>
       <c r="O183" s="7" t="n">
-        <v>-0.09644883378861112</v>
+        <v>0.09266652658121446</v>
       </c>
     </row>
     <row r="184">
@@ -14580,32 +14715,32 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>TWINSICK TAO</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Tao</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D184" s="8" t="n">
-        <v>46270</v>
+        <v>46242</v>
       </c>
       <c r="E184" s="8" t="n">
-        <v>46271</v>
+        <v>46242</v>
       </c>
       <c r="G184" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H184" s="9" t="n">
-        <v>20</v>
+        <v>47.59</v>
       </c>
       <c r="I184" s="9" t="n">
-        <v>27.05</v>
+        <v>55</v>
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -14614,16 +14749,16 @@
         </is>
       </c>
       <c r="L184" s="9" t="n">
-        <v>108.2</v>
+        <v>55</v>
       </c>
       <c r="M184" s="9" t="n">
-        <v>108.2</v>
+        <v>55</v>
       </c>
       <c r="N184" s="9" t="n">
-        <v>28.2</v>
+        <v>7.409999999999997</v>
       </c>
       <c r="O184" s="7" t="n">
-        <v>0.3525</v>
+        <v>0.155704980037823</v>
       </c>
     </row>
     <row r="185">
@@ -14632,32 +14767,32 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Levity / Tape b K Bridge</t>
+          <t>Carlita Sound</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>K bridge</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D185" s="8" t="n">
-        <v>46256</v>
+        <v>46242</v>
       </c>
       <c r="E185" s="8" t="n">
-        <v>46258</v>
+        <v>46242</v>
       </c>
       <c r="G185" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H185" s="9" t="n">
-        <v>95</v>
+        <v>47.59</v>
       </c>
       <c r="I185" s="9" t="n">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
-          <t>Radiate</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K185" t="inlineStr">
@@ -14666,16 +14801,16 @@
         </is>
       </c>
       <c r="L185" s="9" t="n">
-        <v>1080</v>
+        <v>86</v>
       </c>
       <c r="M185" s="9" t="n">
-        <v>1080</v>
+        <v>86</v>
       </c>
       <c r="N185" s="9" t="n">
-        <v>-60</v>
+        <v>-9.180000000000007</v>
       </c>
       <c r="O185" s="7" t="n">
-        <v>-0.05263157894736842</v>
+        <v>-0.09644883378861112</v>
       </c>
     </row>
     <row r="186">
@@ -14684,28 +14819,28 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Parcels ACL</t>
+          <t>TWINSICK TAO</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Stubb's Waller Creek Amphitheater</t>
+          <t>Tao</t>
         </is>
       </c>
       <c r="D186" s="8" t="n">
-        <v>46298</v>
+        <v>46270</v>
       </c>
       <c r="E186" s="8" t="n">
         <v>46271</v>
       </c>
       <c r="G186" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H186" s="9" t="n">
-        <v>65.2</v>
+        <v>20</v>
       </c>
       <c r="I186" s="9" t="n">
-        <v>54.1</v>
+        <v>27.05</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -14718,16 +14853,16 @@
         </is>
       </c>
       <c r="L186" s="9" t="n">
-        <v>54.1</v>
+        <v>108.2</v>
       </c>
       <c r="M186" s="9" t="n">
-        <v>54.1</v>
+        <v>108.2</v>
       </c>
       <c r="N186" s="9" t="n">
-        <v>-11.1</v>
+        <v>28.2</v>
       </c>
       <c r="O186" s="7" t="n">
-        <v>-0.1702453987730062</v>
+        <v>0.3525</v>
       </c>
     </row>
     <row r="187">
@@ -14736,12 +14871,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Levity Tape B NYC afters</t>
+          <t>Levity / Tape b K Bridge</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Brooklyn Steel</t>
+          <t>K bridge</t>
         </is>
       </c>
       <c r="D187" s="8" t="n">
@@ -14751,17 +14886,17 @@
         <v>46258</v>
       </c>
       <c r="G187" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H187" s="9" t="n">
-        <v>62.37</v>
+        <v>95</v>
       </c>
       <c r="I187" s="9" t="n">
-        <v>44.25</v>
+        <v>90</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Radiate</t>
         </is>
       </c>
       <c r="K187" t="inlineStr">
@@ -14770,16 +14905,16 @@
         </is>
       </c>
       <c r="L187" s="9" t="n">
-        <v>177</v>
+        <v>1080</v>
       </c>
       <c r="M187" s="9" t="n">
-        <v>177</v>
+        <v>1080</v>
       </c>
       <c r="N187" s="9" t="n">
-        <v>-72.47999999999999</v>
+        <v>-60</v>
       </c>
       <c r="O187" s="7" t="n">
-        <v>-0.2905242905242905</v>
+        <v>-0.05263157894736842</v>
       </c>
     </row>
     <row r="188">
@@ -14788,16 +14923,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Arc Friday Pass 2026</t>
+          <t>Parcels ACL</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Arc</t>
+          <t>Stubb's Waller Creek Amphitheater</t>
         </is>
       </c>
       <c r="D188" s="8" t="n">
-        <v>46269</v>
+        <v>46298</v>
       </c>
       <c r="E188" s="8" t="n">
         <v>46271</v>
@@ -14806,10 +14941,10 @@
         <v>1</v>
       </c>
       <c r="H188" s="9" t="n">
-        <v>219</v>
+        <v>65.2</v>
       </c>
       <c r="I188" s="9" t="n">
-        <v>162.28</v>
+        <v>54.1</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -14822,16 +14957,16 @@
         </is>
       </c>
       <c r="L188" s="9" t="n">
-        <v>162.28</v>
+        <v>54.1</v>
       </c>
       <c r="M188" s="9" t="n">
-        <v>162.28</v>
+        <v>54.1</v>
       </c>
       <c r="N188" s="9" t="n">
-        <v>-56.72</v>
+        <v>-11.1</v>
       </c>
       <c r="O188" s="7" t="n">
-        <v>-0.2589954337899543</v>
+        <v>-0.1702453987730062</v>
       </c>
     </row>
     <row r="189">
@@ -14840,32 +14975,32 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Chris stussy Arc Afters</t>
+          <t>Levity Tape B NYC afters</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Radius</t>
+          <t>Brooklyn Steel</t>
         </is>
       </c>
       <c r="D189" s="8" t="n">
-        <v>46269</v>
+        <v>46256</v>
       </c>
       <c r="E189" s="8" t="n">
-        <v>46271</v>
+        <v>46258</v>
       </c>
       <c r="G189" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H189" s="9" t="n">
-        <v>100.24</v>
+        <v>62.37</v>
       </c>
       <c r="I189" s="9" t="n">
-        <v>117.21</v>
+        <v>44.25</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
@@ -14874,16 +15009,16 @@
         </is>
       </c>
       <c r="L189" s="9" t="n">
-        <v>117.21</v>
+        <v>177</v>
       </c>
       <c r="M189" s="9" t="n">
-        <v>117.21</v>
+        <v>177</v>
       </c>
       <c r="N189" s="9" t="n">
-        <v>16.97</v>
+        <v>-72.47999999999999</v>
       </c>
       <c r="O189" s="7" t="n">
-        <v>0.169293695131684</v>
+        <v>-0.2905242905242905</v>
       </c>
     </row>
     <row r="190">
@@ -14892,12 +15027,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Max dean ARC afters</t>
+          <t>Arc Friday Pass 2026</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Concord Music Hall</t>
+          <t>Arc</t>
         </is>
       </c>
       <c r="D190" s="8" t="n">
@@ -14907,13 +15042,13 @@
         <v>46271</v>
       </c>
       <c r="G190" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H190" s="9" t="n">
-        <v>42.18</v>
+        <v>219</v>
       </c>
       <c r="I190" s="9" t="n">
-        <v>63.1125</v>
+        <v>162.28</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -14926,16 +15061,16 @@
         </is>
       </c>
       <c r="L190" s="9" t="n">
-        <v>252.45</v>
+        <v>162.28</v>
       </c>
       <c r="M190" s="9" t="n">
-        <v>252.45</v>
+        <v>162.28</v>
       </c>
       <c r="N190" s="9" t="n">
-        <v>83.72999999999999</v>
+        <v>-56.72</v>
       </c>
       <c r="O190" s="7" t="n">
-        <v>0.4962660028449501</v>
+        <v>-0.2589954337899543</v>
       </c>
     </row>
     <row r="191">
@@ -14944,28 +15079,28 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Rufus Du Sol Boulder Bowl</t>
+          <t>Chris stussy Arc Afters</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Folsom</t>
+          <t>Radius</t>
         </is>
       </c>
       <c r="D191" s="8" t="n">
-        <v>46256</v>
+        <v>46269</v>
       </c>
       <c r="E191" s="8" t="n">
-        <v>46258</v>
+        <v>46271</v>
       </c>
       <c r="G191" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H191" s="9" t="n">
-        <v>110</v>
+        <v>100.24</v>
       </c>
       <c r="I191" s="9" t="n">
-        <v>243.43</v>
+        <v>117.21</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -14978,16 +15113,16 @@
         </is>
       </c>
       <c r="L191" s="9" t="n">
-        <v>486.86</v>
+        <v>117.21</v>
       </c>
       <c r="M191" s="9" t="n">
-        <v>486.86</v>
+        <v>117.21</v>
       </c>
       <c r="N191" s="9" t="n">
-        <v>266.86</v>
+        <v>16.97</v>
       </c>
       <c r="O191" s="7" t="n">
-        <v>1.213</v>
+        <v>0.169293695131684</v>
       </c>
     </row>
     <row r="192">
@@ -14996,32 +15131,32 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Goose RR</t>
+          <t>Max dean ARC afters</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Red Rocks</t>
+          <t>Concord Music Hall</t>
         </is>
       </c>
       <c r="D192" s="8" t="n">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="E192" s="8" t="n">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="G192" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H192" s="9" t="n">
-        <v>45</v>
+        <v>42.18</v>
       </c>
       <c r="I192" s="9" t="n">
-        <v>0</v>
+        <v>63.1125</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K192" t="inlineStr">
@@ -15030,16 +15165,16 @@
         </is>
       </c>
       <c r="L192" s="9" t="n">
-        <v>0</v>
+        <v>252.45</v>
       </c>
       <c r="M192" s="9" t="n">
-        <v>0</v>
+        <v>252.45</v>
       </c>
       <c r="N192" s="9" t="n">
-        <v>-45</v>
+        <v>83.72999999999999</v>
       </c>
       <c r="O192" s="7" t="n">
-        <v>-1</v>
+        <v>0.4962660028449501</v>
       </c>
     </row>
     <row r="193">
@@ -15048,32 +15183,32 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Rufus Du Sol Boulder Bowl</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Folsom</t>
         </is>
       </c>
       <c r="D193" s="8" t="n">
-        <v>46263</v>
+        <v>46256</v>
       </c>
       <c r="E193" s="8" t="n">
-        <v>46263</v>
+        <v>46258</v>
       </c>
       <c r="G193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H193" s="9" t="n">
-        <v>151.76</v>
+        <v>110</v>
       </c>
       <c r="I193" s="9" t="n">
-        <v>223.51</v>
+        <v>243.43</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K193" t="inlineStr">
@@ -15082,16 +15217,16 @@
         </is>
       </c>
       <c r="L193" s="9" t="n">
-        <v>223.51</v>
+        <v>486.86</v>
       </c>
       <c r="M193" s="9" t="n">
-        <v>223.51</v>
+        <v>486.86</v>
       </c>
       <c r="N193" s="9" t="n">
-        <v>71.75</v>
+        <v>266.86</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>0.4727859778597786</v>
+        <v>1.213</v>
       </c>
     </row>
     <row r="194">
@@ -15100,32 +15235,32 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Skrillex Gas Works</t>
+          <t>Goose RR</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Gas Works Park</t>
+          <t>Red Rocks</t>
         </is>
       </c>
       <c r="D194" s="8" t="n">
-        <v>46263</v>
+        <v>46266</v>
       </c>
       <c r="E194" s="8" t="n">
-        <v>46263</v>
+        <v>46267</v>
       </c>
       <c r="G194" t="n">
         <v>1</v>
       </c>
       <c r="H194" s="9" t="n">
-        <v>151.76</v>
+        <v>45</v>
       </c>
       <c r="I194" s="9" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
-          <t>radiate</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K194" t="inlineStr">
@@ -15134,16 +15269,16 @@
         </is>
       </c>
       <c r="L194" s="9" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="M194" s="9" t="n">
-        <v>230</v>
+        <v>0</v>
       </c>
       <c r="N194" s="9" t="n">
-        <v>78.24000000000001</v>
+        <v>-45</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0.5155508697944123</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="195">
@@ -15152,32 +15287,32 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>jamie xx NY</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Public Records</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D195" s="8" t="n">
-        <v>46269</v>
+        <v>46263</v>
       </c>
       <c r="E195" s="8" t="n">
-        <v>46271</v>
+        <v>46263</v>
       </c>
       <c r="G195" t="n">
         <v>1</v>
       </c>
       <c r="H195" s="9" t="n">
-        <v>49.44</v>
+        <v>151.76</v>
       </c>
       <c r="I195" s="9" t="n">
-        <v>0</v>
+        <v>223.51</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
-          <t>Loss</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K195" t="inlineStr">
@@ -15186,16 +15321,16 @@
         </is>
       </c>
       <c r="L195" s="9" t="n">
-        <v>0</v>
+        <v>223.51</v>
       </c>
       <c r="M195" s="9" t="n">
-        <v>0</v>
+        <v>223.51</v>
       </c>
       <c r="N195" s="9" t="n">
-        <v>-49.44</v>
+        <v>71.75</v>
       </c>
       <c r="O195" s="7" t="n">
-        <v>-1</v>
+        <v>0.4727859778597786</v>
       </c>
     </row>
     <row r="196">
@@ -15204,32 +15339,32 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Prospa Wednesday LA</t>
+          <t>Skrillex Gas Works</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Shrine</t>
+          <t>Gas Works Park</t>
         </is>
       </c>
       <c r="D196" s="8" t="n">
-        <v>46309</v>
+        <v>46263</v>
       </c>
       <c r="E196" s="8" t="n">
-        <v>46288</v>
+        <v>46263</v>
       </c>
       <c r="G196" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H196" s="9" t="n">
-        <v>59.98999999999999</v>
+        <v>151.76</v>
       </c>
       <c r="I196" s="9" t="n">
-        <v>85.59999999999999</v>
+        <v>230</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>radiate</t>
         </is>
       </c>
       <c r="K196" t="inlineStr">
@@ -15238,16 +15373,16 @@
         </is>
       </c>
       <c r="L196" s="9" t="n">
-        <v>428</v>
+        <v>230</v>
       </c>
       <c r="M196" s="9" t="n">
-        <v>428</v>
+        <v>230</v>
       </c>
       <c r="N196" s="9" t="n">
-        <v>128.05</v>
+        <v>78.24000000000001</v>
       </c>
       <c r="O196" s="7" t="n">
-        <v>0.4269044840806802</v>
+        <v>0.5155508697944123</v>
       </c>
     </row>
     <row r="197">
@@ -15256,32 +15391,32 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Prospa Wednesday LA</t>
+          <t>jamie xx NY</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Shrine</t>
+          <t>Public Records</t>
         </is>
       </c>
       <c r="D197" s="8" t="n">
-        <v>46309</v>
+        <v>46269</v>
       </c>
       <c r="E197" s="8" t="n">
-        <v>46290</v>
+        <v>46271</v>
       </c>
       <c r="G197" t="n">
         <v>1</v>
       </c>
       <c r="H197" s="9" t="n">
-        <v>59.99</v>
+        <v>49.44</v>
       </c>
       <c r="I197" s="9" t="n">
-        <v>85.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="J197" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="K197" t="inlineStr">
@@ -15290,16 +15425,16 @@
         </is>
       </c>
       <c r="L197" s="9" t="n">
-        <v>85.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="M197" s="9" t="n">
-        <v>85.65000000000001</v>
+        <v>0</v>
       </c>
       <c r="N197" s="9" t="n">
-        <v>25.66</v>
+        <v>-49.44</v>
       </c>
       <c r="O197" s="7" t="n">
-        <v>0.4277379563260544</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="198">
@@ -15308,32 +15443,32 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Adriatique B2B Cloonee</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Watson Island Park</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="D198" s="8" t="n">
-        <v>46361</v>
+        <v>46309</v>
       </c>
       <c r="E198" s="8" t="n">
-        <v>46276</v>
+        <v>46288</v>
       </c>
       <c r="G198" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H198" s="9" t="n">
-        <v>103.05</v>
+        <v>59.98999999999999</v>
       </c>
       <c r="I198" s="9" t="n">
-        <v>103.05</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="J198" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K198" t="inlineStr">
@@ -15342,16 +15477,16 @@
         </is>
       </c>
       <c r="L198" s="9" t="n">
-        <v>412.2</v>
+        <v>428</v>
       </c>
       <c r="M198" s="9" t="n">
-        <v>412.2</v>
+        <v>428</v>
       </c>
       <c r="N198" s="9" t="n">
-        <v>0</v>
+        <v>128.05</v>
       </c>
       <c r="O198" s="7" t="n">
-        <v>0</v>
+        <v>0.4269044840806802</v>
       </c>
     </row>
     <row r="199">
@@ -15360,32 +15495,32 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Ben Sterling Afters Sound</t>
+          <t>Prospa Wednesday LA</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Sound</t>
+          <t>Shrine</t>
         </is>
       </c>
       <c r="D199" s="8" t="n">
-        <v>46277</v>
+        <v>46309</v>
       </c>
       <c r="E199" s="8" t="n">
-        <v>46279</v>
+        <v>46290</v>
       </c>
       <c r="G199" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H199" s="9" t="n">
-        <v>47.59</v>
+        <v>59.99</v>
       </c>
       <c r="I199" s="9" t="n">
-        <v>75.5</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -15394,16 +15529,16 @@
         </is>
       </c>
       <c r="L199" s="9" t="n">
-        <v>302</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="M199" s="9" t="n">
-        <v>302</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="N199" s="9" t="n">
-        <v>111.64</v>
+        <v>25.66</v>
       </c>
       <c r="O199" s="7" t="n">
-        <v>0.586467745324648</v>
+        <v>0.4277379563260544</v>
       </c>
     </row>
     <row r="200">
@@ -15412,32 +15547,32 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Adriatique B2B Cloonee</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Watson Island Park</t>
         </is>
       </c>
       <c r="D200" s="8" t="n">
-        <v>46285</v>
+        <v>46361</v>
       </c>
       <c r="E200" s="8" t="n">
-        <v>46288</v>
+        <v>46276</v>
       </c>
       <c r="G200" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H200" s="9" t="n">
-        <v>188</v>
+        <v>103.05</v>
       </c>
       <c r="I200" s="9" t="n">
-        <v>218</v>
+        <v>103.05</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -15446,16 +15581,16 @@
         </is>
       </c>
       <c r="L200" s="9" t="n">
-        <v>218</v>
+        <v>412.2</v>
       </c>
       <c r="M200" s="9" t="n">
-        <v>218</v>
+        <v>412.2</v>
       </c>
       <c r="N200" s="9" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="O200" s="7" t="n">
-        <v>0.1595744680851064</v>
+        <v>0</v>
       </c>
     </row>
     <row r="201">
@@ -15464,28 +15599,28 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
+          <t>Ben Sterling Afters Sound</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Pacha</t>
+          <t>Sound</t>
         </is>
       </c>
       <c r="D201" s="8" t="n">
-        <v>46285</v>
+        <v>46277</v>
       </c>
       <c r="E201" s="8" t="n">
-        <v>46288</v>
+        <v>46279</v>
       </c>
       <c r="G201" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H201" s="9" t="n">
-        <v>188</v>
+        <v>47.59</v>
       </c>
       <c r="I201" s="9" t="n">
-        <v>209</v>
+        <v>75.5</v>
       </c>
       <c r="J201" t="inlineStr">
         <is>
@@ -15498,16 +15633,16 @@
         </is>
       </c>
       <c r="L201" s="9" t="n">
-        <v>418</v>
+        <v>302</v>
       </c>
       <c r="M201" s="9" t="n">
-        <v>418</v>
+        <v>302</v>
       </c>
       <c r="N201" s="9" t="n">
-        <v>42</v>
+        <v>111.64</v>
       </c>
       <c r="O201" s="7" t="n">
-        <v>0.1117021276595745</v>
+        <v>0.586467745324648</v>
       </c>
     </row>
     <row r="202">
@@ -15537,7 +15672,7 @@
         <v>188</v>
       </c>
       <c r="I202" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="J202" t="inlineStr">
         <is>
@@ -15550,16 +15685,16 @@
         </is>
       </c>
       <c r="L202" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="M202" s="9" t="n">
-        <v>190</v>
+        <v>218</v>
       </c>
       <c r="N202" s="9" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="O202" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>0.1595744680851064</v>
       </c>
     </row>
     <row r="203">
@@ -15589,7 +15724,7 @@
         <v>188</v>
       </c>
       <c r="I203" s="9" t="n">
-        <v>190</v>
+        <v>209</v>
       </c>
       <c r="J203" t="inlineStr">
         <is>
@@ -15602,16 +15737,16 @@
         </is>
       </c>
       <c r="L203" s="9" t="n">
-        <v>380</v>
+        <v>418</v>
       </c>
       <c r="M203" s="9" t="n">
-        <v>380</v>
+        <v>418</v>
       </c>
       <c r="N203" s="9" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="O203" s="7" t="n">
-        <v>0.01063829787234043</v>
+        <v>0.1117021276595745</v>
       </c>
     </row>
     <row r="204">
@@ -15620,7 +15755,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -15635,35 +15770,35 @@
         <v>46288</v>
       </c>
       <c r="G204" t="n">
+        <v>1</v>
+      </c>
+      <c r="H204" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I204" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L204" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="M204" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="N204" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="H204" s="9" t="n">
-        <v>326</v>
-      </c>
-      <c r="I204" s="9" t="n">
-        <v>293.92</v>
-      </c>
-      <c r="J204" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L204" s="9" t="n">
-        <v>587.84</v>
-      </c>
-      <c r="M204" s="9" t="n">
-        <v>587.84</v>
-      </c>
-      <c r="N204" s="9" t="n">
-        <v>-64.15999999999997</v>
-      </c>
       <c r="O204" s="7" t="n">
-        <v>-0.09840490797546007</v>
+        <v>0.01063829787234043</v>
       </c>
     </row>
     <row r="205">
@@ -15672,7 +15807,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+          <t>Experts Only (Sunday Afters) — 2026-09-20 — GA</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -15687,34 +15822,138 @@
         <v>46288</v>
       </c>
       <c r="G205" t="n">
+        <v>2</v>
+      </c>
+      <c r="H205" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="I205" s="9" t="n">
+        <v>190</v>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L205" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="M205" s="9" t="n">
+        <v>380</v>
+      </c>
+      <c r="N205" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O205" s="7" t="n">
+        <v>0.01063829787234043</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D206" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E206" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G206" t="n">
+        <v>2</v>
+      </c>
+      <c r="H206" s="9" t="n">
+        <v>326</v>
+      </c>
+      <c r="I206" s="9" t="n">
+        <v>293.92</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L206" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="M206" s="9" t="n">
+        <v>587.84</v>
+      </c>
+      <c r="N206" s="9" t="n">
+        <v>-64.15999999999997</v>
+      </c>
+      <c r="O206" s="7" t="n">
+        <v>-0.09840490797546007</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Experts Only Festival Afterparty — 2026-09-20 — BACKSTAGE DANCING VIP</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D207" s="8" t="n">
+        <v>46285</v>
+      </c>
+      <c r="E207" s="8" t="n">
+        <v>46288</v>
+      </c>
+      <c r="G207" t="n">
         <v>1</v>
       </c>
-      <c r="H205" s="9" t="n">
+      <c r="H207" s="9" t="n">
         <v>326</v>
       </c>
-      <c r="I205" s="9" t="n">
+      <c r="I207" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="J205" t="inlineStr">
+      <c r="J207" t="inlineStr">
         <is>
           <t>CrowdVolt</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr">
-        <is>
-          <t>transferred</t>
-        </is>
-      </c>
-      <c r="L205" s="9" t="n">
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>transferred</t>
+        </is>
+      </c>
+      <c r="L207" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="M205" s="9" t="n">
+      <c r="M207" s="9" t="n">
         <v>253</v>
       </c>
-      <c r="N205" s="9" t="n">
+      <c r="N207" s="9" t="n">
         <v>-73</v>
       </c>
-      <c r="O205" s="7" t="n">
+      <c r="O207" s="7" t="n">
         <v>-0.2239263803680982</v>
       </c>
     </row>
@@ -15729,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15829,271 +16068,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MGMT (DJ Set)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E3" s="8" t="n">
-        <v>46289.42085648148</v>
-      </c>
-      <c r="F3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G3" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="H3" s="9" t="n">
-        <v>153.08</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>MGMT (DJ Set)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>46312</v>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>46289.42576388889</v>
-      </c>
-      <c r="F4" t="n">
-        <v>4</v>
-      </c>
-      <c r="G4" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>153.08</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>46290.59245370371</v>
-      </c>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>AXS</t>
-        </is>
-      </c>
-      <c r="J5" t="b">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>quantity not stated and event details missing</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Max Dean b2b Luke Dean</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>46389</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>46290.50342592593</v>
-      </c>
-      <c r="F6" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="H6" s="9" t="n">
-        <v>378.96</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Max Dean b2b Luke Dean</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>46389</v>
-      </c>
-      <c r="E7" s="8" t="n">
-        <v>46290.50458333334</v>
-      </c>
-      <c r="F7" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>378.96</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Max Dean b2b Luke Dean</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>46389</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>46290.50798611111</v>
-      </c>
-      <c r="F8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G8" s="9" t="n">
-        <v>85</v>
-      </c>
-      <c r="H8" s="9" t="n">
-        <v>640.38</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>buy</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Max Dean b2b Luke Dean</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The Concourse Project</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="n">
-        <v>46389</v>
-      </c>
-      <c r="E9" s="8" t="n">
-        <v>46290.51108796296</v>
-      </c>
-      <c r="F9" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>55</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>416.34</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>See Tickets</t>
-        </is>
-      </c>
-      <c r="J9" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-26 (2 new transactions, 5 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16068,6 +16068,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>151.9</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>151.9</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-27 (2 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16108,6 +16108,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Levity</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46292.70423611111</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="9" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026 Breakaway Music Festival Utah - 2 Day Pass</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>America First Field</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46292.75152777778</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>196</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>196</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-28 (1 new transactions, 1 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16188,6 +16188,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026 Breakaway Music Festival Utah - 2 Day Pass</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>America First Field</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>196</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>196</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-28 (2 new transactions, 10 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16228,6 +16228,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Levity - Admissions</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>46293.79868055556</v>
+      </c>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>279.3</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-29 (2 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16306,6 +16306,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Levity - Admissions</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver, CO</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46294.02842592593</v>
+      </c>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="9" t="n"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Quantity not stated in ticket transfer email</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-29 (1 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16384,6 +16384,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E11" s="8" t="n">
+        <v>46294.15561342592</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-30 (1 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16424,6 +16424,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Parcels</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Stubbs BarBQ</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46294.94034722223</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>127.4</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-30 (3 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16464,6 +16464,129 @@
         <v>0</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Parcels</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Stubbs BBQ</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H13" s="9" t="n">
+        <v>127.4</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>delivery reminder email does not fit standard sale or purchase receipt categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Max Styler - Admissions</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall, Los Angeles, CA</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>quantity not stated in purchase update email</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Max Styler</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Shrine Expo Hall</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>46295.62550925926</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>328.98</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J15" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-30 (1 new transactions, 6 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16587,6 +16587,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Official 2026 ACL Nights: Levity</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Emo's Austin</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Ticketmaster</t>
+        </is>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>quantity not stated in purchase update email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-09-30 (4 new transactions, 6 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16625,6 +16625,165 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Levity - Admissions</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E17" s="8" t="n">
+        <v>46295.80070601852</v>
+      </c>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>quantity not stated and email kind is a pending transfer update</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>46295.88199074074</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Levity</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E19" s="8" t="n">
+        <v>46295.94729166666</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="9" t="n"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>46295.95287037037</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J20" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-01 (1 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16784,6 +16784,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E21" s="8" t="n">
+        <v>46296.01822916666</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H21" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J21" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-01 (1 new transactions, 1 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16824,6 +16824,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Levity - Admissions</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>46296.56278935185</v>
+      </c>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-01 (15 new transactions, 8 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16862,6 +16862,604 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Bunt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E23" s="8" t="n">
+        <v>46296.72788194445</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="H23" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>46296.74041666667</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>80.36</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>80.36</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <v>46296.75560185185</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>80.36</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>80.36</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>46296.7583912037</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E27" s="8" t="n">
+        <v>46296.75979166666</v>
+      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>46296.76119212963</v>
+      </c>
+      <c r="F28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E29" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H29" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>46296.76815972223</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E31" s="8" t="n">
+        <v>46296.76951388889</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>46296.77091435185</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - The Chainsmokers</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>46296.78223379629</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Parcels</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Stubbs BarBQ</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Official 2026 ACL Fest Nights: Parcels</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Stubb's Waller Creek Amphitheater - Austin, TX</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E35" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="9" t="n"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Ticketmaster</t>
+        </is>
+      </c>
+      <c r="J35" t="b">
+        <v>1</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Quantity not stated in ticket transfer email</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Bunt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>46296.8334375</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>34.3</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>46296.8834375</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J37" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-02 (6 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17460,6 +17460,246 @@
         <v>0</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>148.96</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Levity</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Emos Austin</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="9" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="H39" s="9" t="n">
+        <v>74.48</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Its Murph</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>46296</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Its Murph</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>46297.00982638889</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="H41" s="9" t="n">
+        <v>145.04</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Levity</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>46297.04449074074</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Its Murph</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>46297.05145833334</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>72.52</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-02 (6 new transactions, 16 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17700,6 +17700,247 @@
         <v>0</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Levity</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>46297.695625</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Soulection - 15 Year Anniversary</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Reframe Studios Outdoors, Los Angeles, US</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>46297.71891203704</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Soulection - 15 Year Anniversary</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Reframe Studios Outdoors, Los Angeles, US</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>46297.74674768518</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>46297.78476851852</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>97.02</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>97.02</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Soulection - 15 Year Anniversary</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Reframe Studios Outdoors, Los Angeles, US</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>46297.79461805556</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>180</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>46297.80296296296</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="9" t="n">
+        <v>97.02</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>194.04</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J49" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-03 (1 new transactions, 1 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17941,6 +17941,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-03 (4 new transactions, 4 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17981,6 +17981,167 @@
         <v>0</v>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Tape B</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Hallow Rocks - Tape B</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>46298.78775462963</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Max Styler (21+ Event)</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>46298.80431712963</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="9" t="n">
+        <v>59.78</v>
+      </c>
+      <c r="H53" s="9" t="n">
+        <v>59.78</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Max Styler (21+ Event)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>46298.81417824074</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>59.78</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>119.56</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J54" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-04 (4 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18142,6 +18142,166 @@
         <v>0</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Max Styler (21+ Event)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>46298.9431712963</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>59.78</v>
+      </c>
+      <c r="H55" s="9" t="n">
+        <v>59.78</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F56" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>106</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="H57" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Max Styler (21+ Event)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Shrine Auditorium and Expo Hall Los Angeles</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>46298</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>46299.01115740741</v>
+      </c>
+      <c r="F58" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="9" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="H58" s="9" t="n">
+        <v>117.6</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J58" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-04 (1 new transactions, 0 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18302,6 +18302,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>53</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J59" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-05 (1 new transactions, 6 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18382,6 +18382,47 @@
         <v>0</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Tape B</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E61" s="8" t="n">
+        <v>46300.75780092592</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="9" t="n"/>
+      <c r="H61" s="9" t="n"/>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-06 (1 new transactions, 0 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18423,6 +18423,46 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E62" s="8" t="n">
+        <v>46301.02231481481</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H62" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J62" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-07 (1 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18463,6 +18463,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Kettama (Friday)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Knockdown Center</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E63" s="8" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="H63" s="9" t="n">
+        <v>115</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J63" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-07 (3 new transactions, 6 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18503,6 +18503,126 @@
         <v>0</v>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Kettama (Thursday)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Knockdown Center</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="H64" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E65" s="8" t="n">
+        <v>46302.79355324074</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="H65" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Jamie Jones</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E66" s="8" t="n">
+        <v>46302.81402777778</v>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="H66" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J66" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-08 (1 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18623,6 +18623,47 @@
         <v>0</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E67" s="8" t="n">
+        <v>46303.67850694444</v>
+      </c>
+      <c r="F67" t="n">
+        <v>5</v>
+      </c>
+      <c r="G67" s="9" t="n"/>
+      <c r="H67" s="9" t="n"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J67" t="b">
+        <v>1</v>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>total_price and price not provided in ticket transfer email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-09 (3 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18664,6 +18664,126 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>46304.18209490741</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H68" s="9" t="n">
+        <v>143.08</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Main Space at Knockdown Center - Complex</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>46304.24525462963</v>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="9" t="n">
+        <v>126</v>
+      </c>
+      <c r="H69" s="9" t="n">
+        <v>126</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Main Space at Knockdown Center - Complex</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E70" s="8" t="n">
+        <v>46304.34599537037</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="H70" s="9" t="n">
+        <v>135</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J70" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-09 (4 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18784,6 +18784,160 @@
         <v>0</v>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Soulection - 15 Year Anniversary</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F71" t="n">
+        <v>5</v>
+      </c>
+      <c r="G71" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H71" s="9" t="n">
+        <v>450</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>RUSH Presents: Kettama</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Knockdown Center</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E72" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F72" t="n">
+        <v>3</v>
+      </c>
+      <c r="G72" s="9" t="n"/>
+      <c r="H72" s="9" t="n"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J72" t="b">
+        <v>1</v>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>total_price and price not provided in purchase update email</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E73" s="8" t="n">
+        <v>46304.61098379629</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="9" t="n"/>
+      <c r="H73" s="9" t="n"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J73" t="b">
+        <v>1</v>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Kettama (Friday)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Knockdown Center</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E74" s="8" t="n">
+        <v>46304.70957175926</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="H74" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J74" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-09 (10 new transactions, 17 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K74"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18938,6 +18938,407 @@
         <v>0</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Bunt</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E75" s="8" t="n">
+        <v>46304.72655092592</v>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H75" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Bunt</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>46304.73756944444</v>
+      </c>
+      <c r="F76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>jigitz</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>46304.7386574074</v>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="9" t="n"/>
+      <c r="H77" s="9" t="n"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J77" t="b">
+        <v>1</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>total_price and price not provided in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E78" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="H78" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J78" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E79" s="8" t="n">
+        <v>46304.74318287037</v>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="H79" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J79" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Francis Mercier</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="H80" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Francis Mercier</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E81" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F81" t="n">
+        <v>2</v>
+      </c>
+      <c r="G81" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="H81" s="9" t="n">
+        <v>58</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J81" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>46304.77231481481</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="H82" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Francis Mercier</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E83" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="H83" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Francis Mercier</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="H84" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J84" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-10 (2 new transactions, 0 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19339,6 +19339,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Francis Mercier</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="n">
+        <v>46306</v>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="H85" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J85" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ACL Fest Nights - Bunt</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>46304.96396990741</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="H86" s="9" t="n">
+        <v>82.31999999999999</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J86" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-10 (3 new transactions, 5 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19419,6 +19419,126 @@
         <v>0</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>46305.09447916667</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="H87" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J87" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E88" s="8" t="n">
+        <v>46305.10164351852</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="H88" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J88" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E89" s="8" t="n">
+        <v>46305.10165509259</v>
+      </c>
+      <c r="F89" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="H89" s="9" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J89" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-10 (1 new transactions, 0 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:K90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19539,6 +19539,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>jigitz - Admissions</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>46305.6253125</v>
+      </c>
+      <c r="G90" s="9" t="n"/>
+      <c r="H90" s="9" t="n"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J90" t="b">
+        <v>1</v>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>quantity not stated and email kind is a pending transfer update</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-10 (1 new transactions, 2 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K90"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19577,6 +19577,46 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E91" s="8" t="n">
+        <v>46305.64864583333</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>70.56</v>
+      </c>
+      <c r="H91" s="9" t="n">
+        <v>70.56</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J91" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-10 (7 new transactions, 5 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19617,6 +19617,286 @@
         <v>0</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E92" s="8" t="n">
+        <v>46305.91119212963</v>
+      </c>
+      <c r="F92" t="n">
+        <v>1</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="H92" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E93" s="8" t="n">
+        <v>46305.92230324074</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H93" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>46305.94876157407</v>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H94" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J94" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E95" s="8" t="n">
+        <v>46305.9516087963</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="H95" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J95" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>46305.95565972223</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="H96" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J96" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>46305.96258101852</v>
+      </c>
+      <c r="F97" t="n">
+        <v>2</v>
+      </c>
+      <c r="G97" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H97" s="9" t="n">
+        <v>166.6</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J97" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Jigitz</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Ogden Theatre</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>46305.9653587963</v>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H98" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J98" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-11 (1 new transactions, 0 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K98"/>
+  <dimension ref="A1:K99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19897,6 +19897,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>46306.29589120371</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H99" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J99" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-11 (3 new transactions, 3 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K99"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19937,6 +19937,126 @@
         <v>0</v>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Music On: Marco Carola, Franky Rizardo, &amp; More</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>46306.66758101852</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="H100" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J100" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Music On: Marco Carola, Franky Rizardo, &amp; More</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E101" s="8" t="n">
+        <v>46306.66857638889</v>
+      </c>
+      <c r="F101" t="n">
+        <v>2</v>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>150</v>
+      </c>
+      <c r="H101" s="9" t="n">
+        <v>300</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D102" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>46306.73065972222</v>
+      </c>
+      <c r="F102" t="n">
+        <v>1</v>
+      </c>
+      <c r="G102" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H102" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J102" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-12 (2 new transactions, 1 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20177,6 +20177,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D106" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E106" s="8" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1</v>
+      </c>
+      <c r="G106" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H106" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J106" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E107" s="8" t="n">
+        <v>46307.21671296296</v>
+      </c>
+      <c r="F107" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H107" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J107" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-12 (1 new transactions, 1 skipped, 206 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -15968,7 +15968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20257,6 +20257,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D108" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E108" s="8" t="n">
+        <v>46307.51533564815</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1</v>
+      </c>
+      <c r="G108" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H108" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J108" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-13 (-2 new transactions, 9 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19997,37 +19997,36 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Levity</t>
+          <t>Soulection - 15 Year Anniversary</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Red Rocks Amphitheatre</t>
+          <t>Reframe Studios Outdoors, Los Angeles, US</t>
         </is>
       </c>
       <c r="D15" s="8" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>46297.695625</v>
+        <v>46297.71891203704</v>
       </c>
       <c r="F15" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
+      <c r="G15" s="9" t="n">
+        <v>90</v>
+      </c>
+      <c r="H15" s="9" t="n">
+        <v>90</v>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>transfer out with no sale price — possibly an off-platform sale</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -20050,16 +20049,16 @@
         <v>46298</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>46297.71891203704</v>
+        <v>46297.74674768518</v>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" s="9" t="n">
         <v>90</v>
       </c>
       <c r="H16" s="9" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -20090,7 +20089,7 @@
         <v>46298</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>46297.74674768518</v>
+        <v>46297.79461805556</v>
       </c>
       <c r="F17" t="n">
         <v>2</v>
@@ -20118,36 +20117,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Soulection - 15 Year Anniversary</t>
+          <t>Tape B</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Reframe Studios Outdoors, Los Angeles, US</t>
+          <t>Red Rocks Amphitheatre</t>
         </is>
       </c>
       <c r="D18" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E18" s="8" t="n">
         <v>46298</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>46297.79461805556</v>
       </c>
       <c r="F18" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <v>180</v>
-      </c>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>AXS</t>
         </is>
       </c>
       <c r="J18" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -20170,7 +20170,7 @@
         <v>46304</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>46298</v>
+        <v>46300.75780092592</v>
       </c>
       <c r="F19" t="n">
         <v>2</v>
@@ -20199,37 +20199,36 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tape B</t>
+          <t>Odd Mob</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Red Rocks Amphitheatre</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D20" s="8" t="n">
-        <v>46304</v>
+        <v>46318</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>46300.75780092592</v>
+        <v>46301.02231481481</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J20" t="b">
-        <v>1</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>transfer out with no sale price — possibly an off-platform sale</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -20240,32 +20239,32 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Odd Mob</t>
+          <t>Kettama (Thursday)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Knockdown Center</t>
         </is>
       </c>
       <c r="D21" s="8" t="n">
-        <v>46318</v>
+        <v>46303</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>46301.02231481481</v>
+        <v>46302</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>71.54000000000001</v>
+        <v>61</v>
       </c>
       <c r="H21" s="9" t="n">
-        <v>71.54000000000001</v>
+        <v>61</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -20280,32 +20279,32 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Kettama (Thursday)</t>
+          <t>Odd Mob</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Knockdown Center</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D22" s="8" t="n">
-        <v>46303</v>
+        <v>46318</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>46302</v>
+        <v>46304.18209490741</v>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>61</v>
+        <v>71.54000000000001</v>
       </c>
       <c r="H22" s="9" t="n">
-        <v>61</v>
+        <v>143.08</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>CrowdVolt</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J22" t="b">
@@ -20320,32 +20319,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Odd Mob</t>
+          <t>Kettama</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Main Space at Knockdown Center - Complex</t>
         </is>
       </c>
       <c r="D23" s="8" t="n">
-        <v>46318</v>
+        <v>46304</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>46304.18209490741</v>
+        <v>46304.24525462963</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>71.54000000000001</v>
+        <v>126</v>
       </c>
       <c r="H23" s="9" t="n">
-        <v>143.08</v>
+        <v>126</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Lysted</t>
+          <t>StubHub</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -20372,16 +20371,16 @@
         <v>46304</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>46304.24525462963</v>
+        <v>46304.34599537037</v>
       </c>
       <c r="F24" t="n">
         <v>1</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -20400,28 +20399,20 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Kettama</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Main Space at Knockdown Center - Complex</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="n">
+          <t>Soulection - 15 Year Anniversary</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="n">
         <v>46304</v>
       </c>
-      <c r="E25" s="8" t="n">
-        <v>46304.34599537037</v>
-      </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>135</v>
+        <v>90</v>
       </c>
       <c r="H25" s="9" t="n">
-        <v>135</v>
+        <v>450</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -20435,44 +20426,53 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>sell</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Soulection - 15 Year Anniversary</t>
-        </is>
+          <t>RUSH Presents: Kettama</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Knockdown Center</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>46304</v>
       </c>
       <c r="E26" s="8" t="n">
         <v>46304</v>
       </c>
       <c r="F26" t="n">
-        <v>5</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>90</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>450</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="9" t="n"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>StubHub</t>
+          <t>Dice</t>
         </is>
       </c>
       <c r="J26" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>total_price and price not provided in purchase update email</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>sell</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>RUSH Presents: Kettama</t>
+          <t>Kettama (Friday)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -20484,25 +20484,24 @@
         <v>46304</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>46304</v>
+        <v>46304.70957175926</v>
       </c>
       <c r="F27" t="n">
-        <v>3</v>
-      </c>
-      <c r="G27" s="9" t="n"/>
-      <c r="H27" s="9" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="G27" s="9" t="n">
+        <v>130</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>130</v>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Dice</t>
+          <t>CrowdVolt</t>
         </is>
       </c>
       <c r="J27" t="b">
-        <v>1</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>total_price and price not provided in purchase update email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -20513,19 +20512,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sammy Virji</t>
+          <t>jigitz</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Red Rocks Amphitheatre</t>
+          <t>Ogden Theatre</t>
         </is>
       </c>
       <c r="D28" s="8" t="n">
-        <v>46311</v>
+        <v>46305</v>
       </c>
       <c r="E28" s="8" t="n">
-        <v>46304.61098379629</v>
+        <v>46304.7386574074</v>
       </c>
       <c r="F28" t="n">
         <v>1</v>
@@ -20542,7 +20541,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>transfer out with no sale price — possibly an off-platform sale</t>
+          <t>total_price and price not provided in email</t>
         </is>
       </c>
     </row>
@@ -20554,36 +20553,34 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kettama (Friday)</t>
+          <t>jigitz - Admissions</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Knockdown Center</t>
+          <t>Ogden Theatre</t>
         </is>
       </c>
       <c r="D29" s="8" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="E29" s="8" t="n">
-        <v>46304.70957175926</v>
-      </c>
-      <c r="F29" t="n">
+        <v>46305.6253125</v>
+      </c>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J29" t="b">
         <v>1</v>
       </c>
-      <c r="G29" s="9" t="n">
-        <v>130</v>
-      </c>
-      <c r="H29" s="9" t="n">
-        <v>130</v>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>CrowdVolt</t>
-        </is>
-      </c>
-      <c r="J29" t="b">
-        <v>0</v>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>quantity not stated and email kind is a pending transfer update</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -20594,37 +20591,36 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>jigitz</t>
+          <t>Odd Mob</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Ogden Theatre</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D30" s="8" t="n">
-        <v>46305</v>
+        <v>46318</v>
       </c>
       <c r="E30" s="8" t="n">
-        <v>46304.7386574074</v>
+        <v>46305.64864583333</v>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
+      <c r="G30" s="9" t="n">
+        <v>70.56</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>70.56</v>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J30" t="b">
-        <v>1</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>total_price and price not provided in email</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -20635,34 +20631,36 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>jigitz - Admissions</t>
+          <t>Odd Mob</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Ogden Theatre</t>
+          <t>Mission Ballroom</t>
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>46305</v>
+        <v>46318</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>46305.6253125</v>
-      </c>
-      <c r="G31" s="9" t="n"/>
-      <c r="H31" s="9" t="n"/>
+        <v>46305.92230324074</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>71.54000000000001</v>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>AXS</t>
+          <t>Lysted</t>
         </is>
       </c>
       <c r="J31" t="b">
-        <v>1</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>quantity not stated and email kind is a pending transfer update</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -20685,16 +20683,16 @@
         <v>46318</v>
       </c>
       <c r="E32" s="8" t="n">
-        <v>46305.64864583333</v>
+        <v>46305.94876157407</v>
       </c>
       <c r="F32" t="n">
         <v>1</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>70.56</v>
+        <v>71.54000000000001</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>70.56</v>
+        <v>71.54000000000001</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -20725,7 +20723,7 @@
         <v>46318</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>46305.92230324074</v>
+        <v>46306.29589120371</v>
       </c>
       <c r="F33" t="n">
         <v>1</v>
@@ -20765,7 +20763,7 @@
         <v>46318</v>
       </c>
       <c r="E34" s="8" t="n">
-        <v>46305.94876157407</v>
+        <v>46307.21671296296</v>
       </c>
       <c r="F34" t="n">
         <v>1</v>
@@ -20793,28 +20791,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Odd Mob</t>
+          <t>Music On</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Mission Ballroom</t>
+          <t>Pacha New York</t>
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>46318</v>
+        <v>46311</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>46306.29589120371</v>
+        <v>46307.97783564815</v>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>71.54000000000001</v>
+        <v>147</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>71.54000000000001</v>
+        <v>294</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -20822,46 +20820,6 @@
         </is>
       </c>
       <c r="J35" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>sell</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Odd Mob</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Mission Ballroom</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="n">
-        <v>46318</v>
-      </c>
-      <c r="E36" s="8" t="n">
-        <v>46307.21671296296</v>
-      </c>
-      <c r="F36" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="9" t="n">
-        <v>71.54000000000001</v>
-      </c>
-      <c r="H36" s="9" t="n">
-        <v>71.54000000000001</v>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Lysted</t>
-        </is>
-      </c>
-      <c r="J36" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-13 (1 new transactions, 6 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20823,6 +20823,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>46308.73199074074</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J36" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-13 (5 new transactions, 9 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20863,6 +20863,208 @@
         <v>0</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E37" s="8" t="n">
+        <v>46308.77505787037</v>
+      </c>
+      <c r="F37" t="n">
+        <v>6</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H37" s="9" t="n">
+        <v>470.4</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>PAWSA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>The Rio Vista Lot - The Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>46308.80211805556</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <v>108.77</v>
+      </c>
+      <c r="H38" s="9" t="n">
+        <v>108.77</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E39" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="9" t="n"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>transfer out with no sale price — possibly an off-platform sale</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>PAWSA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The Rio Vista Lot - The Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="9" t="n">
+        <v>108.77</v>
+      </c>
+      <c r="H40" s="9" t="n">
+        <v>108.77</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Red Rocks, Morrison, CO</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E41" s="8" t="n">
+        <v>46308.82743055555</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2</v>
+      </c>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="9" t="n"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>transfer update without price or purchase receipt details</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-14 (2 new transactions, 4 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21065,6 +21065,86 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>46309.78200231482</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H42" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E43" s="8" t="n">
+        <v>46309.9111574074</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H43" s="9" t="n">
+        <v>156.8</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J43" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-15 (6 new transactions, 1 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21145,6 +21145,276 @@
         <v>0</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The Concourse Project - Austin, TX</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>46310.16959490741</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H44" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>order is past due and pending fulfillment action</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E45" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H45" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Email indicates a past due sale fulfillment warning rather than a standard sale confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>156.8</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>past due fulfillment notice for an existing sale, email kind does not strictly fit standard categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E47" s="8" t="n">
+        <v>46310.16959490741</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H47" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J47" t="b">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>email is an urgent past due delivery notice rather than a standard sale confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>46310.16959490741</v>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H48" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J48" t="b">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>past due fulfillment notification with unclear sale/purchase state</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The Concourse Project - Complex</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E49" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H49" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Email indicates past due fulfillment/cancellation warning rather than a standard sale confirmation or listing.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-15 (2 new transactions, 6 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21415,6 +21415,83 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>46310.60342592592</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <v>130.5</v>
+      </c>
+      <c r="H50" s="9" t="n">
+        <v>261</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>StubHub</t>
+        </is>
+      </c>
+      <c r="J50" t="b">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>venue and event_date not provided in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MGMT</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E51" s="8" t="n">
+        <v>46310.76116898148</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="9" t="n">
+        <v>78.39</v>
+      </c>
+      <c r="H51" s="9" t="n">
+        <v>78.39</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J51" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-16 (2 new transactions, 1 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21492,6 +21492,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Costa</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>46354</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="F52" t="n">
+        <v>8</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>245.28</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="n">
+        <v>46311.15168981482</v>
+      </c>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>quantity, event details, and pricing not stated in delivery update email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-16 (1 new transactions, 1 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21552,6 +21552,46 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Hugel Presents Make The Girls Dance - On The Beach</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>National Hotel</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>46359</v>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>96.63</v>
+      </c>
+      <c r="H54" s="9" t="n">
+        <v>206.8</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J54" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-16 (4 new transactions, 10 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21592,6 +21592,164 @@
         <v>0</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Music On: Marco Carola, Franky Rizardo, &amp; More</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E55" s="8" t="n">
+        <v>46311.76393518518</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="9" t="n">
+        <v>117</v>
+      </c>
+      <c r="H55" s="9" t="n">
+        <v>117</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Circoloco Miami (Factory Basel 2026)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Factory Town</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>46361</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>46311.77398148148</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="9" t="n">
+        <v>150.48</v>
+      </c>
+      <c r="H56" s="9" t="n">
+        <v>161.01</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Circoloco Miami</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Factory Town</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>46361</v>
+      </c>
+      <c r="E57" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H57" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>The Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G58" s="9" t="n"/>
+      <c r="H58" s="9" t="n"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>TickPick</t>
+        </is>
+      </c>
+      <c r="J58" t="b">
+        <v>1</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>quantity not stated in purchase update email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-17 (2 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21750,6 +21750,86 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E59" s="8" t="n">
+        <v>46311.9543287037</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="H59" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Sammy Virji</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>46311</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>46311.95571759259</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="H60" s="9" t="n">
+        <v>81.33</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J60" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-17 (2 new transactions, 1 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21830,6 +21830,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E61" s="8" t="n">
+        <v>46312.14097222222</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="H61" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E62" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F62" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="9" t="n">
+        <v>140</v>
+      </c>
+      <c r="H62" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J62" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-17 (1 new transactions, 0 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21910,6 +21910,47 @@
         <v>0</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>PAWSA</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>The Rio Vista Lot - The Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E63" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" s="9" t="n"/>
+      <c r="H63" s="9" t="n"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J63" t="b">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>total_price not provided in ticket reminder email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-17 (1 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21951,6 +21951,44 @@
         </is>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>46312.84520833333</v>
+      </c>
+      <c r="G64" s="9" t="n"/>
+      <c r="H64" s="9" t="n"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J64" t="b">
+        <v>1</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>quantity not stated and email is a transfer pending notification rather than a standard sale or purchase</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-18 (3 new transactions, 6 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21989,6 +21989,126 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E65" s="8" t="n">
+        <v>46313.03853009259</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="H65" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E66" s="8" t="n">
+        <v>46313.03878472222</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2</v>
+      </c>
+      <c r="G66" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="H66" s="9" t="n">
+        <v>402</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Pawsa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Historic Sears Building</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="E67" s="8" t="n">
+        <v>46313.04320601852</v>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="H67" s="9" t="n">
+        <v>201</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J67" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-18 (2 new transactions, 0 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K67"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22109,6 +22109,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Łaszewo</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="n">
+        <v>46402</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>46313.88675925926</v>
+      </c>
+      <c r="F68" t="n">
+        <v>6</v>
+      </c>
+      <c r="G68" s="9" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="H68" s="9" t="n">
+        <v>473.04</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="n">
+        <v>46313.88681712963</v>
+      </c>
+      <c r="G69" s="9" t="n"/>
+      <c r="H69" s="9" t="n"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>quantity not stated in email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-19 (4 new transactions, 4 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22169,6 +22169,166 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Kaytranada</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E70" s="8" t="n">
+        <v>46313.89887731482</v>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="9" t="n">
+        <v>270</v>
+      </c>
+      <c r="H70" s="9" t="n">
+        <v>270</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J70" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ANOTR</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Ace Mission Studios</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E71" s="8" t="n">
+        <v>46313.92927083333</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2</v>
+      </c>
+      <c r="G71" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="H71" s="9" t="n">
+        <v>294</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Macklemore</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E72" s="8" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="H72" s="9" t="n">
+        <v>88.2</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J72" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E73" s="8" t="n">
+        <v>46313.96810185185</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H73" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J73" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-19 (5 new transactions, 3 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22329,6 +22329,207 @@
         <v>0</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Macklemore</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Red Rocks, Morrison, CO</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E74" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F74" t="n">
+        <v>2</v>
+      </c>
+      <c r="G74" s="9" t="n"/>
+      <c r="H74" s="9" t="n"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J74" t="b">
+        <v>1</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>total_price and payout_amount not stated in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Macklemore</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E75" s="8" t="n">
+        <v>46314.03199074074</v>
+      </c>
+      <c r="F75" t="n">
+        <v>2</v>
+      </c>
+      <c r="G75" s="9" t="n">
+        <v>88.20999999999999</v>
+      </c>
+      <c r="H75" s="9" t="n">
+        <v>176.42</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J75" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>46314.04612268518</v>
+      </c>
+      <c r="F76" t="n">
+        <v>2</v>
+      </c>
+      <c r="G76" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>127.4</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E77" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H77" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J77" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E78" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H78" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J78" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-19 (1 new transactions, 0 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:K79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22530,6 +22530,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E79" s="8" t="n">
+        <v>46314.68760416667</v>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="9" t="n">
+        <v>62.56</v>
+      </c>
+      <c r="H79" s="9" t="n">
+        <v>62.56</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J79" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-19 (6 new transactions, 6 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22570,6 +22570,226 @@
         <v>0</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Łaszewo</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>46402</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F80" t="n">
+        <v>6</v>
+      </c>
+      <c r="G80" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="H80" s="9" t="n">
+        <v>513.0599999999999</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="n">
+        <v>46314.75868055555</v>
+      </c>
+      <c r="G81" s="9" t="n"/>
+      <c r="H81" s="9" t="n"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J81" t="b">
+        <v>1</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>quantity and event details not stated in delivery confirmation email</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>46314.76832175926</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H82" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J82" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Prospa</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>LIV Nightclub Miami</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>46360</v>
+      </c>
+      <c r="E83" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F83" t="n">
+        <v>6</v>
+      </c>
+      <c r="G83" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H83" s="9" t="n">
+        <v>371.82</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Universe</t>
+        </is>
+      </c>
+      <c r="J83" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>46314.77646990741</v>
+      </c>
+      <c r="F84" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="H84" s="9" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J84" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ANOTR</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Ace Mission Studios</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E85" s="8" t="n">
+        <v>46314.87646990741</v>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="H85" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J85" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-20 (2 new transactions, 1 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K85"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22790,6 +22790,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ANOTR</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Ace Mission Studios</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>46314.94871527778</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="H86" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J86" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ANOTR</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Ace Mission Studios</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E87" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="H87" s="9" t="n">
+        <v>147</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J87" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-20 (1 new transactions, 3 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22870,6 +22870,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E88" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F88" t="n">
+        <v>1</v>
+      </c>
+      <c r="G88" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H88" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J88" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-20 (6 new transactions, 7 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22910,6 +22910,246 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>TINASHE - THE SHOW MUST GO ON</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Stubb's Waller Creek Amphitheater — Austin, TX</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>46492</v>
+      </c>
+      <c r="E89" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G89" s="9" t="n"/>
+      <c r="H89" s="9" t="n">
+        <v>57.38</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Ticketmaster</t>
+        </is>
+      </c>
+      <c r="J89" t="b">
+        <v>1</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>quantity not stated in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Tinashe</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Stubb's Waller Creek Amphitheater</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>46492</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F90" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="9" t="n">
+        <v>57.38</v>
+      </c>
+      <c r="H90" s="9" t="n">
+        <v>57.38</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Victory Live</t>
+        </is>
+      </c>
+      <c r="J90" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E91" s="8" t="n">
+        <v>46315.73202546296</v>
+      </c>
+      <c r="F91" t="n">
+        <v>2</v>
+      </c>
+      <c r="G91" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H91" s="9" t="n">
+        <v>137.2</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J91" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Ian Asher (18+ Event)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E92" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F92" t="n">
+        <v>2</v>
+      </c>
+      <c r="G92" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H92" s="9" t="n">
+        <v>137.2</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J92" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Calvin Harris - North America Tour</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Delta Center, Salt Lake City, UT</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>46512</v>
+      </c>
+      <c r="E93" s="8" t="n">
+        <v>46315.47291666667</v>
+      </c>
+      <c r="F93" t="n">
+        <v>2</v>
+      </c>
+      <c r="G93" s="9" t="n">
+        <v>128.72</v>
+      </c>
+      <c r="H93" s="9" t="n">
+        <v>257.44</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>SeatGeek</t>
+        </is>
+      </c>
+      <c r="J93" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Calvin Harris</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Toyota Center - TX</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>46315.77090277777</v>
+      </c>
+      <c r="F94" t="n">
+        <v>2</v>
+      </c>
+      <c r="G94" s="9" t="n">
+        <v>441</v>
+      </c>
+      <c r="H94" s="9" t="n">
+        <v>882</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J94" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-20 (6 new transactions, 5 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K94"/>
+  <dimension ref="A1:K100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23150,6 +23150,241 @@
         <v>0</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E95" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="G95" s="9" t="n"/>
+      <c r="H95" s="9" t="n"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J95" t="b">
+        <v>1</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>46315.79900462963</v>
+      </c>
+      <c r="G96" s="9" t="n"/>
+      <c r="H96" s="9" t="n"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J96" t="b">
+        <v>1</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>quantity not stated in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E97" s="8" t="n">
+        <v>46315.8000925926</v>
+      </c>
+      <c r="G97" s="9" t="n"/>
+      <c r="H97" s="9" t="n"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J97" t="b">
+        <v>1</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Macklemore</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Red Rocks</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>46315.81836805555</v>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" s="9" t="n"/>
+      <c r="H98" s="9" t="n"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J98" t="b">
+        <v>1</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>total_price and price not stated in email</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Macklemore</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Red Rocks Amphitheatre</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E99" s="8" t="n">
+        <v>46315.81950231481</v>
+      </c>
+      <c r="F99" t="n">
+        <v>1</v>
+      </c>
+      <c r="G99" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="H99" s="9" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J99" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Ian Asher (18+ Event)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>46315.85146990741</v>
+      </c>
+      <c r="F100" t="n">
+        <v>1</v>
+      </c>
+      <c r="G100" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H100" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J100" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-21 (8 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23385,6 +23385,246 @@
         <v>0</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>TINASHE - The Show Must Go On - Artist Presale</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E101" s="8" t="n">
+        <v>46315.99322916667</v>
+      </c>
+      <c r="F101" t="n">
+        <v>4</v>
+      </c>
+      <c r="G101" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H101" s="9" t="n">
+        <v>222.64</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>46315.99324074074</v>
+      </c>
+      <c r="G102" s="9" t="n"/>
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J102" t="b">
+        <v>1</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>quantity, event details, and pricing not stated in delivery confirmation</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>TINASHE - The Show Must Go On</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E103" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F103" t="n">
+        <v>4</v>
+      </c>
+      <c r="G103" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H103" s="9" t="n">
+        <v>222.64</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J103" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E104" s="8" t="n">
+        <v>46316.03075231481</v>
+      </c>
+      <c r="G104" s="9" t="n"/>
+      <c r="H104" s="9" t="n"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J104" t="b">
+        <v>1</v>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>quantity, event details, and pricing not stated in delivery notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>TINASHE - The Show Must Go On</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E105" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F105" t="n">
+        <v>4</v>
+      </c>
+      <c r="G105" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H105" s="9" t="n">
+        <v>222.64</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J105" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E106" s="8" t="n">
+        <v>46316.03822916667</v>
+      </c>
+      <c r="G106" s="9" t="n"/>
+      <c r="H106" s="9" t="n"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J106" t="b">
+        <v>1</v>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>event details, quantity, and price not provided in ticket delivery notification</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>TINASHE - The Show Must Go On</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E107" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F107" t="n">
+        <v>4</v>
+      </c>
+      <c r="G107" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H107" s="9" t="n">
+        <v>222.64</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J107" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E108" s="8" t="n">
+        <v>46316.05293981481</v>
+      </c>
+      <c r="G108" s="9" t="n"/>
+      <c r="H108" s="9" t="n"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J108" t="b">
+        <v>1</v>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>quantity, event details, and order info not stated in delivery update</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-21 (6 new transactions, 3 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23625,6 +23625,226 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Ian Asher (18+ Event)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E109" s="8" t="n">
+        <v>46316.0890162037</v>
+      </c>
+      <c r="F109" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H109" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J109" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Ian Asher (18+ Event)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E110" s="8" t="n">
+        <v>46316.09042824074</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1</v>
+      </c>
+      <c r="G110" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H110" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J110" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>RÜFÜS DU SOL [DJ SET]</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>XS Nightclub</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="n">
+        <v>46348</v>
+      </c>
+      <c r="E111" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F111" t="n">
+        <v>2</v>
+      </c>
+      <c r="G111" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H111" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>Tixr</t>
+        </is>
+      </c>
+      <c r="J111" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Ian Asher (18+ Event)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>The Concourse Project</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E112" s="8" t="n">
+        <v>46316.14171296296</v>
+      </c>
+      <c r="F112" t="n">
+        <v>1</v>
+      </c>
+      <c r="G112" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H112" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J112" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E113" s="8" t="n">
+        <v>46316.14238425926</v>
+      </c>
+      <c r="G113" s="9" t="n"/>
+      <c r="H113" s="9" t="n"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J113" t="b">
+        <v>1</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>event details, quantity, and price not stated in ticket delivery email</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>TINASHE - The Show Must Go On - Artist Presale</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="n">
+        <v>46500</v>
+      </c>
+      <c r="E114" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F114" t="n">
+        <v>4</v>
+      </c>
+      <c r="G114" s="9" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H114" s="9" t="n">
+        <v>222.64</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J114" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-21 (1 new transactions, 3 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K114"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23845,6 +23845,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Dom Dolla</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>The Pinnacle</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E115" s="8" t="n">
+        <v>46316.81392361111</v>
+      </c>
+      <c r="F115" t="n">
+        <v>1</v>
+      </c>
+      <c r="G115" s="9" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="H115" s="9" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J115" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-22 (2 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23885,6 +23885,86 @@
         <v>0</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Kaytranada</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Pacha</t>
+        </is>
+      </c>
+      <c r="D116" s="8" t="n">
+        <v>46325</v>
+      </c>
+      <c r="E116" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1</v>
+      </c>
+      <c r="G116" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="H116" s="9" t="n">
+        <v>280</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J116" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>MGMT (DJ Set)</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>The Church Nightclub</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E117" s="8" t="n">
+        <v>46317.14586805556</v>
+      </c>
+      <c r="F117" t="n">
+        <v>2</v>
+      </c>
+      <c r="G117" s="9" t="n">
+        <v>98</v>
+      </c>
+      <c r="H117" s="9" t="n">
+        <v>196</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J117" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-22 (4 new transactions, 5 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23965,6 +23965,151 @@
         <v>0</v>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>MGMT DJ SET</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>The Church Nightclub</t>
+        </is>
+      </c>
+      <c r="D118" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E118" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F118" t="n">
+        <v>4</v>
+      </c>
+      <c r="G118" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="H118" s="9" t="n">
+        <v>159.8</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>TicketWeb</t>
+        </is>
+      </c>
+      <c r="J118" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>MGMT DJ SET</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>The Church Nightclub</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E119" s="8" t="n">
+        <v>46317.67777777778</v>
+      </c>
+      <c r="F119" t="n">
+        <v>4</v>
+      </c>
+      <c r="G119" s="9" t="n">
+        <v>45</v>
+      </c>
+      <c r="H119" s="9" t="n">
+        <v>199.8</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>TicketWeb</t>
+        </is>
+      </c>
+      <c r="J119" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E120" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G120" s="9" t="n"/>
+      <c r="H120" s="9" t="n"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J120" t="b">
+        <v>1</v>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>quantity and event details not stated in delivery update email</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Teksupport: Circoloco Halloween (Sat) SOLD OUT</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Brooklyn Storehouse</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="n">
+        <v>46326</v>
+      </c>
+      <c r="E121" s="8" t="n">
+        <v>46317.76997685185</v>
+      </c>
+      <c r="F121" t="n">
+        <v>3</v>
+      </c>
+      <c r="G121" s="9" t="n">
+        <v>182.31</v>
+      </c>
+      <c r="H121" s="9" t="n">
+        <v>546.9299999999999</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
+      <c r="J121" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-22 (5 new transactions, 3 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K121"/>
+  <dimension ref="A1:K126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24110,6 +24110,200 @@
         <v>0</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SILO Dallas</t>
+        </is>
+      </c>
+      <c r="D122" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E122" s="8" t="n">
+        <v>46317.78619212963</v>
+      </c>
+      <c r="F122" t="n">
+        <v>1</v>
+      </c>
+      <c r="G122" s="9" t="n">
+        <v>208.73</v>
+      </c>
+      <c r="H122" s="9" t="n">
+        <v>208.73</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J122" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E123" s="8" t="n">
+        <v>46317</v>
+      </c>
+      <c r="G123" s="9" t="n"/>
+      <c r="H123" s="9" t="n"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J123" t="b">
+        <v>1</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Quantity and pricing not stated for transfer out</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D124" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E124" s="8" t="n">
+        <v>46317.79821759259</v>
+      </c>
+      <c r="G124" s="9" t="n"/>
+      <c r="H124" s="9" t="n"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J124" t="b">
+        <v>1</v>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E125" s="8" t="n">
+        <v>46317.79832175926</v>
+      </c>
+      <c r="G125" s="9" t="n"/>
+      <c r="H125" s="9" t="n"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J125" t="b">
+        <v>1</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>quantity not stated and email kind is a pending transfer update</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SILO Dallas</t>
+        </is>
+      </c>
+      <c r="D126" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E126" s="8" t="n">
+        <v>46317.82413194444</v>
+      </c>
+      <c r="F126" t="n">
+        <v>1</v>
+      </c>
+      <c r="G126" s="9" t="n">
+        <v>208.74</v>
+      </c>
+      <c r="H126" s="9" t="n">
+        <v>208.74</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J126" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-23 (1 new transactions, 7 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K126"/>
+  <dimension ref="A1:K127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24304,6 +24304,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E127" s="8" t="n">
+        <v>46318.20003472222</v>
+      </c>
+      <c r="F127" t="n">
+        <v>1</v>
+      </c>
+      <c r="G127" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H127" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J127" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-23 (1 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:K128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24344,6 +24344,51 @@
         <v>0</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Mission Ballroom - Denver, CO</t>
+        </is>
+      </c>
+      <c r="D128" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E128" s="8" t="n">
+        <v>46318.50325231482</v>
+      </c>
+      <c r="F128" t="n">
+        <v>1</v>
+      </c>
+      <c r="G128" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="H128" s="9" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J128" t="b">
+        <v>1</v>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>delivery reminder email for an existing sale, email_kind uncertain</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-23 (6 new transactions, 12 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K128"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24389,6 +24389,240 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Mission Ballroom, Denver , CO</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E129" s="8" t="n">
+        <v>46318.60469907407</v>
+      </c>
+      <c r="G129" s="9" t="n"/>
+      <c r="H129" s="9" t="n"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J129" t="b">
+        <v>1</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>quantity not stated and email kind is a pending transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D130" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E130" s="8" t="n">
+        <v>46318.60484953703</v>
+      </c>
+      <c r="G130" s="9" t="n"/>
+      <c r="H130" s="9" t="n"/>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J130" t="b">
+        <v>1</v>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Odd Mob - Admissions</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E131" s="8" t="n">
+        <v>46318.60483796296</v>
+      </c>
+      <c r="G131" s="9" t="n"/>
+      <c r="H131" s="9" t="n"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>AXS</t>
+        </is>
+      </c>
+      <c r="J131" t="b">
+        <v>1</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>quantity not stated in transfer pending email</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Circoloco Miami</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Factory Town</t>
+        </is>
+      </c>
+      <c r="D132" s="8" t="n">
+        <v>46361</v>
+      </c>
+      <c r="E132" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="F132" t="n">
+        <v>1</v>
+      </c>
+      <c r="G132" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="H132" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J132" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>SILO Dallas</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E133" s="8" t="n">
+        <v>46318.70008101852</v>
+      </c>
+      <c r="F133" t="n">
+        <v>1</v>
+      </c>
+      <c r="G133" s="9" t="n">
+        <v>232.76</v>
+      </c>
+      <c r="H133" s="9" t="n">
+        <v>232.76</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J133" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Kettama</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>SILO Dallas</t>
+        </is>
+      </c>
+      <c r="D134" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E134" s="8" t="n">
+        <v>46318.70289351852</v>
+      </c>
+      <c r="F134" t="n">
+        <v>1</v>
+      </c>
+      <c r="G134" s="9" t="n">
+        <v>235.2</v>
+      </c>
+      <c r="H134" s="9" t="n">
+        <v>235.2</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J134" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-23 (1 new transactions, 5 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K134"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24623,6 +24623,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Circoloco Miami</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Factory Town</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="n">
+        <v>46361</v>
+      </c>
+      <c r="E135" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="F135" t="n">
+        <v>1</v>
+      </c>
+      <c r="G135" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="H135" s="9" t="n">
+        <v>210</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>CrowdVolt</t>
+        </is>
+      </c>
+      <c r="J135" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-24 (1 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K135"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24663,6 +24663,46 @@
         <v>0</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>MGMT (DJ Set)</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>The Church Nightclub</t>
+        </is>
+      </c>
+      <c r="D136" s="8" t="n">
+        <v>46340</v>
+      </c>
+      <c r="E136" s="8" t="n">
+        <v>46319.00430555556</v>
+      </c>
+      <c r="F136" t="n">
+        <v>2</v>
+      </c>
+      <c r="G136" s="9" t="n">
+        <v>83.3</v>
+      </c>
+      <c r="H136" s="9" t="n">
+        <v>166.6</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J136" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: pipeline run 2026-10-24 (2 new transactions, 2 skipped, 270 matched pairs)
</commit_message>
<xml_diff>
--- a/EmailScrape.xlsx
+++ b/EmailScrape.xlsx
@@ -19413,7 +19413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K136"/>
+  <dimension ref="A1:K138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24703,6 +24703,87 @@
         <v>0</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Giveon</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Walt Disney Concert Hall</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="n">
+        <v>46343</v>
+      </c>
+      <c r="E137" s="8" t="n">
+        <v>46319.17089120371</v>
+      </c>
+      <c r="F137" t="n">
+        <v>2</v>
+      </c>
+      <c r="G137" s="9" t="n">
+        <v>225.4</v>
+      </c>
+      <c r="H137" s="9" t="n">
+        <v>450.8</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J137" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Odd Mob</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Mission Ballroom</t>
+        </is>
+      </c>
+      <c r="D138" s="8" t="n">
+        <v>46318</v>
+      </c>
+      <c r="E138" s="8" t="n">
+        <v>46319.21189814815</v>
+      </c>
+      <c r="F138" t="n">
+        <v>1</v>
+      </c>
+      <c r="G138" s="9" t="n"/>
+      <c r="H138" s="9" t="n"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Lysted</t>
+        </is>
+      </c>
+      <c r="J138" t="b">
+        <v>1</v>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>total_price not stated in cancellation email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>